<commit_message>
Painel do dinheiro das Eleicoes 2026, 19/09/2026 21:40
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -15,7 +15,8 @@
     <sheet name="Tabela 6" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Tabela 7" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Tabela 8" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Sinais e fonte" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Tabela 9" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Sinais e fonte" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -941,6 +942,638 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="96" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Sinais convencionais, conforme a Norma de Apresentacao Tabular do IBGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dado numerico igual a zero, nao resultante de arredondamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>..</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>nao se aplica dado numerico</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>dado numerico nao disponivel</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>dado numerico omitido a fim de evitar a individualizacao da informacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>dado numerico igual a zero resultante de arredondamento de valor menor que a metade da unidade adotada</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-09-19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Conferencias desta extracao</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>candidatos_linhas</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>20984</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>candidatos_sq_unicos</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>20984</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>complementar_linhas</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>20984</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>complementar_sem_par_no_principal</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>principal_sem_complementar</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>cpf_publicado</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>20981</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>cpf_nao_publicado</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>cpf_com_digito_invalido</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>cpf_repetido_entre_candidaturas</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>candidaturas_de_pessoa_com_mais_de_uma</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>receitas_linhas</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>118115</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>receitas_valor_ilegivel</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>receitas_total</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>5662847203.74</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>candidatos_com_mais_de_um_prestador</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>data_ultima_prestacao</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>receitas_por_grupo</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>{"REC_FEFC": 4640335681.25, "REC_FINANCIAMENTO_COLETIVO": 13368899.5, "REC_FUNDO_PARTIDARIO": 383435440.19, "REC_ORIGEM_NAO_IDENTIFICADA": 760428.53, "REC_OUTROS_CANDIDATOS": 74533044.08, "REC_PARTIDO_OUTROS_RECURSOS": 97804382.98, "REC_PESSOAS_FISICAS": 358196079.53, "REC_PROPRIOS": 94413247.68, "REC_SEM_ORIGEM": 0.0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>doadores_distintos</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>52198</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>bens_linhas</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>77155</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>bens_valor_ilegivel</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>bens_chave_repetida_sq_ordem</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>bens_total</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>32253496244.68</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>candidatos_com_bem_acima_50mi</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>despesas_contratadas_linhas</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>735740</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>despesas_contratadas_sq_unicos</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>586089</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>despesas_contratadas_total</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>3639294391.85</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>despesas_pagas_linhas</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>370817</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>despesas_pagas_total</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2057636895.87</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>pagas_sem_despesa_contratada</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>pagas_sem_contratada_valor</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>despesas_sem_documento_fornecedor</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>48248</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>pago_sem_documento_fornecedor</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>385539.31</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>fornecedores_com_mais_de_um_municipio</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>fornecedores_distintos</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>424833</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>cnpj_consultados_nesta_rodada</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>cnpj_em_cache</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2085</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>fornecedores_pj</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>46192</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>fornecedores_pj_sem_localizacao</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>43379</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>cnpj_rodada_interrompida_por_429</t>
+        </is>
+      </c>
+      <c r="B50" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>fornecedores_com_documento_invalido</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | pago total</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1779406409.12</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | transferido a outros prestadores</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>43899672.26</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Fundo Partidário | CANDIDATOS | pago total</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>82017230.56999999</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Fundo Partidário | CANDIDATOS | transferido a outros prestadores</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>858310.02</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | pago total</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>4736070164.83</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | transferido a outros prestadores</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>4686383743.4</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Fundo Partidário | PARTIDOS | pago total</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>417477887.97</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Fundo Partidário | PARTIDOS | transferido a outros prestadores</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>373913357.68</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>votacao_linhas</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>gerado_em</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-09-19 18:22:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>soma_receitas_candidatos_confere</t>
+        </is>
+      </c>
+      <c r="B62" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>pago_por_fornecedor_confere</t>
+        </is>
+      </c>
+      <c r="B63" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>receitas_de_sq_fora_do_cadastro</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -16588,12 +17221,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E175"/>
+  <dimension ref="A1:E231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="47" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="41" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
@@ -17089,7 +17722,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Presidenciáveis, circunscrição nacional</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">
@@ -17595,7 +18228,7 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Presidenciáveis, circunscrição nacional</t>
         </is>
       </c>
       <c r="D46" s="6" t="n">
@@ -18423,7 +19056,7 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Presidenciáveis, circunscrição nacional</t>
         </is>
       </c>
       <c r="D82" s="6" t="n">
@@ -19205,7 +19838,7 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Presidenciáveis, circunscrição nacional</t>
         </is>
       </c>
       <c r="D116" s="6" t="n">
@@ -20240,7 +20873,7 @@
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Presidenciáveis, circunscrição nacional</t>
         </is>
       </c>
       <c r="D161" s="6" t="n">
@@ -20458,51 +21091,1339 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="7" t="inlineStr">
+      <c r="A171" s="4" t="inlineStr">
         <is>
           <t>Doacao de pessoa fisica, pela UF do candidato</t>
         </is>
       </c>
-      <c r="B171" s="7" t="inlineStr">
+      <c r="B171" s="4" t="inlineStr">
         <is>
           <t>AP</t>
         </is>
       </c>
-      <c r="C171" s="7" t="inlineStr">
+      <c r="C171" s="4" t="inlineStr">
         <is>
           <t>Amapá</t>
         </is>
       </c>
-      <c r="D171" s="9" t="n">
+      <c r="D171" s="6" t="n">
         <v>1674383.36</v>
       </c>
-      <c r="E171" s="13" t="n">
+      <c r="E171" s="12" t="n">
         <v>0.47</v>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="10" t="inlineStr">
+      <c r="A172" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C172" s="4" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="D172" s="6" t="n">
+        <v>2628</v>
+      </c>
+      <c r="E172" s="12" t="n">
+        <v>12.52</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B173" s="4" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="C173" s="4" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D173" s="6" t="n">
+        <v>2055</v>
+      </c>
+      <c r="E173" s="12" t="n">
+        <v>9.789999999999999</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="C174" s="4" t="inlineStr">
+        <is>
+          <t>Minas Gerais</t>
+        </is>
+      </c>
+      <c r="D174" s="6" t="n">
+        <v>1832</v>
+      </c>
+      <c r="E174" s="12" t="n">
+        <v>8.73</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B175" s="4" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="C175" s="4" t="inlineStr">
+        <is>
+          <t>Bahia</t>
+        </is>
+      </c>
+      <c r="D175" s="6" t="n">
+        <v>1224</v>
+      </c>
+      <c r="E175" s="12" t="n">
+        <v>5.83</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="C176" s="4" t="inlineStr">
+        <is>
+          <t>Paraná</t>
+        </is>
+      </c>
+      <c r="D176" s="6" t="n">
+        <v>1090</v>
+      </c>
+      <c r="E176" s="12" t="n">
+        <v>5.19</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B177" s="4" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="C177" s="4" t="inlineStr">
+        <is>
+          <t>Rio Grande do Sul</t>
+        </is>
+      </c>
+      <c r="D177" s="6" t="n">
+        <v>1053</v>
+      </c>
+      <c r="E177" s="12" t="n">
+        <v>5.02</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="C178" s="4" t="inlineStr">
+        <is>
+          <t>Pernambuco</t>
+        </is>
+      </c>
+      <c r="D178" s="6" t="n">
+        <v>961</v>
+      </c>
+      <c r="E178" s="12" t="n">
+        <v>4.58</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B179" s="4" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="C179" s="4" t="inlineStr">
+        <is>
+          <t>Goiás</t>
+        </is>
+      </c>
+      <c r="D179" s="6" t="n">
+        <v>905</v>
+      </c>
+      <c r="E179" s="12" t="n">
+        <v>4.31</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="C180" s="4" t="inlineStr">
+        <is>
+          <t>Pará</t>
+        </is>
+      </c>
+      <c r="D180" s="6" t="n">
+        <v>741</v>
+      </c>
+      <c r="E180" s="12" t="n">
+        <v>3.53</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="C181" s="4" t="inlineStr">
+        <is>
+          <t>Ceará</t>
+        </is>
+      </c>
+      <c r="D181" s="6" t="n">
+        <v>713</v>
+      </c>
+      <c r="E181" s="12" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="C182" s="4" t="inlineStr">
+        <is>
+          <t>Santa Catarina</t>
+        </is>
+      </c>
+      <c r="D182" s="6" t="n">
+        <v>700</v>
+      </c>
+      <c r="E182" s="12" t="n">
+        <v>3.34</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="C183" s="4" t="inlineStr">
+        <is>
+          <t>Distrito Federal</t>
+        </is>
+      </c>
+      <c r="D183" s="6" t="n">
+        <v>668</v>
+      </c>
+      <c r="E183" s="12" t="n">
+        <v>3.18</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="C184" s="4" t="inlineStr">
+        <is>
+          <t>Maranhão</t>
+        </is>
+      </c>
+      <c r="D184" s="6" t="n">
+        <v>619</v>
+      </c>
+      <c r="E184" s="12" t="n">
+        <v>2.95</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B185" s="4" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="C185" s="4" t="inlineStr">
+        <is>
+          <t>Espírito Santo</t>
+        </is>
+      </c>
+      <c r="D185" s="6" t="n">
+        <v>591</v>
+      </c>
+      <c r="E185" s="12" t="n">
+        <v>2.82</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="C186" s="4" t="inlineStr">
+        <is>
+          <t>Amazonas</t>
+        </is>
+      </c>
+      <c r="D186" s="6" t="n">
+        <v>475</v>
+      </c>
+      <c r="E186" s="12" t="n">
+        <v>2.26</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="C187" s="4" t="inlineStr">
+        <is>
+          <t>Mato Grosso</t>
+        </is>
+      </c>
+      <c r="D187" s="6" t="n">
+        <v>455</v>
+      </c>
+      <c r="E187" s="12" t="n">
+        <v>2.17</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="C188" s="4" t="inlineStr">
+        <is>
+          <t>Paraíba</t>
+        </is>
+      </c>
+      <c r="D188" s="6" t="n">
+        <v>450</v>
+      </c>
+      <c r="E188" s="12" t="n">
+        <v>2.14</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t>Rondônia</t>
+        </is>
+      </c>
+      <c r="D189" s="6" t="n">
+        <v>438</v>
+      </c>
+      <c r="E189" s="12" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="C190" s="4" t="inlineStr">
+        <is>
+          <t>Mato Grosso do Sul</t>
+        </is>
+      </c>
+      <c r="D190" s="6" t="n">
+        <v>425</v>
+      </c>
+      <c r="E190" s="12" t="n">
+        <v>2.03</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t>RR</t>
+        </is>
+      </c>
+      <c r="C191" s="4" t="inlineStr">
+        <is>
+          <t>Roraima</t>
+        </is>
+      </c>
+      <c r="D191" s="6" t="n">
+        <v>413</v>
+      </c>
+      <c r="E191" s="12" t="n">
+        <v>1.97</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="C192" s="4" t="inlineStr">
+        <is>
+          <t>Sergipe</t>
+        </is>
+      </c>
+      <c r="D192" s="6" t="n">
+        <v>411</v>
+      </c>
+      <c r="E192" s="12" t="n">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B193" s="4" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C193" s="4" t="inlineStr">
+        <is>
+          <t>Piauí</t>
+        </is>
+      </c>
+      <c r="D193" s="6" t="n">
+        <v>402</v>
+      </c>
+      <c r="E193" s="12" t="n">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="C194" s="4" t="inlineStr">
+        <is>
+          <t>Acre</t>
+        </is>
+      </c>
+      <c r="D194" s="6" t="n">
+        <v>388</v>
+      </c>
+      <c r="E194" s="12" t="n">
+        <v>1.85</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C195" s="4" t="inlineStr">
+        <is>
+          <t>Tocantins</t>
+        </is>
+      </c>
+      <c r="D195" s="6" t="n">
+        <v>368</v>
+      </c>
+      <c r="E195" s="12" t="n">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>RN</t>
+        </is>
+      </c>
+      <c r="C196" s="4" t="inlineStr">
+        <is>
+          <t>Rio Grande do Norte</t>
+        </is>
+      </c>
+      <c r="D196" s="6" t="n">
+        <v>330</v>
+      </c>
+      <c r="E196" s="12" t="n">
+        <v>1.57</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B197" s="4" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="C197" s="4" t="inlineStr">
+        <is>
+          <t>Amapá</t>
+        </is>
+      </c>
+      <c r="D197" s="6" t="n">
+        <v>322</v>
+      </c>
+      <c r="E197" s="12" t="n">
+        <v>1.53</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="C198" s="4" t="inlineStr">
+        <is>
+          <t>Alagoas</t>
+        </is>
+      </c>
+      <c r="D198" s="6" t="n">
+        <v>299</v>
+      </c>
+      <c r="E198" s="12" t="n">
+        <v>1.42</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="4" t="inlineStr">
+        <is>
+          <t>candidatos</t>
+        </is>
+      </c>
+      <c r="B199" s="4" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="C199" s="4" t="inlineStr">
+        <is>
+          <t>Presidenciáveis, circunscrição nacional</t>
+        </is>
+      </c>
+      <c r="D199" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E199" s="12" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B200" s="4" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="C200" s="4" t="inlineStr">
+        <is>
+          <t>Minas Gerais</t>
+        </is>
+      </c>
+      <c r="D200" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="E200" s="12" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B201" s="4" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="C201" s="4" t="inlineStr">
+        <is>
+          <t>Maranhão</t>
+        </is>
+      </c>
+      <c r="D201" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="E201" s="12" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B202" s="4" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="C202" s="4" t="inlineStr">
+        <is>
+          <t>Distrito Federal</t>
+        </is>
+      </c>
+      <c r="D202" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="E202" s="12" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B203" s="4" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="C203" s="4" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D203" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="E203" s="12" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B204" s="4" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C204" s="4" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="D204" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="E204" s="12" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B205" s="4" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="C205" s="4" t="inlineStr">
+        <is>
+          <t>Pernambuco</t>
+        </is>
+      </c>
+      <c r="D205" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="E205" s="12" t="n">
+        <v>4.05</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t>RN</t>
+        </is>
+      </c>
+      <c r="C206" s="4" t="inlineStr">
+        <is>
+          <t>Rio Grande do Norte</t>
+        </is>
+      </c>
+      <c r="D206" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="E206" s="12" t="n">
+        <v>3.91</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B207" s="4" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="C207" s="4" t="inlineStr">
+        <is>
+          <t>Rio Grande do Sul</t>
+        </is>
+      </c>
+      <c r="D207" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="E207" s="12" t="n">
+        <v>3.91</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="C208" s="4" t="inlineStr">
+        <is>
+          <t>Ceará</t>
+        </is>
+      </c>
+      <c r="D208" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="E208" s="12" t="n">
+        <v>3.91</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B209" s="4" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="C209" s="4" t="inlineStr">
+        <is>
+          <t>Goiás</t>
+        </is>
+      </c>
+      <c r="D209" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E209" s="12" t="n">
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="C210" s="4" t="inlineStr">
+        <is>
+          <t>Santa Catarina</t>
+        </is>
+      </c>
+      <c r="D210" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E210" s="12" t="n">
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B211" s="4" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="C211" s="4" t="inlineStr">
+        <is>
+          <t>Bahia</t>
+        </is>
+      </c>
+      <c r="D211" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E211" s="12" t="n">
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B212" s="4" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="C212" s="4" t="inlineStr">
+        <is>
+          <t>Pará</t>
+        </is>
+      </c>
+      <c r="D212" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E212" s="12" t="n">
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="C213" s="4" t="inlineStr">
+        <is>
+          <t>Paraná</t>
+        </is>
+      </c>
+      <c r="D213" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E213" s="12" t="n">
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="C214" s="4" t="inlineStr">
+        <is>
+          <t>Mato Grosso</t>
+        </is>
+      </c>
+      <c r="D214" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="E214" s="12" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B215" s="4" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="C215" s="4" t="inlineStr">
+        <is>
+          <t>Espírito Santo</t>
+        </is>
+      </c>
+      <c r="D215" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="E215" s="12" t="n">
+        <v>3.62</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B216" s="4" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="C216" s="4" t="inlineStr">
+        <is>
+          <t>Acre</t>
+        </is>
+      </c>
+      <c r="D216" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="E216" s="12" t="n">
+        <v>3.47</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B217" s="4" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="C217" s="4" t="inlineStr">
+        <is>
+          <t>Paraíba</t>
+        </is>
+      </c>
+      <c r="D217" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="E217" s="12" t="n">
+        <v>3.47</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B218" s="4" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C218" s="4" t="inlineStr">
+        <is>
+          <t>Piauí</t>
+        </is>
+      </c>
+      <c r="D218" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="E218" s="12" t="n">
+        <v>3.47</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B219" s="4" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="C219" s="4" t="inlineStr">
+        <is>
+          <t>Amazonas</t>
+        </is>
+      </c>
+      <c r="D219" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="E219" s="12" t="n">
+        <v>3.33</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t>RR</t>
+        </is>
+      </c>
+      <c r="C220" s="4" t="inlineStr">
+        <is>
+          <t>Roraima</t>
+        </is>
+      </c>
+      <c r="D220" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="E220" s="12" t="n">
+        <v>3.33</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B221" s="4" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="C221" s="4" t="inlineStr">
+        <is>
+          <t>Mato Grosso do Sul</t>
+        </is>
+      </c>
+      <c r="D221" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="E221" s="12" t="n">
+        <v>3.33</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B222" s="4" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="C222" s="4" t="inlineStr">
+        <is>
+          <t>Sergipe</t>
+        </is>
+      </c>
+      <c r="D222" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="E222" s="12" t="n">
+        <v>3.18</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B223" s="4" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C223" s="4" t="inlineStr">
+        <is>
+          <t>Tocantins</t>
+        </is>
+      </c>
+      <c r="D223" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="E223" s="12" t="n">
+        <v>3.04</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B224" s="4" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="C224" s="4" t="inlineStr">
+        <is>
+          <t>Amapá</t>
+        </is>
+      </c>
+      <c r="D224" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E224" s="12" t="n">
+        <v>2.89</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B225" s="4" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="C225" s="4" t="inlineStr">
+        <is>
+          <t>Rondônia</t>
+        </is>
+      </c>
+      <c r="D225" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E225" s="12" t="n">
+        <v>2.89</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B226" s="4" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="C226" s="4" t="inlineStr">
+        <is>
+          <t>Alagoas</t>
+        </is>
+      </c>
+      <c r="D226" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="E226" s="12" t="n">
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="7" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B227" s="7" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="C227" s="7" t="inlineStr">
+        <is>
+          <t>Presidenciáveis, circunscrição nacional</t>
+        </is>
+      </c>
+      <c r="D227" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="E227" s="13" t="n">
+        <v>2.03</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="10" t="inlineStr">
         <is>
           <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
         </is>
       </c>
     </row>
-    <row r="173">
-      <c r="A173" s="10" t="inlineStr">
+    <row r="229">
+      <c r="A229" s="10" t="inlineStr">
         <is>
           <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-09-19.</t>
         </is>
       </c>
     </row>
-    <row r="174">
-      <c r="A174" s="10" t="inlineStr">
+    <row r="230">
+      <c r="A230" s="10" t="inlineStr">
         <is>
           <t>Nota 1: a serie de fornecedores cobre 45.5% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
         </is>
       </c>
     </row>
-    <row r="175">
-      <c r="A175" s="10" t="inlineStr">
+    <row r="231">
+      <c r="A231" s="10" t="inlineStr">
         <is>
           <t>Nota 2: a serie por UF do doador cobre apenas 8.3% do valor doado, porque o TSE nao publica a UF do doador pessoa fisica. Para leitura integral use a serie por UF do candidato que recebeu.</t>
         </is>
@@ -26285,628 +28206,1409 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B64"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="96" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>Sinais convencionais, conforme a Norma de Apresentacao Tabular do IBGE</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>dado numerico igual a zero, nao resultante de arredondamento</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tabela 9 - Eleitorado apto, populacao residente e dinheiro de campanha, por unidade da federacao - Brasil - 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Eleitores e habitantes em numero absoluto, valores em R$ 1,00</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>..</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>nao se aplica dado numerico</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Unidade da federacao</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Habitantes</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Eleitores aptos</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Participacao no eleitorado (%)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Eleitores sobre habitantes (%)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Candidaturas</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Vagas</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Eleitores por vaga</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Candidaturas por 100 mil eleitores</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Receita de campanha</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Receita por habitante</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Receita por eleitor</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Dinheiro publico por eleitor</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>46179008</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>34105332</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>21.61</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>73.84999999999999</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>2628</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>172</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>198287</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>7.71</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>810574199.1900001</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>17.55</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>23.77</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>21.18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>21460311</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>16379547</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>76.31999999999999</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>1832</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>118692</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>11.18</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>465589840.32</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>28.43</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>23.73</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>17225410</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>12857388</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>74.64</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>2055</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>124</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>103689</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>15.98</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>452184964.68</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>35.17</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>32.54</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>14889472</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>11321934</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>7.17</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>76.04000000000001</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>1224</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>110</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>102927</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>10.81</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>313098347.49</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>21.03</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>27.65</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>25.49</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>11952456</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>8610076</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>72.04000000000001</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>1090</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>93588</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>288440062.88</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>24.13</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>28.74</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>11233317</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>8526505</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>1053</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>94</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>90708</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>12.35</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>287776923.16</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>25.62</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>33.75</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>29.91</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>9583176</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>7226975</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>75.41</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>961</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>82</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>88134</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>227630341.53</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>23.75</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>28.64</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>9302211</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>7000978</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>75.26000000000001</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>713</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>92118</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>10.18</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>210683767.02</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>22.65</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>30.09</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>26.23</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>8756324</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>6267107</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>71.56999999999999</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>741</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>94956</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>11.82</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>173396708</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>27.67</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>25.02</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>8312759</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>5725998</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>68.88</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>89469</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>186720168.89</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>22.46</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>32.61</v>
+      </c>
+      <c r="M14" s="6" t="n">
+        <v>27.24</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>7024557</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>5188115</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>73.86</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>619</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>76296</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>11.93</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>199700334.94</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>28.43</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>38.49</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>35.02</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7495033</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>5081043</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>67.79000000000001</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>905</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>76986</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>17.81</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>196363339.4</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>38.65</v>
+      </c>
+      <c r="M16" s="6" t="n">
+        <v>32.95</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>4182828</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>3248007</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>77.65000000000001</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>450</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>58000</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>13.85</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>134119341.65</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>32.06</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>41.29</v>
+      </c>
+      <c r="M17" s="6" t="n">
+        <v>38.83</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4150692</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>2990582</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>72.05</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>591</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>62304</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>19.76</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>121510720.38</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>29.27</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>40.63</v>
+      </c>
+      <c r="M18" s="6" t="n">
+        <v>34.96</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>4360926</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>2802091</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>64.25</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>475</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>70052</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>16.95</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>133207564.44</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>30.55</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>47.54</v>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>43.41</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>3392617</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>2708756</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>79.84</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>402</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>56432</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>14.84</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>131934587.08</v>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>38.89</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>48.71</v>
+      </c>
+      <c r="M20" s="6" t="n">
+        <v>42.96</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>RN</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>3463737</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>2660947</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>76.81999999999999</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>330</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>66524</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>96738393.37</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>27.93</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>36.35</v>
+      </c>
+      <c r="M21" s="6" t="n">
+        <v>34.3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>3950330</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>2639075</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>66.81</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>455</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>65977</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>17.24</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>126651011.45</v>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>32.06</v>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="M22" s="6" t="n">
+        <v>34.95</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>3221128</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>2442275</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>75.81999999999999</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>299</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>55506</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>12.24</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>109643825.13</v>
+      </c>
+      <c r="K23" s="6" t="n">
+        <v>34.04</v>
+      </c>
+      <c r="L23" s="6" t="n">
+        <v>44.89</v>
+      </c>
+      <c r="M23" s="6" t="n">
+        <v>42.15</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>3009996</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>2253238</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>74.86</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>668</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>56331</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>29.65</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>138731909.46</v>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>46.09</v>
+      </c>
+      <c r="L24" s="6" t="n">
+        <v>61.57</v>
+      </c>
+      <c r="M24" s="6" t="n">
+        <v>51.94</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>2946317</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>2025001</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>68.73</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>425</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>50625</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>104015513.56</v>
+      </c>
+      <c r="K25" s="6" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="L25" s="6" t="n">
+        <v>51.37</v>
+      </c>
+      <c r="M25" s="6" t="n">
+        <v>45.8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2307255</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>1740240</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>75.42</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>411</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>43506</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>23.62</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>110998484.05</v>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>48.11</v>
+      </c>
+      <c r="L26" s="6" t="n">
+        <v>63.78</v>
+      </c>
+      <c r="M26" s="6" t="n">
+        <v>60.44</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1757338</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>1268667</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>72.19</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>438</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>31717</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>34.52</v>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>121344202.8</v>
+      </c>
+      <c r="K27" s="6" t="n">
+        <v>69.05</v>
+      </c>
+      <c r="L27" s="6" t="n">
+        <v>95.65000000000001</v>
+      </c>
+      <c r="M27" s="6" t="n">
+        <v>83.78</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1595994</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>1182768</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>74.11</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>368</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>29569</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>31.11</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>107313260.82</v>
+      </c>
+      <c r="K28" s="6" t="n">
+        <v>67.23999999999999</v>
+      </c>
+      <c r="L28" s="6" t="n">
+        <v>90.73</v>
+      </c>
+      <c r="M28" s="6" t="n">
+        <v>79.27</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>887794</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>614631</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>69.23</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>388</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>15366</v>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>63.13</v>
+      </c>
+      <c r="J29" s="6" t="n">
+        <v>92017991.75</v>
+      </c>
+      <c r="K29" s="6" t="n">
+        <v>103.65</v>
+      </c>
+      <c r="L29" s="6" t="n">
+        <v>149.71</v>
+      </c>
+      <c r="M29" s="6" t="n">
+        <v>139.69</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>809953</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>577698</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>71.31999999999999</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>322</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>14442</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>55.74</v>
+      </c>
+      <c r="J30" s="6" t="n">
+        <v>102028469.09</v>
+      </c>
+      <c r="K30" s="6" t="n">
+        <v>125.97</v>
+      </c>
+      <c r="L30" s="6" t="n">
+        <v>176.61</v>
+      </c>
+      <c r="M30" s="6" t="n">
+        <v>170.82</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>RR</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>761012</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>401573</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>52.77</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>10039</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="J31" s="6" t="n">
+        <v>99728125.06</v>
+      </c>
+      <c r="K31" s="6" t="n">
+        <v>131.05</v>
+      </c>
+      <c r="L31" s="6" t="n">
+        <v>248.34</v>
+      </c>
+      <c r="M31" s="6" t="n">
+        <v>239.15</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Presidenciaveis (nacional)</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>...</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>dado numerico nao disponivel</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>dado numerico omitido a fim de evitar a individualizacao da informacao</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>dado numerico igual a zero resultante de arredondamento de valor menor que a metade da unidade adotada</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="n">
+        <v>120704806.15</v>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="n">
+        <v>214211951</v>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>157846547</v>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>73.69</v>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>20984</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>1790</v>
+      </c>
+      <c r="H33" s="8" t="n">
+        <v>88182</v>
+      </c>
+      <c r="I33" s="9" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="J33" s="9" t="n">
+        <v>5662847203.74</v>
+      </c>
+      <c r="K33" s="9" t="n">
+        <v>26.44</v>
+      </c>
+      <c r="L33" s="9" t="n">
+        <v>35.88</v>
+      </c>
+      <c r="M33" s="9" t="n">
+        <v>31.83</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Fonte: TSE, perfil do eleitorado, arquivo ATUAL, geracao declarada pela fonte em 01/09/2026; IBGE, estimativa da populacao residente, agregado 6579, referencia 2026; TSE, prestacao de contas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-09-19.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>Conferencias desta extracao</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>candidatos_linhas</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>20984</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>candidatos_sq_unicos</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>20984</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>complementar_linhas</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>20984</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>complementar_sem_par_no_principal</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>principal_sem_complementar</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>cpf_publicado</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>20981</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>cpf_nao_publicado</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>cpf_com_digito_invalido</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>cpf_repetido_entre_candidaturas</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>candidaturas_de_pessoa_com_mais_de_uma</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>receitas_linhas</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>118115</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>receitas_valor_ilegivel</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>receitas_total</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>5662847203.74</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>candidatos_com_mais_de_um_prestador</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>data_ultima_prestacao</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>receitas_por_grupo</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>{"REC_FEFC": 4640335681.25, "REC_FINANCIAMENTO_COLETIVO": 13368899.5, "REC_FUNDO_PARTIDARIO": 383435440.19, "REC_ORIGEM_NAO_IDENTIFICADA": 760428.53, "REC_OUTROS_CANDIDATOS": 74533044.08, "REC_PARTIDO_OUTROS_RECURSOS": 97804382.98, "REC_PESSOAS_FISICAS": 358196079.53, "REC_PROPRIOS": 94413247.68, "REC_SEM_ORIGEM": 0.0}</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>doadores_distintos</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>52198</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>bens_linhas</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>77155</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>bens_valor_ilegivel</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>bens_chave_repetida_sq_ordem</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>bens_total</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>32253496244.68</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>candidatos_com_bem_acima_50mi</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>despesas_contratadas_linhas</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>735740</v>
-      </c>
-    </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>despesas_contratadas_sq_unicos</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>586089</v>
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Nota 1: a linha 'Presidenciaveis (nacional)' e' a circunscricao nacional, onde correm presidente e vice. Ela nao tem populacao nem eleitorado proprios, e por isso os denominadores aparecem vazios.</t>
+        </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>despesas_contratadas_total</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>3639294391.85</v>
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Nota 2: o eleitorado no exterior, de 918.911 eleitores, nao pertence a unidade da federacao alguma e fica fora do rateio por estado.</t>
+        </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>despesas_pagas_linhas</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>370817</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>despesas_pagas_total</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>2057636895.87</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>pagas_sem_despesa_contratada</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>pagas_sem_contratada_valor</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>despesas_sem_documento_fornecedor</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>48248</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>pago_sem_documento_fornecedor</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>385539.31</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>fornecedores_com_mais_de_um_municipio</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>fornecedores_distintos</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>424833</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>cnpj_consultados_nesta_rodada</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>cnpj_em_cache</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>2085</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>fornecedores_pj</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>46192</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>fornecedores_pj_sem_localizacao</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>43379</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>cnpj_rodada_interrompida_por_429</t>
-        </is>
-      </c>
-      <c r="B50" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>fornecedores_com_documento_invalido</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>1008</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | pago total</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>1779406409.12</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | transferido a outros prestadores</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>43899672.26</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Fundo Partidário | CANDIDATOS | pago total</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>82017230.56999999</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Fundo Partidário | CANDIDATOS | transferido a outros prestadores</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>858310.02</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | pago total</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>4736070164.83</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | transferido a outros prestadores</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>4686383743.4</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Fundo Partidário | PARTIDOS | pago total</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>417477887.97</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Fundo Partidário | PARTIDOS | transferido a outros prestadores</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>373913357.68</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>votacao_linhas</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>gerado_em</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>2026-09-19 18:22:23</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>soma_receitas_candidatos_confere</t>
-        </is>
-      </c>
-      <c r="B62" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>pago_por_fornecedor_confere</t>
-        </is>
-      </c>
-      <c r="B63" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>receitas_de_sq_fora_do_cadastro</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>0</v>
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Nota 3: habitante nao vota. A proporcao entre eleitorado e populacao varia entre os estados, e por isso as duas colunas aparecem lado a lado em vez de uma so'.</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:M2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 19/09/2026 21:45
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 21:18:00.</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B64"/>
+  <dimension ref="A1:B66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 21:18:00.</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2085</v>
+        <v>4085</v>
       </c>
     </row>
     <row r="48">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>43379</v>
+        <v>41437</v>
       </c>
     </row>
     <row r="50">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-19 18:22:23</t>
+          <t>2026-09-19 21:18:00</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,31 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0</v>
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>colunas_da_ordem_do_usuario_ausentes</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>colunas_novas_fora_da_ordem_do_usuario</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8818,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 21:18:00.</t>
         </is>
       </c>
     </row>
@@ -15471,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 21:18:00.</t>
         </is>
       </c>
     </row>
@@ -17182,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 21:18:00.</t>
         </is>
       </c>
     </row>
@@ -19221,10 +19245,10 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>462595184.59</v>
+        <v>498139778.39</v>
       </c>
       <c r="E89" s="12" t="n">
-        <v>27.91</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="90">
@@ -19244,10 +19268,10 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>101552567.11</v>
+        <v>123277093.61</v>
       </c>
       <c r="E90" s="12" t="n">
-        <v>6.13</v>
+        <v>6.31</v>
       </c>
     </row>
     <row r="91">
@@ -19258,19 +19282,19 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Distrito Federal</t>
+          <t>Minas Gerais</t>
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>97450940.03</v>
+        <v>115875593.82</v>
       </c>
       <c r="E91" s="12" t="n">
-        <v>5.88</v>
+        <v>5.93</v>
       </c>
     </row>
     <row r="92">
@@ -19281,19 +19305,19 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Minas Gerais</t>
+          <t>Distrito Federal</t>
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>95952384.93000001</v>
+        <v>109143285.14</v>
       </c>
       <c r="E92" s="12" t="n">
-        <v>5.79</v>
+        <v>5.59</v>
       </c>
     </row>
     <row r="93">
@@ -19313,10 +19337,10 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>75382314.42</v>
+        <v>90224348.83</v>
       </c>
       <c r="E93" s="12" t="n">
-        <v>4.55</v>
+        <v>4.62</v>
       </c>
     </row>
     <row r="94">
@@ -19327,19 +19351,19 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Rio Grande do Sul</t>
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>59023776.93</v>
+        <v>72603182.98</v>
       </c>
       <c r="E94" s="12" t="n">
-        <v>3.56</v>
+        <v>3.72</v>
       </c>
     </row>
     <row r="95">
@@ -19350,19 +19374,19 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Sul</t>
+          <t>Maranhão</t>
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>58653681.05</v>
+        <v>71953659.25</v>
       </c>
       <c r="E95" s="12" t="n">
-        <v>3.54</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="96">
@@ -19373,19 +19397,19 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>Maranhão</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>56216311.01</v>
+        <v>70164634.72</v>
       </c>
       <c r="E96" s="12" t="n">
-        <v>3.39</v>
+        <v>3.59</v>
       </c>
     </row>
     <row r="97">
@@ -19405,10 +19429,10 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>55912430.48</v>
+        <v>68388277.31999999</v>
       </c>
       <c r="E97" s="12" t="n">
-        <v>3.37</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="98">
@@ -19428,10 +19452,10 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>54990895.48</v>
+        <v>68299073.65000001</v>
       </c>
       <c r="E98" s="12" t="n">
-        <v>3.32</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="99">
@@ -19451,10 +19475,10 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>54194985.89</v>
+        <v>65686053.35</v>
       </c>
       <c r="E99" s="12" t="n">
-        <v>3.27</v>
+        <v>3.36</v>
       </c>
     </row>
     <row r="100">
@@ -19465,19 +19489,19 @@
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Norte</t>
+          <t>Santa Catarina</t>
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>47402453.19</v>
+        <v>56664663.25</v>
       </c>
       <c r="E100" s="12" t="n">
-        <v>2.86</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="101">
@@ -19488,19 +19512,19 @@
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Santa Catarina</t>
+          <t>Paraíba</t>
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>46648452.04</v>
+        <v>54766020.66</v>
       </c>
       <c r="E101" s="12" t="n">
-        <v>2.81</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="102">
@@ -19511,19 +19535,19 @@
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>Paraíba</t>
+          <t>Rio Grande do Norte</t>
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>45565472.58</v>
+        <v>54024536.17</v>
       </c>
       <c r="E102" s="12" t="n">
-        <v>2.75</v>
+        <v>2.77</v>
       </c>
     </row>
     <row r="103">
@@ -19543,10 +19567,10 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>37022743.63</v>
+        <v>45655169.75</v>
       </c>
       <c r="E103" s="12" t="n">
-        <v>2.23</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="104">
@@ -19557,19 +19581,19 @@
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso</t>
+          <t>Pará</t>
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>32159075.09</v>
+        <v>42981889.7</v>
       </c>
       <c r="E104" s="12" t="n">
-        <v>1.94</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="105">
@@ -19580,19 +19604,19 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Amapá</t>
+          <t>Mato Grosso</t>
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>31737257.25</v>
+        <v>40022422.59</v>
       </c>
       <c r="E105" s="12" t="n">
-        <v>1.92</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="106">
@@ -19603,19 +19627,19 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Alagoas</t>
+          <t>Sergipe</t>
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>31321100.44</v>
+        <v>39931257.77</v>
       </c>
       <c r="E106" s="12" t="n">
-        <v>1.89</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="107">
@@ -19626,19 +19650,19 @@
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Pará</t>
+          <t>Amapá</t>
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>30666950.44</v>
+        <v>38670285.43</v>
       </c>
       <c r="E107" s="12" t="n">
-        <v>1.85</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="108">
@@ -19649,19 +19673,19 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Sergipe</t>
+          <t>Alagoas</t>
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>29400082.53</v>
+        <v>34815776.47</v>
       </c>
       <c r="E108" s="12" t="n">
-        <v>1.77</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="109">
@@ -19672,19 +19696,19 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Rondônia</t>
+          <t>Espírito Santo</t>
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>27283929.47</v>
+        <v>34294871.11</v>
       </c>
       <c r="E109" s="12" t="n">
-        <v>1.65</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="110">
@@ -19695,19 +19719,19 @@
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Espírito Santo</t>
+          <t>Rondônia</t>
         </is>
       </c>
       <c r="D110" s="6" t="n">
-        <v>27266283.34</v>
+        <v>33415958.86</v>
       </c>
       <c r="E110" s="12" t="n">
-        <v>1.65</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="111">
@@ -19727,10 +19751,10 @@
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>25217946.81</v>
+        <v>30479668.63</v>
       </c>
       <c r="E111" s="12" t="n">
-        <v>1.52</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="112">
@@ -19750,10 +19774,10 @@
         </is>
       </c>
       <c r="D112" s="6" t="n">
-        <v>24468624.21</v>
+        <v>29653706.56</v>
       </c>
       <c r="E112" s="12" t="n">
-        <v>1.48</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="113">
@@ -19773,10 +19797,10 @@
         </is>
       </c>
       <c r="D113" s="6" t="n">
-        <v>21320236.66</v>
+        <v>26463959.67</v>
       </c>
       <c r="E113" s="12" t="n">
-        <v>1.29</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="114">
@@ -19796,10 +19820,10 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>15198576.14</v>
+        <v>19996902.86</v>
       </c>
       <c r="E114" s="12" t="n">
-        <v>0.92</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="115">
@@ -19819,10 +19843,10 @@
         </is>
       </c>
       <c r="D115" s="6" t="n">
-        <v>11475857.08</v>
+        <v>16559874.57</v>
       </c>
       <c r="E115" s="12" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="116">
@@ -19845,7 +19869,7 @@
         <v>1095000</v>
       </c>
       <c r="E116" s="12" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="117">
@@ -22404,7 +22428,7 @@
     <row r="228">
       <c r="A228" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 21:18:00.</t>
         </is>
       </c>
     </row>
@@ -22418,7 +22442,7 @@
     <row r="230">
       <c r="A230" s="10" t="inlineStr">
         <is>
-          <t>Nota 1: a serie de fornecedores cobre 45.5% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
+          <t>Nota 1: a serie de fornecedores cobre 53.7% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
         </is>
       </c>
     </row>
@@ -23730,7 +23754,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 21:18:00.</t>
         </is>
       </c>
     </row>
@@ -25257,7 +25281,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 21:18:00.</t>
         </is>
       </c>
     </row>
@@ -28160,7 +28184,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 18:22:23.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-19 21:18:00.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 21/09/2026 16:01
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 08:48:12.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 08:48:12.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
         </is>
       </c>
     </row>
@@ -1380,179 +1380,179 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>cnpj_consultados_nesta_rodada</t>
+          <t>cnpj_falhas_transporte</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2000</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>cnpj_em_cache</t>
+          <t>cnpj_consultados_nesta_rodada</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>10298</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>fornecedores_pj</t>
+          <t>cnpj_em_cache</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>46377</v>
+        <v>14299</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>fornecedores_pj_sem_localizacao</t>
+          <t>fornecedores_pj</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>35641</v>
+        <v>46377</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>cnpj_rodada_interrompida_por_429</t>
-        </is>
-      </c>
-      <c r="B50" t="b">
-        <v>0</v>
+          <t>fornecedores_pj_sem_localizacao</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>31804</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>fornecedores_com_documento_invalido</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>1010</v>
+          <t>cnpj_rodada_interrompida_por_429</t>
+        </is>
+      </c>
+      <c r="B51" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | pago total</t>
+          <t>fornecedores_com_documento_invalido</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1799419147.56</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | transferido a outros prestadores</t>
+          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | pago total</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>43990672.26</v>
+        <v>1799419147.56</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Fundo Partidário | CANDIDATOS | pago total</t>
+          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | transferido a outros prestadores</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>82356216.09</v>
+        <v>43990672.26</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Fundo Partidário | CANDIDATOS | transferido a outros prestadores</t>
+          <t>Fundo Partidário | CANDIDATOS | pago total</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>858310.02</v>
+        <v>82356216.09</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | pago total</t>
+          <t>Fundo Partidário | CANDIDATOS | transferido a outros prestadores</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>4736266491.33</v>
+        <v>858310.02</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | transferido a outros prestadores</t>
+          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | pago total</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>4686473156.8</v>
+        <v>4729329167.93</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Fundo Partidário | PARTIDOS | pago total</t>
+          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | transferido a outros prestadores</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>464413493.97</v>
+        <v>4679535836.8</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Fundo Partidário | PARTIDOS | transferido a outros prestadores</t>
+          <t>Fundo Partidário | PARTIDOS | pago total</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>420753357.68</v>
+        <v>465311994.44</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>votacao_linhas</t>
+          <t>Fundo Partidário | PARTIDOS | transferido a outros prestadores</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0</v>
+        <v>421649296.46</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>gerado_em</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>2026-09-21 08:48:12</t>
-        </is>
+          <t>votacao_linhas</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>soma_receitas_candidatos_confere</t>
-        </is>
-      </c>
-      <c r="B62" t="b">
-        <v>1</v>
+          <t>gerado_em</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:26:41</t>
+        </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>pago_por_fornecedor_confere</t>
+          <t>soma_receitas_candidatos_confere</t>
         </is>
       </c>
       <c r="B63" t="b">
@@ -1562,32 +1562,42 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>receitas_de_sq_fora_do_cadastro</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>0</v>
+          <t>pago_por_fornecedor_confere</t>
+        </is>
+      </c>
+      <c r="B64" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>colunas_da_ordem_do_usuario_ausentes</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
+          <t>receitas_de_sq_fora_do_cadastro</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>colunas_da_ordem_do_usuario_ausentes</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
           <t>colunas_novas_fora_da_ordem_do_usuario</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
@@ -2053,7 +2063,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.9499999</v>
+        <v>575680870.95</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.77</v>
@@ -4751,7 +4761,7 @@
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>75659161.20999999</v>
+        <v>75659161.21000001</v>
       </c>
       <c r="H47" s="6" t="n">
         <v>0.23</v>
@@ -8842,7 +8852,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 08:48:12.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15505,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 08:48:12.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17216,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 08:48:12.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
         </is>
       </c>
     </row>
@@ -19245,10 +19255,10 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>548030399.4299999</v>
+        <v>559559597.25</v>
       </c>
       <c r="E89" s="12" t="n">
-        <v>23.88</v>
+        <v>23.46</v>
       </c>
     </row>
     <row r="90">
@@ -19268,10 +19278,10 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>147327590.89</v>
+        <v>152989718.15</v>
       </c>
       <c r="E90" s="12" t="n">
-        <v>6.42</v>
+        <v>6.41</v>
       </c>
     </row>
     <row r="91">
@@ -19291,10 +19301,10 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>138476052.55</v>
+        <v>145030505.46</v>
       </c>
       <c r="E91" s="12" t="n">
-        <v>6.03</v>
+        <v>6.08</v>
       </c>
     </row>
     <row r="92">
@@ -19314,10 +19324,10 @@
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>120563042.07</v>
+        <v>123005077.01</v>
       </c>
       <c r="E92" s="12" t="n">
-        <v>5.25</v>
+        <v>5.16</v>
       </c>
     </row>
     <row r="93">
@@ -19337,10 +19347,10 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>106991152.11</v>
+        <v>112131463.12</v>
       </c>
       <c r="E93" s="12" t="n">
-        <v>4.66</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="94">
@@ -19360,10 +19370,10 @@
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>89617990.20999999</v>
+        <v>94706370.86</v>
       </c>
       <c r="E94" s="12" t="n">
-        <v>3.9</v>
+        <v>3.97</v>
       </c>
     </row>
     <row r="95">
@@ -19383,10 +19393,10 @@
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>87354522.77</v>
+        <v>92584538.93000001</v>
       </c>
       <c r="E95" s="12" t="n">
-        <v>3.81</v>
+        <v>3.88</v>
       </c>
     </row>
     <row r="96">
@@ -19406,10 +19416,10 @@
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>86664426.72</v>
+        <v>91139252.15000001</v>
       </c>
       <c r="E96" s="12" t="n">
-        <v>3.78</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="97">
@@ -19429,7 +19439,7 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>84152351.08</v>
+        <v>87496556.56</v>
       </c>
       <c r="E97" s="12" t="n">
         <v>3.67</v>
@@ -19452,10 +19462,10 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>78864313.90000001</v>
+        <v>82730067.38</v>
       </c>
       <c r="E98" s="12" t="n">
-        <v>3.44</v>
+        <v>3.47</v>
       </c>
     </row>
     <row r="99">
@@ -19475,10 +19485,10 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>78688487.86</v>
+        <v>81149175.73999999</v>
       </c>
       <c r="E99" s="12" t="n">
-        <v>3.43</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="100">
@@ -19498,10 +19508,10 @@
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>69290664.54000001</v>
+        <v>72754664.08</v>
       </c>
       <c r="E100" s="12" t="n">
-        <v>3.02</v>
+        <v>3.05</v>
       </c>
     </row>
     <row r="101">
@@ -19521,10 +19531,10 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>66219472.98</v>
+        <v>69200572.7</v>
       </c>
       <c r="E101" s="12" t="n">
-        <v>2.89</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="102">
@@ -19544,7 +19554,7 @@
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>63313977.39</v>
+        <v>65843638.06</v>
       </c>
       <c r="E102" s="12" t="n">
         <v>2.76</v>
@@ -19567,10 +19577,10 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>57355532.64</v>
+        <v>60458233.91</v>
       </c>
       <c r="E103" s="12" t="n">
-        <v>2.5</v>
+        <v>2.53</v>
       </c>
     </row>
     <row r="104">
@@ -19590,10 +19600,10 @@
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>53895517.75</v>
+        <v>57231270.25</v>
       </c>
       <c r="E104" s="12" t="n">
-        <v>2.35</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="105">
@@ -19613,10 +19623,10 @@
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>49623915.24</v>
+        <v>52540469.58</v>
       </c>
       <c r="E105" s="12" t="n">
-        <v>2.16</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="106">
@@ -19636,10 +19646,10 @@
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>49091220.97</v>
+        <v>51863893.1</v>
       </c>
       <c r="E106" s="12" t="n">
-        <v>2.14</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="107">
@@ -19659,10 +19669,10 @@
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>43006662.3</v>
+        <v>44057845.64</v>
       </c>
       <c r="E107" s="12" t="n">
-        <v>1.87</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="108">
@@ -19682,10 +19692,10 @@
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>41014541.7</v>
+        <v>43313092.33</v>
       </c>
       <c r="E108" s="12" t="n">
-        <v>1.79</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="109">
@@ -19705,10 +19715,10 @@
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>40507735.88</v>
+        <v>41920605.82</v>
       </c>
       <c r="E109" s="12" t="n">
-        <v>1.77</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="110">
@@ -19728,7 +19738,7 @@
         </is>
       </c>
       <c r="D110" s="6" t="n">
-        <v>40323471.8</v>
+        <v>41916749.8</v>
       </c>
       <c r="E110" s="12" t="n">
         <v>1.76</v>
@@ -19751,7 +19761,7 @@
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>37025135.63</v>
+        <v>38501477.17</v>
       </c>
       <c r="E111" s="12" t="n">
         <v>1.61</v>
@@ -19774,10 +19784,10 @@
         </is>
       </c>
       <c r="D112" s="6" t="n">
-        <v>36640243.55</v>
+        <v>38411616.53</v>
       </c>
       <c r="E112" s="12" t="n">
-        <v>1.6</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="113">
@@ -19797,10 +19807,10 @@
         </is>
       </c>
       <c r="D113" s="6" t="n">
-        <v>33186972.51</v>
+        <v>34320412.13</v>
       </c>
       <c r="E113" s="12" t="n">
-        <v>1.45</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="114">
@@ -19820,10 +19830,10 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>23415004.22</v>
+        <v>25153987.36</v>
       </c>
       <c r="E114" s="12" t="n">
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="115">
@@ -19843,10 +19853,10 @@
         </is>
       </c>
       <c r="D115" s="6" t="n">
-        <v>23273327.69</v>
+        <v>23943473.94</v>
       </c>
       <c r="E115" s="12" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116">
@@ -22428,7 +22438,7 @@
     <row r="228">
       <c r="A228" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 08:48:12.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
         </is>
       </c>
     </row>
@@ -22442,7 +22452,7 @@
     <row r="230">
       <c r="A230" s="10" t="inlineStr">
         <is>
-          <t>Nota 1: a serie de fornecedores cobre 62.8% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
+          <t>Nota 1: a serie de fornecedores cobre 65.3% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
         </is>
       </c>
     </row>
@@ -22620,10 +22630,10 @@
         <v>4405616.89</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>13393511.95</v>
+        <v>13394786.95</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>14740734.54</v>
+        <v>14742009.54</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>11.78</v>
@@ -22930,10 +22940,10 @@
         <v>145297.42</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1209956.13</v>
+        <v>1210842.82</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>2459605.62</v>
+        <v>2460492.31</v>
       </c>
       <c r="G17" s="6" t="n">
         <v>1.97</v>
@@ -23209,10 +23219,10 @@
         <v>19500</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>29110.94</v>
+        <v>29510.94</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>252560.9</v>
+        <v>252960.9</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>0.2</v>
@@ -23547,7 +23557,7 @@
         <v>10906.01</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>86753.31</v>
+        <v>86749.91</v>
       </c>
       <c r="E37" s="6" t="n">
         <v>7321.34</v>
@@ -23559,7 +23569,7 @@
         <v>0.01</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>317908.35</v>
+        <v>317904.95</v>
       </c>
       <c r="I37" s="6" t="n">
         <v>0.02</v>
@@ -23754,7 +23764,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 08:48:12.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
         </is>
       </c>
     </row>
@@ -25281,7 +25291,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 08:48:12.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
         </is>
       </c>
     </row>
@@ -28184,7 +28194,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 08:48:12.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 21/09/2026 21:53
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -671,7 +671,7 @@
         <v>53.81</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>12371172120.18</v>
+        <v>12372157364.57</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>38.14</v>
@@ -702,7 +702,7 @@
         <v>37.17</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>8707872900.040001</v>
+        <v>8706972900.040001</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>26.84</v>
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32439034482.1</v>
+        <v>32439119726.49</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 21:19:15.</t>
         </is>
       </c>
     </row>
@@ -948,7 +948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B67"/>
+  <dimension ref="A1:B66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 21:19:15.</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>32439034482.1</v>
+        <v>32439119726.49</v>
       </c>
     </row>
     <row r="34">
@@ -1380,179 +1380,179 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>cnpj_falhas_transporte</t>
+          <t>cnpj_consultados_nesta_rodada</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>cnpj_consultados_nesta_rodada</t>
+          <t>cnpj_em_cache</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2000</v>
+        <v>17297</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>cnpj_em_cache</t>
+          <t>fornecedores_pj</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>14299</v>
+        <v>46377</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>fornecedores_pj</t>
+          <t>fornecedores_pj_sem_localizacao</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>46377</v>
+        <v>28851</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>fornecedores_pj_sem_localizacao</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>31804</v>
+          <t>cnpj_rodada_interrompida_por_429</t>
+        </is>
+      </c>
+      <c r="B50" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>cnpj_rodada_interrompida_por_429</t>
-        </is>
-      </c>
-      <c r="B51" t="b">
-        <v>0</v>
+          <t>fornecedores_com_documento_invalido</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1010</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>fornecedores_com_documento_invalido</t>
+          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | pago total</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1010</v>
+        <v>1799419147.56</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | pago total</t>
+          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | transferido a outros prestadores</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1799419147.56</v>
+        <v>43990672.26</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Fundo Especial de Financiamento de Campanha | CANDIDATOS | transferido a outros prestadores</t>
+          <t>Fundo Partidário | CANDIDATOS | pago total</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>43990672.26</v>
+        <v>82356216.09</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Fundo Partidário | CANDIDATOS | pago total</t>
+          <t>Fundo Partidário | CANDIDATOS | transferido a outros prestadores</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>82356216.09</v>
+        <v>858310.02</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Fundo Partidário | CANDIDATOS | transferido a outros prestadores</t>
+          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | pago total</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>858310.02</v>
+        <v>4729329167.93</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | pago total</t>
+          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | transferido a outros prestadores</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>4729329167.93</v>
+        <v>4679535836.8</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Fundo Especial de Financiamento de Campanha | PARTIDOS | transferido a outros prestadores</t>
+          <t>Fundo Partidário | PARTIDOS | pago total</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>4679535836.8</v>
+        <v>465311994.44</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Fundo Partidário | PARTIDOS | pago total</t>
+          <t>Fundo Partidário | PARTIDOS | transferido a outros prestadores</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>465311994.44</v>
+        <v>421649296.46</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Fundo Partidário | PARTIDOS | transferido a outros prestadores</t>
+          <t>votacao_linhas</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>421649296.46</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>votacao_linhas</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>0</v>
+          <t>gerado_em</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-09-21 21:19:15</t>
+        </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>gerado_em</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>2026-09-21 15:26:41</t>
-        </is>
+          <t>soma_receitas_candidatos_confere</t>
+        </is>
+      </c>
+      <c r="B62" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>soma_receitas_candidatos_confere</t>
+          <t>pago_por_fornecedor_confere</t>
         </is>
       </c>
       <c r="B63" t="b">
@@ -1562,42 +1562,32 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>pago_por_fornecedor_confere</t>
-        </is>
-      </c>
-      <c r="B64" t="b">
-        <v>1</v>
+          <t>receitas_de_sq_fora_do_cadastro</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>receitas_de_sq_fora_do_cadastro</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>0</v>
+          <t>colunas_da_ordem_do_usuario_ausentes</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>colunas_da_ordem_do_usuario_ausentes</t>
+          <t>colunas_novas_fora_da_ordem_do_usuario</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>colunas_novas_fora_da_ordem_do_usuario</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
@@ -2063,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.95</v>
+        <v>575680870.9499999</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.77</v>
@@ -8852,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 21:19:15.</t>
         </is>
       </c>
     </row>
@@ -15505,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 21:19:15.</t>
         </is>
       </c>
     </row>
@@ -17216,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 21:19:15.</t>
         </is>
       </c>
     </row>
@@ -19255,10 +19245,10 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>559559597.25</v>
+        <v>566657118.96</v>
       </c>
       <c r="E89" s="12" t="n">
-        <v>23.46</v>
+        <v>23.33</v>
       </c>
     </row>
     <row r="90">
@@ -19278,10 +19268,10 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>152989718.15</v>
+        <v>155238081.43</v>
       </c>
       <c r="E90" s="12" t="n">
-        <v>6.41</v>
+        <v>6.39</v>
       </c>
     </row>
     <row r="91">
@@ -19301,10 +19291,10 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>145030505.46</v>
+        <v>148266487.92</v>
       </c>
       <c r="E91" s="12" t="n">
-        <v>6.08</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="92">
@@ -19324,10 +19314,10 @@
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>123005077.01</v>
+        <v>124145548.38</v>
       </c>
       <c r="E92" s="12" t="n">
-        <v>5.16</v>
+        <v>5.11</v>
       </c>
     </row>
     <row r="93">
@@ -19347,10 +19337,10 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>112131463.12</v>
+        <v>114685296.02</v>
       </c>
       <c r="E93" s="12" t="n">
-        <v>4.7</v>
+        <v>4.72</v>
       </c>
     </row>
     <row r="94">
@@ -19370,10 +19360,10 @@
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>94706370.86</v>
+        <v>97816359.68000001</v>
       </c>
       <c r="E94" s="12" t="n">
-        <v>3.97</v>
+        <v>4.03</v>
       </c>
     </row>
     <row r="95">
@@ -19393,10 +19383,10 @@
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>92584538.93000001</v>
+        <v>94764516.70999999</v>
       </c>
       <c r="E95" s="12" t="n">
-        <v>3.88</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="96">
@@ -19416,10 +19406,10 @@
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>91139252.15000001</v>
+        <v>93129252.87</v>
       </c>
       <c r="E96" s="12" t="n">
-        <v>3.82</v>
+        <v>3.83</v>
       </c>
     </row>
     <row r="97">
@@ -19439,10 +19429,10 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>87496556.56</v>
+        <v>88938226.75</v>
       </c>
       <c r="E97" s="12" t="n">
-        <v>3.67</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="98">
@@ -19462,10 +19452,10 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>82730067.38</v>
+        <v>84507017.28</v>
       </c>
       <c r="E98" s="12" t="n">
-        <v>3.47</v>
+        <v>3.48</v>
       </c>
     </row>
     <row r="99">
@@ -19485,10 +19475,10 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>81149175.73999999</v>
+        <v>81900135.95999999</v>
       </c>
       <c r="E99" s="12" t="n">
-        <v>3.4</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="100">
@@ -19508,10 +19498,10 @@
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>72754664.08</v>
+        <v>74744454.3</v>
       </c>
       <c r="E100" s="12" t="n">
-        <v>3.05</v>
+        <v>3.08</v>
       </c>
     </row>
     <row r="101">
@@ -19531,7 +19521,7 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>69200572.7</v>
+        <v>70355357.59</v>
       </c>
       <c r="E101" s="12" t="n">
         <v>2.9</v>
@@ -19554,7 +19544,7 @@
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>65843638.06</v>
+        <v>67100547.61</v>
       </c>
       <c r="E102" s="12" t="n">
         <v>2.76</v>
@@ -19577,10 +19567,10 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>60458233.91</v>
+        <v>61936138.99</v>
       </c>
       <c r="E103" s="12" t="n">
-        <v>2.53</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="104">
@@ -19600,10 +19590,10 @@
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>57231270.25</v>
+        <v>58939356.4</v>
       </c>
       <c r="E104" s="12" t="n">
-        <v>2.4</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="105">
@@ -19623,10 +19613,10 @@
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>52540469.58</v>
+        <v>53777645.42</v>
       </c>
       <c r="E105" s="12" t="n">
-        <v>2.2</v>
+        <v>2.21</v>
       </c>
     </row>
     <row r="106">
@@ -19646,10 +19636,10 @@
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>51863893.1</v>
+        <v>53089363.21</v>
       </c>
       <c r="E106" s="12" t="n">
-        <v>2.17</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="107">
@@ -19660,19 +19650,19 @@
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Amapá</t>
+          <t>Espírito Santo</t>
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>44057845.64</v>
+        <v>44426828.53</v>
       </c>
       <c r="E107" s="12" t="n">
-        <v>1.85</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="108">
@@ -19683,16 +19673,16 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Espírito Santo</t>
+          <t>Amapá</t>
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>43313092.33</v>
+        <v>44308814.37</v>
       </c>
       <c r="E108" s="12" t="n">
         <v>1.82</v>
@@ -19706,16 +19696,16 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Alagoas</t>
+          <t>Rondônia</t>
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>41920605.82</v>
+        <v>42863716.15</v>
       </c>
       <c r="E109" s="12" t="n">
         <v>1.76</v>
@@ -19729,19 +19719,19 @@
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Rondônia</t>
+          <t>Alagoas</t>
         </is>
       </c>
       <c r="D110" s="6" t="n">
-        <v>41916749.8</v>
+        <v>42471422.45</v>
       </c>
       <c r="E110" s="12" t="n">
-        <v>1.76</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="111">
@@ -19752,16 +19742,16 @@
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Amazonas</t>
+          <t>Tocantins</t>
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>38501477.17</v>
+        <v>39178507.76</v>
       </c>
       <c r="E111" s="12" t="n">
         <v>1.61</v>
@@ -19775,16 +19765,16 @@
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Tocantins</t>
+          <t>Amazonas</t>
         </is>
       </c>
       <c r="D112" s="6" t="n">
-        <v>38411616.53</v>
+        <v>39134639.44</v>
       </c>
       <c r="E112" s="12" t="n">
         <v>1.61</v>
@@ -19807,7 +19797,7 @@
         </is>
       </c>
       <c r="D113" s="6" t="n">
-        <v>34320412.13</v>
+        <v>34914355.11</v>
       </c>
       <c r="E113" s="12" t="n">
         <v>1.44</v>
@@ -19830,10 +19820,10 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>25153987.36</v>
+        <v>25972008.08</v>
       </c>
       <c r="E114" s="12" t="n">
-        <v>1.05</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="115">
@@ -19853,7 +19843,7 @@
         </is>
       </c>
       <c r="D115" s="6" t="n">
-        <v>23943473.94</v>
+        <v>24286229.65</v>
       </c>
       <c r="E115" s="12" t="n">
         <v>1</v>
@@ -22438,7 +22428,7 @@
     <row r="228">
       <c r="A228" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 21:19:15.</t>
         </is>
       </c>
     </row>
@@ -22452,7 +22442,7 @@
     <row r="230">
       <c r="A230" s="10" t="inlineStr">
         <is>
-          <t>Nota 1: a serie de fornecedores cobre 65.3% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
+          <t>Nota 1: a serie de fornecedores cobre 66.5% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
         </is>
       </c>
     </row>
@@ -23764,7 +23754,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 21:19:15.</t>
         </is>
       </c>
     </row>
@@ -23921,7 +23911,7 @@
         <v>7.85</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>4898708042.51</v>
+        <v>4897808042.51</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>1027468247.63</v>
@@ -24013,7 +24003,7 @@
         <v>4.03</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>1816726464.43</v>
+        <v>1817691708.82</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>571969347.25</v>
@@ -24105,7 +24095,7 @@
         <v>6.24</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>2484173186.63</v>
+        <v>2484193186.63</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>494951834.63</v>
@@ -25291,7 +25281,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 21:19:15.</t>
         </is>
       </c>
     </row>
@@ -28194,7 +28184,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 15:26:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-21 21:19:15.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 22/09/2026 21:55
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -581,7 +581,7 @@
         <v>4488861531.07</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>13.84</v>
+        <v>13.85</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>0</v>
@@ -640,7 +640,7 @@
         <v>2.06</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>337096041.14</v>
+        <v>337146041.14</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>1.04</v>
@@ -671,10 +671,10 @@
         <v>53.81</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>12372157364.57</v>
+        <v>12354475064.57</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>38.14</v>
+        <v>38.11</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>1493416713.82</v>
@@ -702,10 +702,10 @@
         <v>37.17</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>8706972900.040001</v>
+        <v>8706826204.209999</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>26.84</v>
+        <v>26.86</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>3105368925.3</v>
@@ -767,7 +767,7 @@
         <v>1185110246.56</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>3.65</v>
+        <v>3.66</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>136347659.97</v>
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32439119726.49</v>
+        <v>32421340730.66</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 09:19:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 21:18:32.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 09:19:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 21:18:32.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>77233</v>
+        <v>77234</v>
       </c>
     </row>
     <row r="31">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>32439119726.49</v>
+        <v>32421340730.66</v>
       </c>
     </row>
     <row r="34">
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>20299</v>
+        <v>23299</v>
       </c>
     </row>
     <row r="48">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>26445</v>
+        <v>23468</v>
       </c>
     </row>
     <row r="50">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-22 09:19:31</t>
+          <t>2026-09-22 21:18:32</t>
         </is>
       </c>
     </row>
@@ -2053,10 +2053,10 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.9499999</v>
+        <v>575680870.95</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>1.77</v>
+        <v>1.78</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>22</v>
@@ -2198,7 +2198,7 @@
         <v>501085000</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>1.54</v>
+        <v>1.55</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>9</v>
@@ -4822,7 +4822,7 @@
         </is>
       </c>
       <c r="G48" s="6" t="n">
-        <v>75658784.06999999</v>
+        <v>75658784.07000001</v>
       </c>
       <c r="H48" s="6" t="n">
         <v>0.23</v>
@@ -5603,7 +5603,7 @@
         </is>
       </c>
       <c r="G59" s="6" t="n">
-        <v>62944315.4</v>
+        <v>62944315.40000001</v>
       </c>
       <c r="H59" s="6" t="n">
         <v>0.19</v>
@@ -6600,7 +6600,7 @@
         <v>50280000</v>
       </c>
       <c r="H73" s="6" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="I73" s="5" t="n">
         <v>3</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 09:19:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 21:18:32.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 09:19:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 21:18:32.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 09:19:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 21:18:32.</t>
         </is>
       </c>
     </row>
@@ -19245,10 +19245,10 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>582788070</v>
+        <v>586202407.04</v>
       </c>
       <c r="E89" s="12" t="n">
-        <v>23.44</v>
+        <v>23.38</v>
       </c>
     </row>
     <row r="90">
@@ -19268,10 +19268,10 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>162784561.86</v>
+        <v>163692040.49</v>
       </c>
       <c r="E90" s="12" t="n">
-        <v>6.55</v>
+        <v>6.53</v>
       </c>
     </row>
     <row r="91">
@@ -19291,10 +19291,10 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>152036260.51</v>
+        <v>154081573.55</v>
       </c>
       <c r="E91" s="12" t="n">
-        <v>6.11</v>
+        <v>6.14</v>
       </c>
     </row>
     <row r="92">
@@ -19314,10 +19314,10 @@
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>125774783.9</v>
+        <v>126366850.9</v>
       </c>
       <c r="E92" s="12" t="n">
-        <v>5.06</v>
+        <v>5.04</v>
       </c>
     </row>
     <row r="93">
@@ -19337,10 +19337,10 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>117366024.97</v>
+        <v>118592461.52</v>
       </c>
       <c r="E93" s="12" t="n">
-        <v>4.72</v>
+        <v>4.73</v>
       </c>
     </row>
     <row r="94">
@@ -19360,10 +19360,10 @@
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>101050867.01</v>
+        <v>102684036.47</v>
       </c>
       <c r="E94" s="12" t="n">
-        <v>4.06</v>
+        <v>4.09</v>
       </c>
     </row>
     <row r="95">
@@ -19383,10 +19383,10 @@
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>97403249.45</v>
+        <v>98840685.39</v>
       </c>
       <c r="E95" s="12" t="n">
-        <v>3.92</v>
+        <v>3.94</v>
       </c>
     </row>
     <row r="96">
@@ -19406,10 +19406,10 @@
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>94817568.09</v>
+        <v>95775751.31</v>
       </c>
       <c r="E96" s="12" t="n">
-        <v>3.81</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="97">
@@ -19429,10 +19429,10 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>90192566.48</v>
+        <v>90621945.61</v>
       </c>
       <c r="E97" s="12" t="n">
-        <v>3.63</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="98">
@@ -19452,7 +19452,7 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>86280095.59999999</v>
+        <v>87084855.31</v>
       </c>
       <c r="E98" s="12" t="n">
         <v>3.47</v>
@@ -19475,10 +19475,10 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>82832872.51000001</v>
+        <v>83163697.64</v>
       </c>
       <c r="E99" s="12" t="n">
-        <v>3.33</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="100">
@@ -19498,10 +19498,10 @@
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>76123580.68000001</v>
+        <v>77256447.73999999</v>
       </c>
       <c r="E100" s="12" t="n">
-        <v>3.06</v>
+        <v>3.08</v>
       </c>
     </row>
     <row r="101">
@@ -19521,7 +19521,7 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>71432907.81</v>
+        <v>72005073.73999999</v>
       </c>
       <c r="E101" s="12" t="n">
         <v>2.87</v>
@@ -19544,10 +19544,10 @@
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>68117774.27</v>
+        <v>68565335.68000001</v>
       </c>
       <c r="E102" s="12" t="n">
-        <v>2.74</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="103">
@@ -19567,10 +19567,10 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>63997669.94</v>
+        <v>64810137.51</v>
       </c>
       <c r="E103" s="12" t="n">
-        <v>2.57</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="104">
@@ -19590,7 +19590,7 @@
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>61229903.01</v>
+        <v>61774777.62</v>
       </c>
       <c r="E104" s="12" t="n">
         <v>2.46</v>
@@ -19613,7 +19613,7 @@
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>54434748.16</v>
+        <v>54880461.09</v>
       </c>
       <c r="E105" s="12" t="n">
         <v>2.19</v>
@@ -19636,10 +19636,10 @@
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>54320821.45</v>
+        <v>54848648.93</v>
       </c>
       <c r="E106" s="12" t="n">
-        <v>2.18</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="107">
@@ -19659,7 +19659,7 @@
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>44915318.26</v>
+        <v>45507143.42</v>
       </c>
       <c r="E107" s="12" t="n">
         <v>1.81</v>
@@ -19682,10 +19682,10 @@
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>44333337.7</v>
+        <v>44490631.2</v>
       </c>
       <c r="E108" s="12" t="n">
-        <v>1.78</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="109">
@@ -19705,7 +19705,7 @@
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>43429045.49</v>
+        <v>43822645.81</v>
       </c>
       <c r="E109" s="12" t="n">
         <v>1.75</v>
@@ -19728,7 +19728,7 @@
         </is>
       </c>
       <c r="D110" s="6" t="n">
-        <v>43221283.06</v>
+        <v>43511705.34</v>
       </c>
       <c r="E110" s="12" t="n">
         <v>1.74</v>
@@ -19751,7 +19751,7 @@
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>40215693.2</v>
+        <v>40626110.42</v>
       </c>
       <c r="E111" s="12" t="n">
         <v>1.62</v>
@@ -19774,7 +19774,7 @@
         </is>
       </c>
       <c r="D112" s="6" t="n">
-        <v>40024464.31</v>
+        <v>40317383.31</v>
       </c>
       <c r="E112" s="12" t="n">
         <v>1.61</v>
@@ -19797,10 +19797,10 @@
         </is>
       </c>
       <c r="D113" s="6" t="n">
-        <v>35209006.6</v>
+        <v>35355535.04</v>
       </c>
       <c r="E113" s="12" t="n">
-        <v>1.42</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="114">
@@ -19820,10 +19820,10 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>26435662.75</v>
+        <v>26822083.87</v>
       </c>
       <c r="E114" s="12" t="n">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="115">
@@ -19843,7 +19843,7 @@
         </is>
       </c>
       <c r="D115" s="6" t="n">
-        <v>24771808.17</v>
+        <v>24957278.21</v>
       </c>
       <c r="E115" s="12" t="n">
         <v>1</v>
@@ -22428,7 +22428,7 @@
     <row r="228">
       <c r="A228" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 09:19:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 21:18:32.</t>
         </is>
       </c>
     </row>
@@ -22442,7 +22442,7 @@
     <row r="230">
       <c r="A230" s="10" t="inlineStr">
         <is>
-          <t>Nota 1: a serie de fornecedores cobre 67.3% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
+          <t>Nota 1: a serie de fornecedores cobre 67.9% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
         </is>
       </c>
     </row>
@@ -23754,7 +23754,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 09:19:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 21:18:32.</t>
         </is>
       </c>
     </row>
@@ -23802,7 +23802,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
@@ -23957,7 +23957,7 @@
         <v>5.26</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>788901122.24</v>
+        <v>771218822.24</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>610172112.4</v>
@@ -24325,7 +24325,7 @@
         <v>4.6</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>930897493.99</v>
+        <v>930727493.99</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>186158214.82</v>
@@ -24877,7 +24877,7 @@
         <v>2.61</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>183981649.68</v>
+        <v>184054953.85</v>
       </c>
       <c r="E26" s="6" t="n">
         <v>8219868.98</v>
@@ -25281,7 +25281,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 09:19:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 21:18:32.</t>
         </is>
       </c>
     </row>
@@ -28184,7 +28184,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 09:19:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-22 21:18:32.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 23/09/2026 16:01
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 09:17:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 15:20:52.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 09:17:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 15:20:52.</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>26299</v>
+        <v>29298</v>
       </c>
     </row>
     <row r="48">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>20860</v>
+        <v>17880</v>
       </c>
     </row>
     <row r="50">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-23 09:17:53</t>
+          <t>2026-09-23 15:20:52</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>75659161.20999999</v>
+        <v>75659161.21000001</v>
       </c>
       <c r="H47" s="6" t="n">
         <v>0.23</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 09:17:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 15:20:52.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 09:17:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 15:20:52.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 09:17:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 15:20:52.</t>
         </is>
       </c>
     </row>
@@ -19245,10 +19245,10 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>596837953.77</v>
+        <v>598444864.4400001</v>
       </c>
       <c r="E89" s="12" t="n">
-        <v>23.49</v>
+        <v>23.46</v>
       </c>
     </row>
     <row r="90">
@@ -19268,10 +19268,10 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>164683280.01</v>
+        <v>165156983.71</v>
       </c>
       <c r="E90" s="12" t="n">
-        <v>6.48</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="91">
@@ -19291,10 +19291,10 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>156442101.35</v>
+        <v>157484419.62</v>
       </c>
       <c r="E91" s="12" t="n">
-        <v>6.16</v>
+        <v>6.17</v>
       </c>
     </row>
     <row r="92">
@@ -19314,7 +19314,7 @@
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>127146823.16</v>
+        <v>127458248.79</v>
       </c>
       <c r="E92" s="12" t="n">
         <v>5</v>
@@ -19337,10 +19337,10 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>119731453.47</v>
+        <v>120320431.42</v>
       </c>
       <c r="E93" s="12" t="n">
-        <v>4.71</v>
+        <v>4.72</v>
       </c>
     </row>
     <row r="94">
@@ -19360,10 +19360,10 @@
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>105018777.32</v>
+        <v>105831247.37</v>
       </c>
       <c r="E94" s="12" t="n">
-        <v>4.13</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="95">
@@ -19383,10 +19383,10 @@
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>100772555.84</v>
+        <v>101507628.22</v>
       </c>
       <c r="E95" s="12" t="n">
-        <v>3.97</v>
+        <v>3.98</v>
       </c>
     </row>
     <row r="96">
@@ -19406,7 +19406,7 @@
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>97133403.63</v>
+        <v>97466671.56</v>
       </c>
       <c r="E96" s="12" t="n">
         <v>3.82</v>
@@ -19429,7 +19429,7 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>91767176.59999999</v>
+        <v>91988965.93000001</v>
       </c>
       <c r="E97" s="12" t="n">
         <v>3.61</v>
@@ -19452,7 +19452,7 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>87685363</v>
+        <v>88118529.61</v>
       </c>
       <c r="E98" s="12" t="n">
         <v>3.45</v>
@@ -19475,7 +19475,7 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>83644136.72</v>
+        <v>83824991.72</v>
       </c>
       <c r="E99" s="12" t="n">
         <v>3.29</v>
@@ -19498,10 +19498,10 @@
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>78707049.53</v>
+        <v>79228185</v>
       </c>
       <c r="E100" s="12" t="n">
-        <v>3.1</v>
+        <v>3.11</v>
       </c>
     </row>
     <row r="101">
@@ -19521,10 +19521,10 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>72573697.29000001</v>
+        <v>72779424.06</v>
       </c>
       <c r="E101" s="12" t="n">
-        <v>2.86</v>
+        <v>2.85</v>
       </c>
     </row>
     <row r="102">
@@ -19544,7 +19544,7 @@
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>68851162.08</v>
+        <v>69052699.27</v>
       </c>
       <c r="E102" s="12" t="n">
         <v>2.71</v>
@@ -19567,10 +19567,10 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>66238723.53</v>
+        <v>66779026.83</v>
       </c>
       <c r="E103" s="12" t="n">
-        <v>2.61</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="104">
@@ -19590,7 +19590,7 @@
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>62369707.4</v>
+        <v>62589885.01</v>
       </c>
       <c r="E104" s="12" t="n">
         <v>2.45</v>
@@ -19613,7 +19613,7 @@
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>55859891.88</v>
+        <v>56205272.09</v>
       </c>
       <c r="E105" s="12" t="n">
         <v>2.2</v>
@@ -19636,7 +19636,7 @@
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>55239359.08</v>
+        <v>55412642.3</v>
       </c>
       <c r="E106" s="12" t="n">
         <v>2.17</v>
@@ -19659,7 +19659,7 @@
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>46220288.81</v>
+        <v>46475147.24</v>
       </c>
       <c r="E107" s="12" t="n">
         <v>1.82</v>
@@ -19682,7 +19682,7 @@
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>44590223.2</v>
+        <v>44644398.81</v>
       </c>
       <c r="E108" s="12" t="n">
         <v>1.75</v>
@@ -19705,7 +19705,7 @@
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>44252658.84</v>
+        <v>44471806.78</v>
       </c>
       <c r="E109" s="12" t="n">
         <v>1.74</v>
@@ -19728,7 +19728,7 @@
         </is>
       </c>
       <c r="D110" s="6" t="n">
-        <v>43680404.44</v>
+        <v>43803566.64</v>
       </c>
       <c r="E110" s="12" t="n">
         <v>1.72</v>
@@ -19751,7 +19751,7 @@
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>41867563.86</v>
+        <v>42032253.44</v>
       </c>
       <c r="E111" s="12" t="n">
         <v>1.65</v>
@@ -19774,7 +19774,7 @@
         </is>
       </c>
       <c r="D112" s="6" t="n">
-        <v>40670496.86</v>
+        <v>40808673.05</v>
       </c>
       <c r="E112" s="12" t="n">
         <v>1.6</v>
@@ -19797,10 +19797,10 @@
         </is>
       </c>
       <c r="D113" s="6" t="n">
-        <v>35469082.96</v>
+        <v>35534051.36</v>
       </c>
       <c r="E113" s="12" t="n">
-        <v>1.4</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="114">
@@ -19820,7 +19820,7 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>27151030.86</v>
+        <v>27320526.46</v>
       </c>
       <c r="E114" s="12" t="n">
         <v>1.07</v>
@@ -19843,7 +19843,7 @@
         </is>
       </c>
       <c r="D115" s="6" t="n">
-        <v>25234984.45</v>
+        <v>25286467.35</v>
       </c>
       <c r="E115" s="12" t="n">
         <v>0.99</v>
@@ -22428,7 +22428,7 @@
     <row r="228">
       <c r="A228" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 09:17:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 15:20:52.</t>
         </is>
       </c>
     </row>
@@ -22442,7 +22442,7 @@
     <row r="230">
       <c r="A230" s="10" t="inlineStr">
         <is>
-          <t>Nota 1: a serie de fornecedores cobre 68.3% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
+          <t>Nota 1: a serie de fornecedores cobre 68.6% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
         </is>
       </c>
     </row>
@@ -23754,7 +23754,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 09:17:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 15:20:52.</t>
         </is>
       </c>
     </row>
@@ -25281,7 +25281,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 09:17:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 15:20:52.</t>
         </is>
       </c>
     </row>
@@ -28184,7 +28184,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 09:17:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-23 15:20:52.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 24/09/2026 09:53
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 07:47:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 07:47:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>34299</v>
+        <v>36299</v>
       </c>
     </row>
     <row r="48">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>13353</v>
+        <v>11382</v>
       </c>
     </row>
     <row r="50">
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>4764744082.58</v>
+        <v>4772139234.33</v>
       </c>
     </row>
     <row r="57">
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>4714432640.58</v>
+        <v>4718525185.58</v>
       </c>
     </row>
     <row r="58">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>476531234.12</v>
+        <v>479003500.02</v>
       </c>
     </row>
     <row r="59">
@@ -1514,7 +1514,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>431335868.73</v>
+        <v>433269095.24</v>
       </c>
     </row>
     <row r="60">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-24 07:47:46</t>
+          <t>2026-09-24 09:19:07</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.95</v>
+        <v>575680870.9499999</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.78</v>
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>75659161.21000001</v>
+        <v>75659161.20999999</v>
       </c>
       <c r="H47" s="6" t="n">
         <v>0.23</v>
@@ -5603,7 +5603,7 @@
         </is>
       </c>
       <c r="G59" s="6" t="n">
-        <v>62944315.40000001</v>
+        <v>62944315.4</v>
       </c>
       <c r="H59" s="6" t="n">
         <v>0.19</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 07:47:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 07:47:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 07:47:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
         </is>
       </c>
     </row>
@@ -17245,7 +17245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E231"/>
+  <dimension ref="A1:E232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="47" customWidth="1" min="1" max="1"/>
@@ -19245,10 +19245,10 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>610066087</v>
+        <v>610399910.0599999</v>
       </c>
       <c r="E89" s="12" t="n">
-        <v>23.64</v>
+        <v>23.63</v>
       </c>
     </row>
     <row r="90">
@@ -19268,7 +19268,7 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>167360024.85</v>
+        <v>167437678.87</v>
       </c>
       <c r="E90" s="12" t="n">
         <v>6.48</v>
@@ -19291,10 +19291,10 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>160040844.6</v>
+        <v>160315545.81</v>
       </c>
       <c r="E91" s="12" t="n">
-        <v>6.2</v>
+        <v>6.21</v>
       </c>
     </row>
     <row r="92">
@@ -19314,7 +19314,7 @@
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>128277981.05</v>
+        <v>128343924.02</v>
       </c>
       <c r="E92" s="12" t="n">
         <v>4.97</v>
@@ -19337,7 +19337,7 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>121414088.47</v>
+        <v>121512202.79</v>
       </c>
       <c r="E93" s="12" t="n">
         <v>4.7</v>
@@ -19360,7 +19360,7 @@
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>106878184.52</v>
+        <v>107062353.14</v>
       </c>
       <c r="E94" s="12" t="n">
         <v>4.14</v>
@@ -19383,7 +19383,7 @@
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>102860939.22</v>
+        <v>103040938.56</v>
       </c>
       <c r="E95" s="12" t="n">
         <v>3.99</v>
@@ -19406,7 +19406,7 @@
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>98512850.88</v>
+        <v>98581276.86</v>
       </c>
       <c r="E96" s="12" t="n">
         <v>3.82</v>
@@ -19429,7 +19429,7 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>92424083.16</v>
+        <v>92451872.34999999</v>
       </c>
       <c r="E97" s="12" t="n">
         <v>3.58</v>
@@ -19452,7 +19452,7 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>88566491.56</v>
+        <v>88629734.43000001</v>
       </c>
       <c r="E98" s="12" t="n">
         <v>3.43</v>
@@ -19475,7 +19475,7 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>84112765.19</v>
+        <v>84157310.75</v>
       </c>
       <c r="E99" s="12" t="n">
         <v>3.26</v>
@@ -19498,7 +19498,7 @@
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>80214793.27</v>
+        <v>80328521.43000001</v>
       </c>
       <c r="E100" s="12" t="n">
         <v>3.11</v>
@@ -19521,7 +19521,7 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>73072162.7</v>
+        <v>73117225.06</v>
       </c>
       <c r="E101" s="12" t="n">
         <v>2.83</v>
@@ -19544,7 +19544,7 @@
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>69505943.75</v>
+        <v>69544574.78</v>
       </c>
       <c r="E102" s="12" t="n">
         <v>2.69</v>
@@ -19567,7 +19567,7 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>67622093.89</v>
+        <v>67724974.7</v>
       </c>
       <c r="E103" s="12" t="n">
         <v>2.62</v>
@@ -19590,7 +19590,7 @@
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>63390322.43</v>
+        <v>63445152.62</v>
       </c>
       <c r="E104" s="12" t="n">
         <v>2.46</v>
@@ -19613,7 +19613,7 @@
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>56936427.55</v>
+        <v>57006831.18</v>
       </c>
       <c r="E105" s="12" t="n">
         <v>2.21</v>
@@ -19636,7 +19636,7 @@
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>55594909.26</v>
+        <v>55631376.34</v>
       </c>
       <c r="E106" s="12" t="n">
         <v>2.15</v>
@@ -19659,7 +19659,7 @@
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>47128542.41</v>
+        <v>47201182.01</v>
       </c>
       <c r="E107" s="12" t="n">
         <v>1.83</v>
@@ -19682,7 +19682,7 @@
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>44923739.43</v>
+        <v>44938130.46</v>
       </c>
       <c r="E108" s="12" t="n">
         <v>1.74</v>
@@ -19705,7 +19705,7 @@
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>44815685.95</v>
+        <v>44887831.16</v>
       </c>
       <c r="E109" s="12" t="n">
         <v>1.74</v>
@@ -19728,7 +19728,7 @@
         </is>
       </c>
       <c r="D110" s="6" t="n">
-        <v>43945126.59</v>
+        <v>43976203.98</v>
       </c>
       <c r="E110" s="12" t="n">
         <v>1.7</v>
@@ -19751,7 +19751,7 @@
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>42236505.79</v>
+        <v>42273490.41</v>
       </c>
       <c r="E111" s="12" t="n">
         <v>1.64</v>
@@ -19774,7 +19774,7 @@
         </is>
       </c>
       <c r="D112" s="6" t="n">
-        <v>41491444.46</v>
+        <v>41517892.79</v>
       </c>
       <c r="E112" s="12" t="n">
         <v>1.61</v>
@@ -19797,7 +19797,7 @@
         </is>
       </c>
       <c r="D113" s="6" t="n">
-        <v>35604161.05</v>
+        <v>35611767.07</v>
       </c>
       <c r="E113" s="12" t="n">
         <v>1.38</v>
@@ -19820,7 +19820,7 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>27533766.51</v>
+        <v>27567405.68</v>
       </c>
       <c r="E114" s="12" t="n">
         <v>1.07</v>
@@ -19843,7 +19843,7 @@
         </is>
       </c>
       <c r="D115" s="6" t="n">
-        <v>25328005.44</v>
+        <v>25341311.92</v>
       </c>
       <c r="E115" s="12" t="n">
         <v>0.98</v>
@@ -19875,24 +19875,24 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>Valor doado, pela UF do doador</t>
+          <t>Valor contratado de fornecedores</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>EX</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>EX</t>
         </is>
       </c>
       <c r="D117" s="6" t="n">
-        <v>114899305.01</v>
+        <v>1010.55</v>
       </c>
       <c r="E117" s="12" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
@@ -19903,19 +19903,19 @@
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>Rio de Janeiro</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D118" s="6" t="n">
-        <v>40037432.89</v>
+        <v>114899305.01</v>
       </c>
       <c r="E118" s="12" t="n">
-        <v>7.67</v>
+        <v>22</v>
       </c>
     </row>
     <row r="119">
@@ -19926,19 +19926,19 @@
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>Minas Gerais</t>
+          <t>Rio de Janeiro</t>
         </is>
       </c>
       <c r="D119" s="6" t="n">
-        <v>38680832.03</v>
+        <v>40037432.89</v>
       </c>
       <c r="E119" s="12" t="n">
-        <v>7.41</v>
+        <v>7.67</v>
       </c>
     </row>
     <row r="120">
@@ -19949,19 +19949,19 @@
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Minas Gerais</t>
         </is>
       </c>
       <c r="D120" s="6" t="n">
-        <v>36464616.78</v>
+        <v>38680832.03</v>
       </c>
       <c r="E120" s="12" t="n">
-        <v>6.98</v>
+        <v>7.41</v>
       </c>
     </row>
     <row r="121">
@@ -19972,19 +19972,19 @@
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>Goiás</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D121" s="6" t="n">
-        <v>25243345.44</v>
+        <v>36464616.78</v>
       </c>
       <c r="E121" s="12" t="n">
-        <v>4.83</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="122">
@@ -19995,19 +19995,19 @@
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Sul</t>
+          <t>Goiás</t>
         </is>
       </c>
       <c r="D122" s="6" t="n">
-        <v>21817618.71</v>
+        <v>25243345.44</v>
       </c>
       <c r="E122" s="12" t="n">
-        <v>4.18</v>
+        <v>4.83</v>
       </c>
     </row>
     <row r="123">
@@ -20018,19 +20018,19 @@
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>Santa Catarina</t>
+          <t>Rio Grande do Sul</t>
         </is>
       </c>
       <c r="D123" s="6" t="n">
-        <v>19557005.19</v>
+        <v>21817618.71</v>
       </c>
       <c r="E123" s="12" t="n">
-        <v>3.74</v>
+        <v>4.18</v>
       </c>
     </row>
     <row r="124">
@@ -20041,19 +20041,19 @@
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>Pernambuco</t>
+          <t>Santa Catarina</t>
         </is>
       </c>
       <c r="D124" s="6" t="n">
-        <v>18614196.06</v>
+        <v>19557005.19</v>
       </c>
       <c r="E124" s="12" t="n">
-        <v>3.56</v>
+        <v>3.74</v>
       </c>
     </row>
     <row r="125">
@@ -20064,19 +20064,19 @@
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso</t>
+          <t>Pernambuco</t>
         </is>
       </c>
       <c r="D125" s="6" t="n">
-        <v>17994047.39</v>
+        <v>18614196.06</v>
       </c>
       <c r="E125" s="12" t="n">
-        <v>3.45</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="126">
@@ -20087,19 +20087,19 @@
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>Distrito Federal</t>
+          <t>Mato Grosso</t>
         </is>
       </c>
       <c r="D126" s="6" t="n">
-        <v>16168065.74</v>
+        <v>17994047.39</v>
       </c>
       <c r="E126" s="12" t="n">
-        <v>3.1</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="127">
@@ -20110,19 +20110,19 @@
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>Tocantins</t>
+          <t>Distrito Federal</t>
         </is>
       </c>
       <c r="D127" s="6" t="n">
-        <v>15430690.89</v>
+        <v>16168065.74</v>
       </c>
       <c r="E127" s="12" t="n">
-        <v>2.95</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="128">
@@ -20133,19 +20133,19 @@
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>Maranhão</t>
+          <t>Tocantins</t>
         </is>
       </c>
       <c r="D128" s="6" t="n">
-        <v>15374746.01</v>
+        <v>15430690.89</v>
       </c>
       <c r="E128" s="12" t="n">
-        <v>2.94</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="129">
@@ -20156,19 +20156,19 @@
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Espírito Santo</t>
+          <t>Maranhão</t>
         </is>
       </c>
       <c r="D129" s="6" t="n">
-        <v>15167790.85</v>
+        <v>15374746.01</v>
       </c>
       <c r="E129" s="12" t="n">
-        <v>2.9</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="130">
@@ -20179,19 +20179,19 @@
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Paraíba</t>
+          <t>Espírito Santo</t>
         </is>
       </c>
       <c r="D130" s="6" t="n">
-        <v>14662450.88</v>
+        <v>15167790.85</v>
       </c>
       <c r="E130" s="12" t="n">
-        <v>2.81</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="131">
@@ -20202,19 +20202,19 @@
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Paraíba</t>
         </is>
       </c>
       <c r="D131" s="6" t="n">
-        <v>13504364.28</v>
+        <v>14662450.88</v>
       </c>
       <c r="E131" s="12" t="n">
-        <v>2.59</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="132">
@@ -20225,19 +20225,19 @@
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso do Sul</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="D132" s="6" t="n">
-        <v>11395718.8</v>
+        <v>13504364.28</v>
       </c>
       <c r="E132" s="12" t="n">
-        <v>2.18</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="133">
@@ -20248,16 +20248,16 @@
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Pará</t>
+          <t>Mato Grosso do Sul</t>
         </is>
       </c>
       <c r="D133" s="6" t="n">
-        <v>11374266.99</v>
+        <v>11395718.8</v>
       </c>
       <c r="E133" s="12" t="n">
         <v>2.18</v>
@@ -20271,19 +20271,19 @@
       </c>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Rondônia</t>
+          <t>Pará</t>
         </is>
       </c>
       <c r="D134" s="6" t="n">
-        <v>10909260.75</v>
+        <v>11374266.99</v>
       </c>
       <c r="E134" s="12" t="n">
-        <v>2.09</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="135">
@@ -20294,19 +20294,19 @@
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Amazonas</t>
+          <t>Rondônia</t>
         </is>
       </c>
       <c r="D135" s="6" t="n">
-        <v>9559738.529999999</v>
+        <v>10909260.75</v>
       </c>
       <c r="E135" s="12" t="n">
-        <v>1.83</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="136">
@@ -20317,19 +20317,19 @@
       </c>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Amazonas</t>
         </is>
       </c>
       <c r="D136" s="6" t="n">
-        <v>9421680.49</v>
+        <v>9559738.529999999</v>
       </c>
       <c r="E136" s="12" t="n">
-        <v>1.8</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="137">
@@ -20340,19 +20340,19 @@
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>Piauí</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="D137" s="6" t="n">
-        <v>8552970.23</v>
+        <v>9421680.49</v>
       </c>
       <c r="E137" s="12" t="n">
-        <v>1.64</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="138">
@@ -20363,19 +20363,19 @@
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>Acre</t>
+          <t>Piauí</t>
         </is>
       </c>
       <c r="D138" s="6" t="n">
-        <v>7472958.47</v>
+        <v>8552970.23</v>
       </c>
       <c r="E138" s="12" t="n">
-        <v>1.43</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="139">
@@ -20386,19 +20386,19 @@
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>Roraima</t>
+          <t>Acre</t>
         </is>
       </c>
       <c r="D139" s="6" t="n">
-        <v>7155890.22</v>
+        <v>7472958.47</v>
       </c>
       <c r="E139" s="12" t="n">
-        <v>1.37</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="140">
@@ -20409,19 +20409,19 @@
       </c>
       <c r="B140" s="4" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Alagoas</t>
+          <t>Roraima</t>
         </is>
       </c>
       <c r="D140" s="6" t="n">
-        <v>6781567.4</v>
+        <v>7155890.22</v>
       </c>
       <c r="E140" s="12" t="n">
-        <v>1.3</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="141">
@@ -20432,19 +20432,19 @@
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>Sergipe</t>
+          <t>Alagoas</t>
         </is>
       </c>
       <c r="D141" s="6" t="n">
-        <v>5626098.78</v>
+        <v>6781567.4</v>
       </c>
       <c r="E141" s="12" t="n">
-        <v>1.08</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="142">
@@ -20455,19 +20455,19 @@
       </c>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>Amapá</t>
+          <t>Sergipe</t>
         </is>
       </c>
       <c r="D142" s="6" t="n">
-        <v>5383564.5</v>
+        <v>5626098.78</v>
       </c>
       <c r="E142" s="12" t="n">
-        <v>1.03</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="143">
@@ -20478,42 +20478,42 @@
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Norte</t>
+          <t>Amapá</t>
         </is>
       </c>
       <c r="D143" s="6" t="n">
-        <v>5013592.3</v>
+        <v>5383564.5</v>
       </c>
       <c r="E143" s="12" t="n">
-        <v>0.96</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>Doacao de pessoa fisica, pela UF do candidato</t>
+          <t>Valor doado, pela UF do doador</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Rio Grande do Norte</t>
         </is>
       </c>
       <c r="D144" s="6" t="n">
-        <v>64138783.06</v>
+        <v>5013592.3</v>
       </c>
       <c r="E144" s="12" t="n">
-        <v>15.75</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="145">
@@ -20524,19 +20524,19 @@
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>Minas Gerais</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D145" s="6" t="n">
-        <v>51151182.79</v>
+        <v>64138783.06</v>
       </c>
       <c r="E145" s="12" t="n">
-        <v>12.56</v>
+        <v>15.75</v>
       </c>
     </row>
     <row r="146">
@@ -20547,19 +20547,19 @@
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso</t>
+          <t>Minas Gerais</t>
         </is>
       </c>
       <c r="D146" s="6" t="n">
-        <v>24233913.07</v>
+        <v>51151182.79</v>
       </c>
       <c r="E146" s="12" t="n">
-        <v>5.95</v>
+        <v>12.56</v>
       </c>
     </row>
     <row r="147">
@@ -20570,19 +20570,19 @@
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Mato Grosso</t>
         </is>
       </c>
       <c r="D147" s="6" t="n">
-        <v>23033154.85</v>
+        <v>24233913.07</v>
       </c>
       <c r="E147" s="12" t="n">
-        <v>5.66</v>
+        <v>5.95</v>
       </c>
     </row>
     <row r="148">
@@ -20593,19 +20593,19 @@
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>Rio de Janeiro</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="D148" s="6" t="n">
-        <v>22671481.34</v>
+        <v>23033154.85</v>
       </c>
       <c r="E148" s="12" t="n">
-        <v>5.57</v>
+        <v>5.66</v>
       </c>
     </row>
     <row r="149">
@@ -20616,19 +20616,19 @@
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Rio de Janeiro</t>
         </is>
       </c>
       <c r="D149" s="6" t="n">
-        <v>21672779.44</v>
+        <v>22671481.34</v>
       </c>
       <c r="E149" s="12" t="n">
-        <v>5.32</v>
+        <v>5.57</v>
       </c>
     </row>
     <row r="150">
@@ -20639,19 +20639,19 @@
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>Goiás</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D150" s="6" t="n">
-        <v>20038777.52</v>
+        <v>21672779.44</v>
       </c>
       <c r="E150" s="12" t="n">
-        <v>4.92</v>
+        <v>5.32</v>
       </c>
     </row>
     <row r="151">
@@ -20662,19 +20662,19 @@
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Sul</t>
+          <t>Goiás</t>
         </is>
       </c>
       <c r="D151" s="6" t="n">
-        <v>19005254.09</v>
+        <v>20038777.52</v>
       </c>
       <c r="E151" s="12" t="n">
-        <v>4.67</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="152">
@@ -20685,19 +20685,19 @@
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Rio Grande do Sul</t>
         </is>
       </c>
       <c r="D152" s="6" t="n">
-        <v>15656007.44</v>
+        <v>19005254.09</v>
       </c>
       <c r="E152" s="12" t="n">
-        <v>3.85</v>
+        <v>4.67</v>
       </c>
     </row>
     <row r="153">
@@ -20708,19 +20708,19 @@
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>Santa Catarina</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="D153" s="6" t="n">
-        <v>15407239.46</v>
+        <v>15656007.44</v>
       </c>
       <c r="E153" s="12" t="n">
-        <v>3.78</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="154">
@@ -20731,19 +20731,19 @@
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>Distrito Federal</t>
+          <t>Santa Catarina</t>
         </is>
       </c>
       <c r="D154" s="6" t="n">
-        <v>14420380.52</v>
+        <v>15407239.46</v>
       </c>
       <c r="E154" s="12" t="n">
-        <v>3.54</v>
+        <v>3.78</v>
       </c>
     </row>
     <row r="155">
@@ -20754,19 +20754,19 @@
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>Pernambuco</t>
+          <t>Distrito Federal</t>
         </is>
       </c>
       <c r="D155" s="6" t="n">
-        <v>12974654.42</v>
+        <v>14420380.52</v>
       </c>
       <c r="E155" s="12" t="n">
-        <v>3.19</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="156">
@@ -20777,19 +20777,19 @@
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>Maranhão</t>
+          <t>Pernambuco</t>
         </is>
       </c>
       <c r="D156" s="6" t="n">
-        <v>12497985.68</v>
+        <v>12974654.42</v>
       </c>
       <c r="E156" s="12" t="n">
-        <v>3.07</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="157">
@@ -20800,19 +20800,19 @@
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Rondônia</t>
+          <t>Maranhão</t>
         </is>
       </c>
       <c r="D157" s="6" t="n">
-        <v>11093129.79</v>
+        <v>12497985.68</v>
       </c>
       <c r="E157" s="12" t="n">
-        <v>2.72</v>
+        <v>3.07</v>
       </c>
     </row>
     <row r="158">
@@ -20823,19 +20823,19 @@
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>Pará</t>
+          <t>Rondônia</t>
         </is>
       </c>
       <c r="D158" s="6" t="n">
-        <v>9846151.369999999</v>
+        <v>11093129.79</v>
       </c>
       <c r="E158" s="12" t="n">
-        <v>2.42</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="159">
@@ -20846,19 +20846,19 @@
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>Piauí</t>
+          <t>Pará</t>
         </is>
       </c>
       <c r="D159" s="6" t="n">
-        <v>8884066.109999999</v>
+        <v>9846151.369999999</v>
       </c>
       <c r="E159" s="12" t="n">
-        <v>2.18</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="160">
@@ -20869,19 +20869,19 @@
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>Espírito Santo</t>
+          <t>Piauí</t>
         </is>
       </c>
       <c r="D160" s="6" t="n">
-        <v>8176294.7</v>
+        <v>8884066.109999999</v>
       </c>
       <c r="E160" s="12" t="n">
-        <v>2.01</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="161">
@@ -20892,19 +20892,19 @@
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Presidenciáveis, circunscrição nacional</t>
+          <t>Espírito Santo</t>
         </is>
       </c>
       <c r="D161" s="6" t="n">
-        <v>8044237.19</v>
+        <v>8176294.7</v>
       </c>
       <c r="E161" s="12" t="n">
-        <v>1.98</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="162">
@@ -20915,19 +20915,19 @@
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>Amazonas</t>
+          <t>Presidenciáveis, circunscrição nacional</t>
         </is>
       </c>
       <c r="D162" s="6" t="n">
-        <v>6783926.8</v>
+        <v>8044237.19</v>
       </c>
       <c r="E162" s="12" t="n">
-        <v>1.67</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="163">
@@ -20938,19 +20938,19 @@
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>Tocantins</t>
+          <t>Amazonas</t>
         </is>
       </c>
       <c r="D163" s="6" t="n">
-        <v>6584908.54</v>
+        <v>6783926.8</v>
       </c>
       <c r="E163" s="12" t="n">
-        <v>1.62</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="164">
@@ -20961,19 +20961,19 @@
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>Sergipe</t>
+          <t>Tocantins</t>
         </is>
       </c>
       <c r="D164" s="6" t="n">
-        <v>5743109.92</v>
+        <v>6584908.54</v>
       </c>
       <c r="E164" s="12" t="n">
-        <v>1.41</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="165">
@@ -20984,19 +20984,19 @@
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso do Sul</t>
+          <t>Sergipe</t>
         </is>
       </c>
       <c r="D165" s="6" t="n">
-        <v>5693835.81</v>
+        <v>5743109.92</v>
       </c>
       <c r="E165" s="12" t="n">
-        <v>1.4</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="166">
@@ -21007,19 +21007,19 @@
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>Paraíba</t>
+          <t>Mato Grosso do Sul</t>
         </is>
       </c>
       <c r="D166" s="6" t="n">
-        <v>4614157.08</v>
+        <v>5693835.81</v>
       </c>
       <c r="E166" s="12" t="n">
-        <v>1.13</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="167">
@@ -21030,19 +21030,19 @@
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>Alagoas</t>
+          <t>Paraíba</t>
         </is>
       </c>
       <c r="D167" s="6" t="n">
-        <v>4562900.79</v>
+        <v>4614157.08</v>
       </c>
       <c r="E167" s="12" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="168">
@@ -21053,19 +21053,19 @@
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>Acre</t>
+          <t>Alagoas</t>
         </is>
       </c>
       <c r="D168" s="6" t="n">
-        <v>3173862.49</v>
+        <v>4562900.79</v>
       </c>
       <c r="E168" s="12" t="n">
-        <v>0.78</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="169">
@@ -21076,19 +21076,19 @@
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Norte</t>
+          <t>Acre</t>
         </is>
       </c>
       <c r="D169" s="6" t="n">
-        <v>2673769.35</v>
+        <v>3173862.49</v>
       </c>
       <c r="E169" s="12" t="n">
-        <v>0.66</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="170">
@@ -21099,19 +21099,19 @@
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>Roraima</t>
+          <t>Rio Grande do Norte</t>
         </is>
       </c>
       <c r="D170" s="6" t="n">
-        <v>2589888.97</v>
+        <v>2673769.35</v>
       </c>
       <c r="E170" s="12" t="n">
-        <v>0.64</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="171">
@@ -21122,42 +21122,42 @@
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>Amapá</t>
+          <t>Roraima</t>
         </is>
       </c>
       <c r="D171" s="6" t="n">
-        <v>1755108.36</v>
+        <v>2589888.97</v>
       </c>
       <c r="E171" s="12" t="n">
-        <v>0.43</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>candidatos</t>
+          <t>Doacao de pessoa fisica, pela UF do candidato</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Amapá</t>
         </is>
       </c>
       <c r="D172" s="6" t="n">
-        <v>2630</v>
+        <v>1755108.36</v>
       </c>
       <c r="E172" s="12" t="n">
-        <v>12.53</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="173">
@@ -21168,19 +21168,19 @@
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>Rio de Janeiro</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D173" s="6" t="n">
-        <v>2055</v>
+        <v>2630</v>
       </c>
       <c r="E173" s="12" t="n">
-        <v>9.789999999999999</v>
+        <v>12.53</v>
       </c>
     </row>
     <row r="174">
@@ -21191,19 +21191,19 @@
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>Minas Gerais</t>
+          <t>Rio de Janeiro</t>
         </is>
       </c>
       <c r="D174" s="6" t="n">
-        <v>1832</v>
+        <v>2055</v>
       </c>
       <c r="E174" s="12" t="n">
-        <v>8.73</v>
+        <v>9.789999999999999</v>
       </c>
     </row>
     <row r="175">
@@ -21214,19 +21214,19 @@
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Minas Gerais</t>
         </is>
       </c>
       <c r="D175" s="6" t="n">
-        <v>1224</v>
+        <v>1832</v>
       </c>
       <c r="E175" s="12" t="n">
-        <v>5.83</v>
+        <v>8.73</v>
       </c>
     </row>
     <row r="176">
@@ -21237,19 +21237,19 @@
       </c>
       <c r="B176" s="4" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="D176" s="6" t="n">
-        <v>1090</v>
+        <v>1224</v>
       </c>
       <c r="E176" s="12" t="n">
-        <v>5.19</v>
+        <v>5.83</v>
       </c>
     </row>
     <row r="177">
@@ -21260,19 +21260,19 @@
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Sul</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D177" s="6" t="n">
-        <v>1053</v>
+        <v>1090</v>
       </c>
       <c r="E177" s="12" t="n">
-        <v>5.02</v>
+        <v>5.19</v>
       </c>
     </row>
     <row r="178">
@@ -21283,19 +21283,19 @@
       </c>
       <c r="B178" s="4" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>Pernambuco</t>
+          <t>Rio Grande do Sul</t>
         </is>
       </c>
       <c r="D178" s="6" t="n">
-        <v>961</v>
+        <v>1053</v>
       </c>
       <c r="E178" s="12" t="n">
-        <v>4.58</v>
+        <v>5.02</v>
       </c>
     </row>
     <row r="179">
@@ -21306,19 +21306,19 @@
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>Goiás</t>
+          <t>Pernambuco</t>
         </is>
       </c>
       <c r="D179" s="6" t="n">
-        <v>905</v>
+        <v>961</v>
       </c>
       <c r="E179" s="12" t="n">
-        <v>4.31</v>
+        <v>4.58</v>
       </c>
     </row>
     <row r="180">
@@ -21329,19 +21329,19 @@
       </c>
       <c r="B180" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>Pará</t>
+          <t>Goiás</t>
         </is>
       </c>
       <c r="D180" s="6" t="n">
-        <v>741</v>
+        <v>905</v>
       </c>
       <c r="E180" s="12" t="n">
-        <v>3.53</v>
+        <v>4.31</v>
       </c>
     </row>
     <row r="181">
@@ -21352,19 +21352,19 @@
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Pará</t>
         </is>
       </c>
       <c r="D181" s="6" t="n">
-        <v>713</v>
+        <v>741</v>
       </c>
       <c r="E181" s="12" t="n">
-        <v>3.4</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="182">
@@ -21375,19 +21375,19 @@
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
         <is>
-          <t>Santa Catarina</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="D182" s="6" t="n">
-        <v>700</v>
+        <v>713</v>
       </c>
       <c r="E182" s="12" t="n">
-        <v>3.34</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="183">
@@ -21398,19 +21398,19 @@
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>Distrito Federal</t>
+          <t>Santa Catarina</t>
         </is>
       </c>
       <c r="D183" s="6" t="n">
-        <v>668</v>
+        <v>700</v>
       </c>
       <c r="E183" s="12" t="n">
-        <v>3.18</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="184">
@@ -21421,19 +21421,19 @@
       </c>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="C184" s="4" t="inlineStr">
         <is>
-          <t>Maranhão</t>
+          <t>Distrito Federal</t>
         </is>
       </c>
       <c r="D184" s="6" t="n">
-        <v>619</v>
+        <v>668</v>
       </c>
       <c r="E184" s="12" t="n">
-        <v>2.95</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="185">
@@ -21444,19 +21444,19 @@
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>Espírito Santo</t>
+          <t>Maranhão</t>
         </is>
       </c>
       <c r="D185" s="6" t="n">
-        <v>591</v>
+        <v>619</v>
       </c>
       <c r="E185" s="12" t="n">
-        <v>2.82</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="186">
@@ -21467,19 +21467,19 @@
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Amazonas</t>
+          <t>Espírito Santo</t>
         </is>
       </c>
       <c r="D186" s="6" t="n">
-        <v>475</v>
+        <v>591</v>
       </c>
       <c r="E186" s="12" t="n">
-        <v>2.26</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="187">
@@ -21490,19 +21490,19 @@
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso</t>
+          <t>Amazonas</t>
         </is>
       </c>
       <c r="D187" s="6" t="n">
-        <v>455</v>
+        <v>475</v>
       </c>
       <c r="E187" s="12" t="n">
-        <v>2.17</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="188">
@@ -21513,19 +21513,19 @@
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t>Paraíba</t>
+          <t>Mato Grosso</t>
         </is>
       </c>
       <c r="D188" s="6" t="n">
-        <v>450</v>
+        <v>455</v>
       </c>
       <c r="E188" s="12" t="n">
-        <v>2.14</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="189">
@@ -21536,19 +21536,19 @@
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C189" s="4" t="inlineStr">
         <is>
-          <t>Rondônia</t>
+          <t>Paraíba</t>
         </is>
       </c>
       <c r="D189" s="6" t="n">
-        <v>438</v>
+        <v>450</v>
       </c>
       <c r="E189" s="12" t="n">
-        <v>2.09</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="190">
@@ -21559,19 +21559,19 @@
       </c>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso do Sul</t>
+          <t>Rondônia</t>
         </is>
       </c>
       <c r="D190" s="6" t="n">
-        <v>425</v>
+        <v>438</v>
       </c>
       <c r="E190" s="12" t="n">
-        <v>2.03</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="191">
@@ -21582,19 +21582,19 @@
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
         <is>
-          <t>Roraima</t>
+          <t>Mato Grosso do Sul</t>
         </is>
       </c>
       <c r="D191" s="6" t="n">
-        <v>413</v>
+        <v>425</v>
       </c>
       <c r="E191" s="12" t="n">
-        <v>1.97</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="192">
@@ -21605,19 +21605,19 @@
       </c>
       <c r="B192" s="4" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
         <is>
-          <t>Sergipe</t>
+          <t>Roraima</t>
         </is>
       </c>
       <c r="D192" s="6" t="n">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="E192" s="12" t="n">
-        <v>1.96</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="193">
@@ -21628,19 +21628,19 @@
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
         <is>
-          <t>Piauí</t>
+          <t>Sergipe</t>
         </is>
       </c>
       <c r="D193" s="6" t="n">
-        <v>402</v>
+        <v>411</v>
       </c>
       <c r="E193" s="12" t="n">
-        <v>1.92</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="194">
@@ -21651,19 +21651,19 @@
       </c>
       <c r="B194" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
         <is>
-          <t>Acre</t>
+          <t>Piauí</t>
         </is>
       </c>
       <c r="D194" s="6" t="n">
-        <v>388</v>
+        <v>402</v>
       </c>
       <c r="E194" s="12" t="n">
-        <v>1.85</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="195">
@@ -21674,19 +21674,19 @@
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
         <is>
-          <t>Tocantins</t>
+          <t>Acre</t>
         </is>
       </c>
       <c r="D195" s="6" t="n">
-        <v>368</v>
+        <v>388</v>
       </c>
       <c r="E195" s="12" t="n">
-        <v>1.75</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="196">
@@ -21697,19 +21697,19 @@
       </c>
       <c r="B196" s="4" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Norte</t>
+          <t>Tocantins</t>
         </is>
       </c>
       <c r="D196" s="6" t="n">
-        <v>330</v>
+        <v>368</v>
       </c>
       <c r="E196" s="12" t="n">
-        <v>1.57</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="197">
@@ -21720,19 +21720,19 @@
       </c>
       <c r="B197" s="4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
-          <t>Amapá</t>
+          <t>Rio Grande do Norte</t>
         </is>
       </c>
       <c r="D197" s="6" t="n">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="E197" s="12" t="n">
-        <v>1.53</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="198">
@@ -21743,19 +21743,19 @@
       </c>
       <c r="B198" s="4" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
-          <t>Alagoas</t>
+          <t>Amapá</t>
         </is>
       </c>
       <c r="D198" s="6" t="n">
-        <v>299</v>
+        <v>322</v>
       </c>
       <c r="E198" s="12" t="n">
-        <v>1.42</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="199">
@@ -21766,42 +21766,42 @@
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>Presidenciáveis, circunscrição nacional</t>
+          <t>Alagoas</t>
         </is>
       </c>
       <c r="D199" s="6" t="n">
-        <v>28</v>
+        <v>299</v>
       </c>
       <c r="E199" s="12" t="n">
-        <v>0.13</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>partidos</t>
+          <t>candidatos</t>
         </is>
       </c>
       <c r="B200" s="4" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="C200" s="4" t="inlineStr">
         <is>
-          <t>Minas Gerais</t>
+          <t>Presidenciáveis, circunscrição nacional</t>
         </is>
       </c>
       <c r="D200" s="6" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E200" s="12" t="n">
-        <v>4.2</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="201">
@@ -21812,12 +21812,12 @@
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="C201" s="4" t="inlineStr">
         <is>
-          <t>Maranhão</t>
+          <t>Minas Gerais</t>
         </is>
       </c>
       <c r="D201" s="6" t="n">
@@ -21835,12 +21835,12 @@
       </c>
       <c r="B202" s="4" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C202" s="4" t="inlineStr">
         <is>
-          <t>Distrito Federal</t>
+          <t>Maranhão</t>
         </is>
       </c>
       <c r="D202" s="6" t="n">
@@ -21858,12 +21858,12 @@
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="C203" s="4" t="inlineStr">
         <is>
-          <t>Rio de Janeiro</t>
+          <t>Distrito Federal</t>
         </is>
       </c>
       <c r="D203" s="6" t="n">
@@ -21881,12 +21881,12 @@
       </c>
       <c r="B204" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C204" s="4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Rio de Janeiro</t>
         </is>
       </c>
       <c r="D204" s="6" t="n">
@@ -21904,19 +21904,19 @@
       </c>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C205" s="4" t="inlineStr">
         <is>
-          <t>Pernambuco</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D205" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E205" s="12" t="n">
-        <v>4.05</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="206">
@@ -21927,19 +21927,19 @@
       </c>
       <c r="B206" s="4" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="C206" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Norte</t>
+          <t>Pernambuco</t>
         </is>
       </c>
       <c r="D206" s="6" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E206" s="12" t="n">
-        <v>3.91</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="207">
@@ -21950,12 +21950,12 @@
       </c>
       <c r="B207" s="4" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C207" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Sul</t>
+          <t>Rio Grande do Norte</t>
         </is>
       </c>
       <c r="D207" s="6" t="n">
@@ -21973,12 +21973,12 @@
       </c>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C208" s="4" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Rio Grande do Sul</t>
         </is>
       </c>
       <c r="D208" s="6" t="n">
@@ -21996,19 +21996,19 @@
       </c>
       <c r="B209" s="4" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="C209" s="4" t="inlineStr">
         <is>
-          <t>Goiás</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="D209" s="6" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E209" s="12" t="n">
-        <v>3.76</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="210">
@@ -22019,12 +22019,12 @@
       </c>
       <c r="B210" s="4" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="C210" s="4" t="inlineStr">
         <is>
-          <t>Santa Catarina</t>
+          <t>Goiás</t>
         </is>
       </c>
       <c r="D210" s="6" t="n">
@@ -22042,12 +22042,12 @@
       </c>
       <c r="B211" s="4" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C211" s="4" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Santa Catarina</t>
         </is>
       </c>
       <c r="D211" s="6" t="n">
@@ -22065,12 +22065,12 @@
       </c>
       <c r="B212" s="4" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C212" s="4" t="inlineStr">
         <is>
-          <t>Pará</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="D212" s="6" t="n">
@@ -22088,12 +22088,12 @@
       </c>
       <c r="B213" s="4" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="C213" s="4" t="inlineStr">
         <is>
-          <t>Paraná</t>
+          <t>Pará</t>
         </is>
       </c>
       <c r="D213" s="6" t="n">
@@ -22111,19 +22111,19 @@
       </c>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C214" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso</t>
+          <t>Paraná</t>
         </is>
       </c>
       <c r="D214" s="6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E214" s="12" t="n">
-        <v>3.62</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="215">
@@ -22134,12 +22134,12 @@
       </c>
       <c r="B215" s="4" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="C215" s="4" t="inlineStr">
         <is>
-          <t>Espírito Santo</t>
+          <t>Mato Grosso</t>
         </is>
       </c>
       <c r="D215" s="6" t="n">
@@ -22157,19 +22157,19 @@
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t>Acre</t>
+          <t>Espírito Santo</t>
         </is>
       </c>
       <c r="D216" s="6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E216" s="12" t="n">
-        <v>3.47</v>
+        <v>3.62</v>
       </c>
     </row>
     <row r="217">
@@ -22180,12 +22180,12 @@
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
-          <t>Paraíba</t>
+          <t>Acre</t>
         </is>
       </c>
       <c r="D217" s="6" t="n">
@@ -22203,12 +22203,12 @@
       </c>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
-          <t>Piauí</t>
+          <t>Paraíba</t>
         </is>
       </c>
       <c r="D218" s="6" t="n">
@@ -22226,19 +22226,19 @@
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t>Amazonas</t>
+          <t>Piauí</t>
         </is>
       </c>
       <c r="D219" s="6" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E219" s="12" t="n">
-        <v>3.33</v>
+        <v>3.47</v>
       </c>
     </row>
     <row r="220">
@@ -22249,12 +22249,12 @@
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="C220" s="4" t="inlineStr">
         <is>
-          <t>Roraima</t>
+          <t>Amazonas</t>
         </is>
       </c>
       <c r="D220" s="6" t="n">
@@ -22272,12 +22272,12 @@
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso do Sul</t>
+          <t>Roraima</t>
         </is>
       </c>
       <c r="D221" s="6" t="n">
@@ -22295,19 +22295,19 @@
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C222" s="4" t="inlineStr">
         <is>
-          <t>Sergipe</t>
+          <t>Mato Grosso do Sul</t>
         </is>
       </c>
       <c r="D222" s="6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E222" s="12" t="n">
-        <v>3.18</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="223">
@@ -22318,19 +22318,19 @@
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t>Tocantins</t>
+          <t>Sergipe</t>
         </is>
       </c>
       <c r="D223" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E223" s="12" t="n">
-        <v>3.04</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="224">
@@ -22341,19 +22341,19 @@
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t>Amapá</t>
+          <t>Tocantins</t>
         </is>
       </c>
       <c r="D224" s="6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E224" s="12" t="n">
-        <v>2.89</v>
+        <v>3.04</v>
       </c>
     </row>
     <row r="225">
@@ -22364,12 +22364,12 @@
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C225" s="4" t="inlineStr">
         <is>
-          <t>Rondônia</t>
+          <t>Amapá</t>
         </is>
       </c>
       <c r="D225" s="6" t="n">
@@ -22387,67 +22387,90 @@
       </c>
       <c r="B226" s="4" t="inlineStr">
         <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="C226" s="4" t="inlineStr">
+        <is>
+          <t>Rondônia</t>
+        </is>
+      </c>
+      <c r="D226" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E226" s="12" t="n">
+        <v>2.89</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="4" t="inlineStr">
+        <is>
+          <t>partidos</t>
+        </is>
+      </c>
+      <c r="B227" s="4" t="inlineStr">
+        <is>
           <t>AL</t>
         </is>
       </c>
-      <c r="C226" s="4" t="inlineStr">
+      <c r="C227" s="4" t="inlineStr">
         <is>
           <t>Alagoas</t>
         </is>
       </c>
-      <c r="D226" s="6" t="n">
+      <c r="D227" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="E226" s="12" t="n">
+      <c r="E227" s="12" t="n">
         <v>2.75</v>
       </c>
     </row>
-    <row r="227">
-      <c r="A227" s="7" t="inlineStr">
+    <row r="228">
+      <c r="A228" s="7" t="inlineStr">
         <is>
           <t>partidos</t>
         </is>
       </c>
-      <c r="B227" s="7" t="inlineStr">
+      <c r="B228" s="7" t="inlineStr">
         <is>
           <t>BR</t>
         </is>
       </c>
-      <c r="C227" s="7" t="inlineStr">
+      <c r="C228" s="7" t="inlineStr">
         <is>
           <t>Presidenciáveis, circunscrição nacional</t>
         </is>
       </c>
-      <c r="D227" s="9" t="n">
+      <c r="D228" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="E227" s="13" t="n">
+      <c r="E228" s="13" t="n">
         <v>2.03</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" s="10" t="inlineStr">
-        <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 07:47:46.</t>
-        </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-09-24.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="10" t="inlineStr">
         <is>
-          <t>Nota 1: a serie de fornecedores cobre 68.8% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-09-24.</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="10" t="inlineStr">
+        <is>
+          <t>Nota 1: a serie de fornecedores cobre 68.9% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="10" t="inlineStr">
         <is>
           <t>Nota 2: a serie por UF do doador cobre apenas 8.9% do valor doado, porque o TSE nao publica a UF do doador pessoa fisica. Para leitura integral use a serie por UF do candidato que recebeu.</t>
         </is>
@@ -22555,22 +22578,22 @@
         <v>18485111.6</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>4556010.95</v>
+        <v>5013285.95</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>7330302.17</v>
+        <v>7506630.92</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>25815413.77</v>
+        <v>25991742.52</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>18.84</v>
+        <v>18.9</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>425203448.53</v>
+        <v>425660723.53</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>22.41</v>
+        <v>22.4</v>
       </c>
     </row>
     <row r="6">
@@ -22586,22 +22609,22 @@
         <v>18767611.87</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>15420541.37</v>
+        <v>15423331.37</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>4710150.94</v>
+        <v>4970836.14</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>23477762.81</v>
+        <v>23738448.01</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>17.14</v>
+        <v>17.26</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>318668598.53</v>
+        <v>318671388.53</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>16.8</v>
+        <v>16.77</v>
       </c>
     </row>
     <row r="7">
@@ -22617,22 +22640,22 @@
         <v>2024422.59</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>4405616.89</v>
+        <v>4755616.89</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>13634436.95</v>
+        <v>13373751.75</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>15658859.54</v>
+        <v>15398174.34</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>11.43</v>
+        <v>11.19</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>127902245.35</v>
+        <v>128252245.35</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.74</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="8">
@@ -22657,13 +22680,13 @@
         <v>15087102.75</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>11.01</v>
+        <v>10.97</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>172914762.35</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>9.109999999999999</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="9">
@@ -22679,22 +22702,22 @@
         <v>6213996.63</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>10048725.59</v>
+        <v>10352176.89</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>7246108.82</v>
+        <v>7469958.82</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>13460105.45</v>
+        <v>13683955.45</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>9.82</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>104807058</v>
+        <v>105110509.3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.52</v>
+        <v>5.53</v>
       </c>
     </row>
     <row r="10">
@@ -22710,22 +22733,22 @@
         <v>6181808.82</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>848977</v>
+        <v>941897</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>135747.66</v>
+        <v>169747.66</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>6317556.48</v>
+        <v>6351556.48</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>4.61</v>
+        <v>4.62</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>142036297.98</v>
+        <v>142129217.98</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>7.49</v>
+        <v>7.48</v>
       </c>
     </row>
     <row r="11">
@@ -22744,19 +22767,19 @@
         <v>2145619.45</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>2068680.85</v>
+        <v>2015572.35</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>6306180.640000001</v>
+        <v>6253072.140000001</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>4.6</v>
+        <v>4.55</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>127727630.51</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>6.73</v>
+        <v>6.72</v>
       </c>
     </row>
     <row r="12">
@@ -22772,22 +22795,22 @@
         <v>2370564.76</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>8707553.99</v>
+        <v>10803413.04</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>3518340.69</v>
+        <v>3568340.77</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>5888905.449999999</v>
+        <v>5938905.529999999</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>4.3</v>
+        <v>4.32</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>61626161.59</v>
+        <v>63722020.64</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>3.25</v>
+        <v>3.35</v>
       </c>
     </row>
     <row r="13">
@@ -22812,13 +22835,13 @@
         <v>5628437.98</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>4.11</v>
+        <v>4.09</v>
       </c>
       <c r="H13" s="6" t="n">
         <v>134762194.74</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>7.1</v>
+        <v>7.09</v>
       </c>
     </row>
     <row r="14">
@@ -22843,7 +22866,7 @@
         <v>3019071.63</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>2.2</v>
+        <v>2.19</v>
       </c>
       <c r="H14" s="6" t="n">
         <v>61699039.53</v>
@@ -22868,10 +22891,10 @@
         <v>752452.6</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1153315.55</v>
+        <v>1154315.55</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>2910177.28</v>
+        <v>2911177.28</v>
       </c>
       <c r="G15" s="6" t="n">
         <v>2.12</v>
@@ -22905,7 +22928,7 @@
         <v>2760868.21</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>2.02</v>
+        <v>2.01</v>
       </c>
       <c r="H16" s="6" t="n">
         <v>32675488.27</v>
@@ -22936,7 +22959,7 @@
         <v>2508732.31</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>1.83</v>
+        <v>1.82</v>
       </c>
       <c r="H17" s="6" t="n">
         <v>19049050.9</v>
@@ -22961,19 +22984,19 @@
         <v>766982</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1299563</v>
+        <v>1400921</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>1505663</v>
+        <v>1607021</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>1.1</v>
+        <v>1.17</v>
       </c>
       <c r="H18" s="6" t="n">
         <v>10924162.75</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="19">
@@ -23004,7 +23027,7 @@
         <v>15867628.34</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="20">
@@ -23302,7 +23325,7 @@
         <v>8076.8</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>48965.99</v>
+        <v>48965.99000000001</v>
       </c>
       <c r="F29" s="6" t="n">
         <v>209391.57</v>
@@ -23423,7 +23446,7 @@
         <v>923.7</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>51744.89</v>
+        <v>51744.89000000001</v>
       </c>
       <c r="E33" s="6" t="n">
         <v>40426.19</v>
@@ -23537,63 +23560,63 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Encargos financeiros, taxas bancárias e/ou op. cartão de crédito</t>
+          <t>Energia elétrica</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>258182.07</v>
+        <v>17696.69</v>
       </c>
       <c r="C37" s="6" t="n">
-        <v>11474.01</v>
+        <v>0</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>89167.28999999999</v>
+        <v>0</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>7451.54</v>
+        <v>23429.19</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>18925.55</v>
+        <v>23429.19</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>347349.36</v>
+        <v>17696.69</v>
       </c>
       <c r="I37" s="6" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Energia elétrica</t>
+          <t>Encargos financeiros, taxas bancárias e/ou op. cartão de crédito</t>
         </is>
       </c>
       <c r="B38" s="6" t="n">
-        <v>17696.69</v>
+        <v>258182.07</v>
       </c>
       <c r="C38" s="6" t="n">
-        <v>0</v>
+        <v>11474.01</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>0</v>
+        <v>89478.69</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>17836.93</v>
+        <v>7470.34</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>17836.93</v>
+        <v>18944.35</v>
       </c>
       <c r="G38" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>17696.69</v>
+        <v>347660.76</v>
       </c>
       <c r="I38" s="6" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="39">
@@ -23754,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 07:47:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
         </is>
       </c>
     </row>
@@ -25281,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 07:47:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
         </is>
       </c>
     </row>
@@ -28184,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 07:47:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 24/09/2026 15:56
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>36299</v>
+        <v>38299</v>
       </c>
     </row>
     <row r="48">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>11382</v>
+        <v>9388</v>
       </c>
     </row>
     <row r="50">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-24 09:19:07</t>
+          <t>2026-09-24 15:20:22</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
         </is>
       </c>
     </row>
@@ -19245,10 +19245,10 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>610399910.0599999</v>
+        <v>610635408.6</v>
       </c>
       <c r="E89" s="12" t="n">
-        <v>23.63</v>
+        <v>23.62</v>
       </c>
     </row>
     <row r="90">
@@ -19268,7 +19268,7 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>167437678.87</v>
+        <v>167492273.67</v>
       </c>
       <c r="E90" s="12" t="n">
         <v>6.48</v>
@@ -19291,7 +19291,7 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>160315545.81</v>
+        <v>160531043.51</v>
       </c>
       <c r="E91" s="12" t="n">
         <v>6.21</v>
@@ -19314,7 +19314,7 @@
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>128343924.02</v>
+        <v>128378900.29</v>
       </c>
       <c r="E92" s="12" t="n">
         <v>4.97</v>
@@ -19337,7 +19337,7 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>121512202.79</v>
+        <v>121583362.46</v>
       </c>
       <c r="E93" s="12" t="n">
         <v>4.7</v>
@@ -19360,10 +19360,10 @@
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>107062353.14</v>
+        <v>107218219.4</v>
       </c>
       <c r="E94" s="12" t="n">
-        <v>4.14</v>
+        <v>4.15</v>
       </c>
     </row>
     <row r="95">
@@ -19383,7 +19383,7 @@
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>103040938.56</v>
+        <v>103186668.67</v>
       </c>
       <c r="E95" s="12" t="n">
         <v>3.99</v>
@@ -19406,7 +19406,7 @@
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>98581276.86</v>
+        <v>98631902.77</v>
       </c>
       <c r="E96" s="12" t="n">
         <v>3.82</v>
@@ -19429,7 +19429,7 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>92451872.34999999</v>
+        <v>92465423.15000001</v>
       </c>
       <c r="E97" s="12" t="n">
         <v>3.58</v>
@@ -19452,7 +19452,7 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>88629734.43000001</v>
+        <v>88672478.52</v>
       </c>
       <c r="E98" s="12" t="n">
         <v>3.43</v>
@@ -19475,7 +19475,7 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>84157310.75</v>
+        <v>84187598.81999999</v>
       </c>
       <c r="E99" s="12" t="n">
         <v>3.26</v>
@@ -19498,7 +19498,7 @@
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>80328521.43000001</v>
+        <v>80408738.55</v>
       </c>
       <c r="E100" s="12" t="n">
         <v>3.11</v>
@@ -19521,7 +19521,7 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>73117225.06</v>
+        <v>73142071.83</v>
       </c>
       <c r="E101" s="12" t="n">
         <v>2.83</v>
@@ -19544,7 +19544,7 @@
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>69544574.78</v>
+        <v>69583027.84999999</v>
       </c>
       <c r="E102" s="12" t="n">
         <v>2.69</v>
@@ -19567,7 +19567,7 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>67724974.7</v>
+        <v>67794648.15000001</v>
       </c>
       <c r="E103" s="12" t="n">
         <v>2.62</v>
@@ -19590,7 +19590,7 @@
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>63445152.62</v>
+        <v>63475860.89</v>
       </c>
       <c r="E104" s="12" t="n">
         <v>2.46</v>
@@ -19613,7 +19613,7 @@
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>57006831.18</v>
+        <v>57079358.25</v>
       </c>
       <c r="E105" s="12" t="n">
         <v>2.21</v>
@@ -19636,7 +19636,7 @@
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>55631376.34</v>
+        <v>55645363.38</v>
       </c>
       <c r="E106" s="12" t="n">
         <v>2.15</v>
@@ -19659,7 +19659,7 @@
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>47201182.01</v>
+        <v>47234880.15</v>
       </c>
       <c r="E107" s="12" t="n">
         <v>1.83</v>
@@ -19682,7 +19682,7 @@
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>44938130.46</v>
+        <v>44943052.59</v>
       </c>
       <c r="E108" s="12" t="n">
         <v>1.74</v>
@@ -19705,7 +19705,7 @@
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>44887831.16</v>
+        <v>44931106.03</v>
       </c>
       <c r="E109" s="12" t="n">
         <v>1.74</v>
@@ -19728,7 +19728,7 @@
         </is>
       </c>
       <c r="D110" s="6" t="n">
-        <v>43976203.98</v>
+        <v>43995454.21</v>
       </c>
       <c r="E110" s="12" t="n">
         <v>1.7</v>
@@ -19751,7 +19751,7 @@
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>42273490.41</v>
+        <v>42294991.35</v>
       </c>
       <c r="E111" s="12" t="n">
         <v>1.64</v>
@@ -19774,7 +19774,7 @@
         </is>
       </c>
       <c r="D112" s="6" t="n">
-        <v>41517892.79</v>
+        <v>41534065.8</v>
       </c>
       <c r="E112" s="12" t="n">
         <v>1.61</v>
@@ -19797,7 +19797,7 @@
         </is>
       </c>
       <c r="D113" s="6" t="n">
-        <v>35611767.07</v>
+        <v>35617710.8</v>
       </c>
       <c r="E113" s="12" t="n">
         <v>1.38</v>
@@ -19820,7 +19820,7 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>27567405.68</v>
+        <v>27600150.33</v>
       </c>
       <c r="E114" s="12" t="n">
         <v>1.07</v>
@@ -19843,7 +19843,7 @@
         </is>
       </c>
       <c r="D115" s="6" t="n">
-        <v>25341311.92</v>
+        <v>25346575.28</v>
       </c>
       <c r="E115" s="12" t="n">
         <v>0.98</v>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
         </is>
       </c>
     </row>
@@ -23823,7 +23823,7 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 09:19:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 25/09/2026 09:50
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -671,7 +671,7 @@
         <v>53.81</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>12355237266.73</v>
+        <v>12355307266.73</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>38.14</v>
@@ -702,7 +702,7 @@
         <v>37.18</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>8706826684.209999</v>
+        <v>8707006684.209999</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>26.88</v>
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32395103412.82</v>
+        <v>32395353412.82</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>77251</v>
+        <v>77254</v>
       </c>
     </row>
     <row r="31">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>32395103412.82</v>
+        <v>32395353412.82</v>
       </c>
     </row>
     <row r="34">
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>38299</v>
+        <v>41299</v>
       </c>
     </row>
     <row r="48">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>9388</v>
+        <v>6394</v>
       </c>
     </row>
     <row r="50">
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>4772139234.33</v>
+        <v>4773054933.99</v>
       </c>
     </row>
     <row r="57">
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>4718525185.58</v>
+        <v>4718944665.58</v>
       </c>
     </row>
     <row r="58">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>479003500.02</v>
+        <v>481594978.42</v>
       </c>
     </row>
     <row r="59">
@@ -1514,7 +1514,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>433269095.24</v>
+        <v>435070177.29</v>
       </c>
     </row>
     <row r="60">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-24 15:20:22</t>
+          <t>2026-09-25 09:17:40</t>
         </is>
       </c>
     </row>
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="G63" s="6" t="n">
-        <v>58445503.79</v>
+        <v>58445503.79000001</v>
       </c>
       <c r="H63" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
         </is>
       </c>
     </row>
@@ -19245,7 +19245,7 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>610635408.6</v>
+        <v>610846190.9299999</v>
       </c>
       <c r="E89" s="12" t="n">
         <v>23.62</v>
@@ -19268,7 +19268,7 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>167492273.67</v>
+        <v>167536445.27</v>
       </c>
       <c r="E90" s="12" t="n">
         <v>6.48</v>
@@ -19291,10 +19291,10 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>160531043.51</v>
+        <v>160744853.84</v>
       </c>
       <c r="E91" s="12" t="n">
-        <v>6.21</v>
+        <v>6.22</v>
       </c>
     </row>
     <row r="92">
@@ -19314,7 +19314,7 @@
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>128378900.29</v>
+        <v>128421003.07</v>
       </c>
       <c r="E92" s="12" t="n">
         <v>4.97</v>
@@ -19337,7 +19337,7 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>121583362.46</v>
+        <v>121665049.83</v>
       </c>
       <c r="E93" s="12" t="n">
         <v>4.7</v>
@@ -19360,7 +19360,7 @@
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>107218219.4</v>
+        <v>107359698.44</v>
       </c>
       <c r="E94" s="12" t="n">
         <v>4.15</v>
@@ -19383,7 +19383,7 @@
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>103186668.67</v>
+        <v>103302328.44</v>
       </c>
       <c r="E95" s="12" t="n">
         <v>3.99</v>
@@ -19406,7 +19406,7 @@
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>98631902.77</v>
+        <v>98668430.09999999</v>
       </c>
       <c r="E96" s="12" t="n">
         <v>3.82</v>
@@ -19429,7 +19429,7 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>92465423.15000001</v>
+        <v>92487807.61</v>
       </c>
       <c r="E97" s="12" t="n">
         <v>3.58</v>
@@ -19452,7 +19452,7 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>88672478.52</v>
+        <v>88715475.05</v>
       </c>
       <c r="E98" s="12" t="n">
         <v>3.43</v>
@@ -19475,7 +19475,7 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>84187598.81999999</v>
+        <v>84219299.45</v>
       </c>
       <c r="E99" s="12" t="n">
         <v>3.26</v>
@@ -19498,7 +19498,7 @@
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>80408738.55</v>
+        <v>80477201.81999999</v>
       </c>
       <c r="E100" s="12" t="n">
         <v>3.11</v>
@@ -19521,7 +19521,7 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>73142071.83</v>
+        <v>73168666.61</v>
       </c>
       <c r="E101" s="12" t="n">
         <v>2.83</v>
@@ -19544,7 +19544,7 @@
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>69583027.84999999</v>
+        <v>69607927.37</v>
       </c>
       <c r="E102" s="12" t="n">
         <v>2.69</v>
@@ -19567,7 +19567,7 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>67794648.15000001</v>
+        <v>67862763.75</v>
       </c>
       <c r="E103" s="12" t="n">
         <v>2.62</v>
@@ -19590,7 +19590,7 @@
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>63475860.89</v>
+        <v>63501156.98</v>
       </c>
       <c r="E104" s="12" t="n">
         <v>2.46</v>
@@ -19613,7 +19613,7 @@
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>57079358.25</v>
+        <v>57145340.82</v>
       </c>
       <c r="E105" s="12" t="n">
         <v>2.21</v>
@@ -19636,7 +19636,7 @@
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>55645363.38</v>
+        <v>55666882.79</v>
       </c>
       <c r="E106" s="12" t="n">
         <v>2.15</v>
@@ -19659,7 +19659,7 @@
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>47234880.15</v>
+        <v>47271306.16</v>
       </c>
       <c r="E107" s="12" t="n">
         <v>1.83</v>
@@ -19673,16 +19673,16 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Amapá</t>
+          <t>Rondônia</t>
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>44943052.59</v>
+        <v>44961266.69</v>
       </c>
       <c r="E108" s="12" t="n">
         <v>1.74</v>
@@ -19696,16 +19696,16 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Rondônia</t>
+          <t>Amapá</t>
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>44931106.03</v>
+        <v>44949128.99</v>
       </c>
       <c r="E109" s="12" t="n">
         <v>1.74</v>
@@ -19728,7 +19728,7 @@
         </is>
       </c>
       <c r="D110" s="6" t="n">
-        <v>43995454.21</v>
+        <v>44012231.34</v>
       </c>
       <c r="E110" s="12" t="n">
         <v>1.7</v>
@@ -19751,7 +19751,7 @@
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>42294991.35</v>
+        <v>42316501.36</v>
       </c>
       <c r="E111" s="12" t="n">
         <v>1.64</v>
@@ -19774,7 +19774,7 @@
         </is>
       </c>
       <c r="D112" s="6" t="n">
-        <v>41534065.8</v>
+        <v>41549782.74</v>
       </c>
       <c r="E112" s="12" t="n">
         <v>1.61</v>
@@ -19797,7 +19797,7 @@
         </is>
       </c>
       <c r="D113" s="6" t="n">
-        <v>35617710.8</v>
+        <v>35621478.43</v>
       </c>
       <c r="E113" s="12" t="n">
         <v>1.38</v>
@@ -19820,7 +19820,7 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>27600150.33</v>
+        <v>27627477.94</v>
       </c>
       <c r="E114" s="12" t="n">
         <v>1.07</v>
@@ -19843,7 +19843,7 @@
         </is>
       </c>
       <c r="D115" s="6" t="n">
-        <v>25346575.28</v>
+        <v>25350876.29</v>
       </c>
       <c r="E115" s="12" t="n">
         <v>0.98</v>
@@ -19889,7 +19889,7 @@
         </is>
       </c>
       <c r="D117" s="6" t="n">
-        <v>1010.55</v>
+        <v>1510.55</v>
       </c>
       <c r="E117" s="12" t="n">
         <v>0</v>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
         </is>
       </c>
     </row>
@@ -22465,7 +22465,7 @@
     <row r="231">
       <c r="A231" s="10" t="inlineStr">
         <is>
-          <t>Nota 1: a serie de fornecedores cobre 68.9% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
+          <t>Nota 1: a serie de fornecedores cobre 69.0% do valor contratado, que e' a parcela com UF conhecida na data desta extracao, e cresce a cada consulta de CNPJ.</t>
         </is>
       </c>
     </row>
@@ -22578,22 +22578,22 @@
         <v>18485111.6</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>5013285.95</v>
+        <v>5043776.95</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>7506630.92</v>
+        <v>7671920.92</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>25991742.52</v>
+        <v>26157032.52</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>18.9</v>
+        <v>18.91</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>425660723.53</v>
+        <v>425691214.53</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>22.4</v>
+        <v>22.39</v>
       </c>
     </row>
     <row r="6">
@@ -22609,7 +22609,7 @@
         <v>18767611.87</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>15423331.37</v>
+        <v>15440831.37</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>4970836.14</v>
@@ -22618,13 +22618,13 @@
         <v>23738448.01</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>17.26</v>
+        <v>17.16</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>318671388.53</v>
+        <v>318688888.53</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>16.77</v>
+        <v>16.76</v>
       </c>
     </row>
     <row r="7">
@@ -22640,19 +22640,19 @@
         <v>2024422.59</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>4755616.89</v>
+        <v>4773716.89</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>13373751.75</v>
+        <v>13491962.55</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>15398174.34</v>
+        <v>15516385.14</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>11.19</v>
+        <v>11.22</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>128252245.35</v>
+        <v>128270345.35</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>6.75</v>
@@ -22671,7 +22671,7 @@
         <v>14924272.42</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>317350</v>
+        <v>317650</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>162830.33</v>
@@ -22680,10 +22680,10 @@
         <v>15087102.75</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>10.97</v>
+        <v>10.91</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>172914762.35</v>
+        <v>172915062.35</v>
       </c>
       <c r="I8" s="6" t="n">
         <v>9.1</v>
@@ -22711,7 +22711,7 @@
         <v>13683955.45</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>9.949999999999999</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>105110509.3</v>
@@ -22733,22 +22733,22 @@
         <v>6181808.82</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>941897</v>
+        <v>1276644</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>169747.66</v>
+        <v>382542.16</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>6351556.48</v>
+        <v>6564350.98</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>4.62</v>
+        <v>4.75</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>142129217.98</v>
+        <v>142463964.98</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>7.48</v>
+        <v>7.49</v>
       </c>
     </row>
     <row r="11">
@@ -22767,13 +22767,13 @@
         <v>2145619.45</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>2015572.35</v>
+        <v>2025570.6</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>6253072.140000001</v>
+        <v>6263070.390000001</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>4.55</v>
+        <v>4.53</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>127727630.51</v>
@@ -22795,7 +22795,7 @@
         <v>2370564.76</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>10803413.04</v>
+        <v>10853996.9</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>3568340.77</v>
@@ -22804,10 +22804,10 @@
         <v>5938905.529999999</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>4.32</v>
+        <v>4.29</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>63722020.64</v>
+        <v>63772604.5</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>3.35</v>
@@ -22829,13 +22829,13 @@
         <v>542259.41</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>123368</v>
+        <v>202368</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>5628437.98</v>
+        <v>5707437.98</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>4.09</v>
+        <v>4.13</v>
       </c>
       <c r="H13" s="6" t="n">
         <v>134762194.74</v>
@@ -22847,63 +22847,63 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Cessão ou locação de veículos</t>
+          <t>Diversas a especificar</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>61648999.53</v>
+        <v>45621032.07</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>2114826.85</v>
+        <v>1756861.73</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>50040</v>
+        <v>752452.6</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>904244.78</v>
+        <v>1358698.35</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>3019071.63</v>
+        <v>3115560.08</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>2.19</v>
+        <v>2.25</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>61699039.53</v>
+        <v>46373484.67</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>3.25</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Diversas a especificar</t>
+          <t>Cessão ou locação de veículos</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>45621032.07</v>
+        <v>61648999.53</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>1756861.73</v>
+        <v>2114826.85</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>752452.6</v>
+        <v>50040</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1154315.55</v>
+        <v>904244.78</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>2911177.28</v>
+        <v>3019071.63</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>2.12</v>
+        <v>2.18</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>46373484.67</v>
+        <v>61699039.53</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.44</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="16">
@@ -22928,7 +22928,7 @@
         <v>2760868.21</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>2.01</v>
+        <v>2</v>
       </c>
       <c r="H16" s="6" t="n">
         <v>32675488.27</v>
@@ -22950,19 +22950,19 @@
         <v>1297889.49</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>284297.42</v>
+        <v>326185.19</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1210842.82</v>
+        <v>1211542.82</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>2508732.31</v>
+        <v>2509432.31</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>1.82</v>
+        <v>1.81</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>19049050.9</v>
+        <v>19090938.67</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>1</v>
@@ -22990,7 +22990,7 @@
         <v>1607021</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="H18" s="6" t="n">
         <v>10924162.75</v>
@@ -23021,7 +23021,7 @@
         <v>1177839.04</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="H19" s="6" t="n">
         <v>15867628.34</v>
@@ -23052,7 +23052,7 @@
         <v>1013264.29</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="H20" s="6" t="n">
         <v>18566885.41</v>
@@ -23083,7 +23083,7 @@
         <v>725663.76</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="H21" s="6" t="n">
         <v>9455125.310000001</v>
@@ -23145,7 +23145,7 @@
         <v>683734.35</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="H23" s="6" t="n">
         <v>11938959.46</v>
@@ -23173,7 +23173,7 @@
         <v>151786.7</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>538409.7899999999</v>
+        <v>538409.79</v>
       </c>
       <c r="G24" s="6" t="n">
         <v>0.39</v>
@@ -23198,7 +23198,7 @@
         <v>313333.95</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>931000</v>
+        <v>933500</v>
       </c>
       <c r="E25" s="6" t="n">
         <v>0</v>
@@ -23210,7 +23210,7 @@
         <v>0.23</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>9978290.66</v>
+        <v>9980790.66</v>
       </c>
       <c r="I25" s="6" t="n">
         <v>0.53</v>
@@ -23325,7 +23325,7 @@
         <v>8076.8</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>48965.99000000001</v>
+        <v>48965.99</v>
       </c>
       <c r="F29" s="6" t="n">
         <v>209391.57</v>
@@ -23446,7 +23446,7 @@
         <v>923.7</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>51744.89000000001</v>
+        <v>51744.89</v>
       </c>
       <c r="E33" s="6" t="n">
         <v>40426.19</v>
@@ -23601,19 +23601,19 @@
         <v>11474.01</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>89478.69</v>
+        <v>89588.72</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>7470.34</v>
+        <v>7490.34</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>18944.35</v>
+        <v>18964.35</v>
       </c>
       <c r="G38" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>347660.76</v>
+        <v>347770.79</v>
       </c>
       <c r="I38" s="6" t="n">
         <v>0.02</v>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
         </is>
       </c>
     </row>
@@ -23823,7 +23823,7 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -23934,7 +23934,7 @@
         <v>7.85</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>4898570244.67</v>
+        <v>4898750244.67</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>1049723932.87</v>
@@ -24026,7 +24026,7 @@
         <v>4.03</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>1817691708.82</v>
+        <v>1817696708.82</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>585224449.03</v>
@@ -24164,7 +24164,7 @@
         <v>3.43</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1294302106.67</v>
+        <v>1294367106.67</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>491285958.95</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-24 15:20:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 25/09/2026 16:25
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 15:22:28.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 15:22:28.</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>41299</v>
+        <v>44299</v>
       </c>
     </row>
     <row r="48">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>6394</v>
+        <v>3398</v>
       </c>
     </row>
     <row r="50">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-25 09:17:40</t>
+          <t>2026-09-25 15:22:28</t>
         </is>
       </c>
     </row>
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="G63" s="6" t="n">
-        <v>58445503.79000001</v>
+        <v>58445503.79</v>
       </c>
       <c r="H63" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 15:22:28.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 15:22:28.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 15:22:28.</t>
         </is>
       </c>
     </row>
@@ -19245,7 +19245,7 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>610846190.9299999</v>
+        <v>610954988.74</v>
       </c>
       <c r="E89" s="12" t="n">
         <v>23.62</v>
@@ -19268,7 +19268,7 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>167536445.27</v>
+        <v>167563007.99</v>
       </c>
       <c r="E90" s="12" t="n">
         <v>6.48</v>
@@ -19291,7 +19291,7 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>160744853.84</v>
+        <v>160891101.2</v>
       </c>
       <c r="E91" s="12" t="n">
         <v>6.22</v>
@@ -19314,10 +19314,10 @@
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>128421003.07</v>
+        <v>128441851.4</v>
       </c>
       <c r="E92" s="12" t="n">
-        <v>4.97</v>
+        <v>4.96</v>
       </c>
     </row>
     <row r="93">
@@ -19337,7 +19337,7 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>121665049.83</v>
+        <v>121706586.89</v>
       </c>
       <c r="E93" s="12" t="n">
         <v>4.7</v>
@@ -19360,7 +19360,7 @@
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>107359698.44</v>
+        <v>107451059.43</v>
       </c>
       <c r="E94" s="12" t="n">
         <v>4.15</v>
@@ -19383,10 +19383,10 @@
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>103302328.44</v>
+        <v>103375597.68</v>
       </c>
       <c r="E95" s="12" t="n">
-        <v>3.99</v>
+        <v>4</v>
       </c>
     </row>
     <row r="96">
@@ -19406,10 +19406,10 @@
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>98668430.09999999</v>
+        <v>98688693.78</v>
       </c>
       <c r="E96" s="12" t="n">
-        <v>3.82</v>
+        <v>3.81</v>
       </c>
     </row>
     <row r="97">
@@ -19429,7 +19429,7 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>92487807.61</v>
+        <v>92496839.87</v>
       </c>
       <c r="E97" s="12" t="n">
         <v>3.58</v>
@@ -19452,7 +19452,7 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>88715475.05</v>
+        <v>88730845.01000001</v>
       </c>
       <c r="E98" s="12" t="n">
         <v>3.43</v>
@@ -19475,7 +19475,7 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>84219299.45</v>
+        <v>84233880.98999999</v>
       </c>
       <c r="E99" s="12" t="n">
         <v>3.26</v>
@@ -19498,7 +19498,7 @@
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>80477201.81999999</v>
+        <v>80516471.73</v>
       </c>
       <c r="E100" s="12" t="n">
         <v>3.11</v>
@@ -19521,7 +19521,7 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>73168666.61</v>
+        <v>73184842.70999999</v>
       </c>
       <c r="E101" s="12" t="n">
         <v>2.83</v>
@@ -19544,7 +19544,7 @@
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>69607927.37</v>
+        <v>69616117.09999999</v>
       </c>
       <c r="E102" s="12" t="n">
         <v>2.69</v>
@@ -19567,7 +19567,7 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>67862763.75</v>
+        <v>67900019.25</v>
       </c>
       <c r="E103" s="12" t="n">
         <v>2.62</v>
@@ -19590,7 +19590,7 @@
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>63501156.98</v>
+        <v>63516081.46</v>
       </c>
       <c r="E104" s="12" t="n">
         <v>2.46</v>
@@ -19613,7 +19613,7 @@
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>57145340.82</v>
+        <v>57174482.15</v>
       </c>
       <c r="E105" s="12" t="n">
         <v>2.21</v>
@@ -19636,7 +19636,7 @@
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>55666882.79</v>
+        <v>55675092.03</v>
       </c>
       <c r="E106" s="12" t="n">
         <v>2.15</v>
@@ -19659,7 +19659,7 @@
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>47271306.16</v>
+        <v>47295265.79</v>
       </c>
       <c r="E107" s="12" t="n">
         <v>1.83</v>
@@ -19682,7 +19682,7 @@
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>44961266.69</v>
+        <v>44973680.18</v>
       </c>
       <c r="E108" s="12" t="n">
         <v>1.74</v>
@@ -19705,7 +19705,7 @@
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>44949128.99</v>
+        <v>44954101.79</v>
       </c>
       <c r="E109" s="12" t="n">
         <v>1.74</v>
@@ -19728,7 +19728,7 @@
         </is>
       </c>
       <c r="D110" s="6" t="n">
-        <v>44012231.34</v>
+        <v>44021491.03</v>
       </c>
       <c r="E110" s="12" t="n">
         <v>1.7</v>
@@ -19751,7 +19751,7 @@
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>42316501.36</v>
+        <v>42324034.78</v>
       </c>
       <c r="E111" s="12" t="n">
         <v>1.64</v>
@@ -19774,7 +19774,7 @@
         </is>
       </c>
       <c r="D112" s="6" t="n">
-        <v>41549782.74</v>
+        <v>41557645.04</v>
       </c>
       <c r="E112" s="12" t="n">
         <v>1.61</v>
@@ -19797,7 +19797,7 @@
         </is>
       </c>
       <c r="D113" s="6" t="n">
-        <v>35621478.43</v>
+        <v>35622700.33</v>
       </c>
       <c r="E113" s="12" t="n">
         <v>1.38</v>
@@ -19820,7 +19820,7 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>27627477.94</v>
+        <v>27646250.52</v>
       </c>
       <c r="E114" s="12" t="n">
         <v>1.07</v>
@@ -19843,7 +19843,7 @@
         </is>
       </c>
       <c r="D115" s="6" t="n">
-        <v>25350876.29</v>
+        <v>25353499.59</v>
       </c>
       <c r="E115" s="12" t="n">
         <v>0.98</v>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 15:22:28.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 15:22:28.</t>
         </is>
       </c>
     </row>
@@ -23823,7 +23823,7 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 15:22:28.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 09:17:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-25 15:22:28.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 27/09/2026 09:10
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -702,7 +702,7 @@
         <v>37.18</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>8707690841.16</v>
+        <v>8708281692.280001</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>26.88</v>
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32396037569.77</v>
+        <v>32396628420.89</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-26 09:17:45.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 09:01:54.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-26 09:17:45.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 09:01:54.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>77264</v>
+        <v>77272</v>
       </c>
     </row>
     <row r="31">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>32396037569.77</v>
+        <v>32396628420.89</v>
       </c>
     </row>
     <row r="34">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>47298</v>
+        <v>48146</v>
       </c>
     </row>
     <row r="48">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>870</v>
+        <v>22</v>
       </c>
     </row>
     <row r="50">
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>4773054933.99</v>
+        <v>4808511355.97</v>
       </c>
     </row>
     <row r="57">
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>4718944665.58</v>
+        <v>4754567725.27</v>
       </c>
     </row>
     <row r="58">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>481594978.42</v>
+        <v>501869180.65</v>
       </c>
     </row>
     <row r="59">
@@ -1514,7 +1514,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>435070177.29</v>
+        <v>454145362.3</v>
       </c>
     </row>
     <row r="60">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-26 09:17:45</t>
+          <t>2026-09-27 09:01:54</t>
         </is>
       </c>
     </row>
@@ -4822,7 +4822,7 @@
         </is>
       </c>
       <c r="G48" s="6" t="n">
-        <v>75658784.07000001</v>
+        <v>75658784.06999999</v>
       </c>
       <c r="H48" s="6" t="n">
         <v>0.23</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-26 09:17:45.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 09:01:54.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-26 09:17:45.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 09:01:54.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-26 09:17:45.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 09:01:54.</t>
         </is>
       </c>
     </row>
@@ -19245,7 +19245,7 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>624278126.8099999</v>
+        <v>624283690.54</v>
       </c>
       <c r="E89" s="12" t="n">
         <v>23.85</v>
@@ -19268,7 +19268,7 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>169521130.46</v>
+        <v>169522158.94</v>
       </c>
       <c r="E90" s="12" t="n">
         <v>6.48</v>
@@ -19291,7 +19291,7 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>161929039.94</v>
+        <v>161936482.22</v>
       </c>
       <c r="E91" s="12" t="n">
         <v>6.19</v>
@@ -19314,7 +19314,7 @@
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>129041550.02</v>
+        <v>129043454.95</v>
       </c>
       <c r="E92" s="12" t="n">
         <v>4.93</v>
@@ -19337,7 +19337,7 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>122192554.86</v>
+        <v>122195675.28</v>
       </c>
       <c r="E93" s="12" t="n">
         <v>4.67</v>
@@ -19360,7 +19360,7 @@
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>108453001.54</v>
+        <v>108456139.85</v>
       </c>
       <c r="E94" s="12" t="n">
         <v>4.14</v>
@@ -19383,7 +19383,7 @@
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>104612520.3</v>
+        <v>104615766.46</v>
       </c>
       <c r="E95" s="12" t="n">
         <v>4</v>
@@ -19406,7 +19406,7 @@
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>100927707.42</v>
+        <v>100928292.37</v>
       </c>
       <c r="E96" s="12" t="n">
         <v>3.86</v>
@@ -19429,7 +19429,7 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>92630495.37</v>
+        <v>92630748.37</v>
       </c>
       <c r="E97" s="12" t="n">
         <v>3.54</v>
@@ -19452,7 +19452,7 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>90204087.08</v>
+        <v>90204957.91</v>
       </c>
       <c r="E98" s="12" t="n">
         <v>3.45</v>
@@ -19475,7 +19475,7 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>84326194.87</v>
+        <v>84326369.94</v>
       </c>
       <c r="E99" s="12" t="n">
         <v>3.22</v>
@@ -19498,7 +19498,7 @@
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>81777912.06</v>
+        <v>81779449.09999999</v>
       </c>
       <c r="E100" s="12" t="n">
         <v>3.12</v>
@@ -19521,7 +19521,7 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>73446137.18000001</v>
+        <v>73446754.23999999</v>
       </c>
       <c r="E101" s="12" t="n">
         <v>2.81</v>
@@ -19544,7 +19544,7 @@
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>69735726.16</v>
+        <v>69736088.06999999</v>
       </c>
       <c r="E102" s="12" t="n">
         <v>2.66</v>
@@ -19567,7 +19567,7 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>68894949.47</v>
+        <v>68896580.34999999</v>
       </c>
       <c r="E103" s="12" t="n">
         <v>2.63</v>
@@ -19590,7 +19590,7 @@
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>63952697.66</v>
+        <v>63953073.2</v>
       </c>
       <c r="E104" s="12" t="n">
         <v>2.44</v>
@@ -19613,7 +19613,7 @@
         </is>
       </c>
       <c r="D105" s="6" t="n">
-        <v>58193961.23</v>
+        <v>58194508.79</v>
       </c>
       <c r="E105" s="12" t="n">
         <v>2.22</v>
@@ -19636,7 +19636,7 @@
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>56148967.83</v>
+        <v>56149337.83</v>
       </c>
       <c r="E106" s="12" t="n">
         <v>2.15</v>
@@ -19659,7 +19659,7 @@
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>47393236.7</v>
+        <v>47394053.15</v>
       </c>
       <c r="E107" s="12" t="n">
         <v>1.81</v>
@@ -19682,7 +19682,7 @@
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>46283661.9</v>
+        <v>46284731.82</v>
       </c>
       <c r="E108" s="12" t="n">
         <v>1.77</v>
@@ -19705,7 +19705,7 @@
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>45152823.49</v>
+        <v>45153063.13</v>
       </c>
       <c r="E109" s="12" t="n">
         <v>1.73</v>
@@ -19728,7 +19728,7 @@
         </is>
       </c>
       <c r="D110" s="6" t="n">
-        <v>44131438.22</v>
+        <v>44131907.24</v>
       </c>
       <c r="E110" s="12" t="n">
         <v>1.69</v>
@@ -19751,7 +19751,7 @@
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>42374174.35</v>
+        <v>42374379.09</v>
       </c>
       <c r="E111" s="12" t="n">
         <v>1.62</v>
@@ -19774,7 +19774,7 @@
         </is>
       </c>
       <c r="D112" s="6" t="n">
-        <v>41739509.63</v>
+        <v>41739817.8</v>
       </c>
       <c r="E112" s="12" t="n">
         <v>1.59</v>
@@ -19797,7 +19797,7 @@
         </is>
       </c>
       <c r="D113" s="6" t="n">
-        <v>35624630.42</v>
+        <v>35624690.42</v>
       </c>
       <c r="E113" s="12" t="n">
         <v>1.36</v>
@@ -19820,7 +19820,7 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>27673572.69</v>
+        <v>27673990.25</v>
       </c>
       <c r="E114" s="12" t="n">
         <v>1.06</v>
@@ -19843,7 +19843,7 @@
         </is>
       </c>
       <c r="D115" s="6" t="n">
-        <v>25358805.36</v>
+        <v>25359098.32</v>
       </c>
       <c r="E115" s="12" t="n">
         <v>0.97</v>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-26 09:17:45.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 09:01:54.</t>
         </is>
       </c>
     </row>
@@ -22581,13 +22581,13 @@
         <v>5043776.95</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>7671920.92</v>
+        <v>7793773.42</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>27260890.51</v>
+        <v>27382743.01</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>18.72</v>
+        <v>18.65</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>432131697.64</v>
@@ -22609,22 +22609,22 @@
         <v>20822161.87</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>15440831.37</v>
+        <v>15515831.37</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>4970836.14</v>
+        <v>5120836.14</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>25792998.01</v>
+        <v>25942998.01</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>17.72</v>
+        <v>17.67</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>322079944.32</v>
+        <v>322154944.32</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>16.65</v>
+        <v>16.66</v>
       </c>
     </row>
     <row r="7">
@@ -22649,7 +22649,7 @@
         <v>16031380.14</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>11.01</v>
+        <v>10.92</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>129267947.35</v>
@@ -22680,7 +22680,7 @@
         <v>15832602.75</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>10.87</v>
+        <v>10.79</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>178497634.1</v>
@@ -22705,13 +22705,13 @@
         <v>10352176.89</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>7469958.82</v>
+        <v>7629708.82</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>14267057.45</v>
+        <v>14426807.45</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>9.800000000000001</v>
+        <v>9.83</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>106182009.34</v>
@@ -22742,7 +22742,7 @@
         <v>7281014.58</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>5</v>
+        <v>4.96</v>
       </c>
       <c r="H10" s="6" t="n">
         <v>146467770.79</v>
@@ -22773,7 +22773,7 @@
         <v>6579241.1</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>4.52</v>
+        <v>4.48</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>129425907.52</v>
@@ -22795,22 +22795,22 @@
         <v>2398064.76</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>10853996.9</v>
+        <v>10611259.25</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>3568340.77</v>
+        <v>3833813.59</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>5966405.529999999</v>
+        <v>6231878.35</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>4.1</v>
+        <v>4.25</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>64480995.5</v>
+        <v>64238257.85</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>3.33</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="13">
@@ -22835,7 +22835,7 @@
         <v>5935999.58</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>4.08</v>
+        <v>4.04</v>
       </c>
       <c r="H13" s="6" t="n">
         <v>139900815.51</v>
@@ -22860,13 +22860,13 @@
         <v>50040</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>904244.78</v>
+        <v>962161.61</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>3161155.83</v>
+        <v>3219072.66</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>2.17</v>
+        <v>2.19</v>
       </c>
       <c r="H14" s="6" t="n">
         <v>62465731.73</v>
@@ -22897,7 +22897,7 @@
         <v>3107574.63</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>2.13</v>
+        <v>2.12</v>
       </c>
       <c r="H15" s="6" t="n">
         <v>46919216.33</v>
@@ -22922,13 +22922,13 @@
         <v>212885.86</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>595304.64</v>
+        <v>649607.63</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>2815219.2</v>
+        <v>2869522.19</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>1.93</v>
+        <v>1.95</v>
       </c>
       <c r="H16" s="6" t="n">
         <v>33012515.92</v>
@@ -22959,7 +22959,7 @@
         <v>2658732.31</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>1.83</v>
+        <v>1.81</v>
       </c>
       <c r="H17" s="6" t="n">
         <v>19269657</v>
@@ -22984,13 +22984,13 @@
         <v>766982</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1400921</v>
+        <v>1585921</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>1607021</v>
+        <v>1792021</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>1.1</v>
+        <v>1.22</v>
       </c>
       <c r="H18" s="6" t="n">
         <v>11294162.75</v>
@@ -23015,10 +23015,10 @@
         <v>16144.98</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>177284.49</v>
+        <v>195694.49</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>1231243.76</v>
+        <v>1249653.76</v>
       </c>
       <c r="G19" s="6" t="n">
         <v>0.85</v>
@@ -23052,7 +23052,7 @@
         <v>1206319.04</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0.83</v>
+        <v>0.82</v>
       </c>
       <c r="H20" s="6" t="n">
         <v>16005356.34</v>
@@ -23077,13 +23077,13 @@
         <v>25327.5</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>48767.64</v>
+        <v>128380.68</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>1029020.79</v>
+        <v>1108633.83</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>0.71</v>
+        <v>0.76</v>
       </c>
       <c r="H21" s="6" t="n">
         <v>19006025.91</v>
@@ -23201,13 +23201,13 @@
         <v>933500</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>334753.95</v>
+        <v>394753.95</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>0.23</v>
+        <v>0.27</v>
       </c>
       <c r="H25" s="6" t="n">
         <v>10399296.46</v>
@@ -23232,13 +23232,13 @@
         <v>19500</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>29510.94</v>
+        <v>69512.94</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>285706.22</v>
+        <v>325708.22</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="H26" s="6" t="n">
         <v>4369783.01</v>
@@ -23312,63 +23312,63 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Correspondências e despesas postais</t>
+          <t>Materiais de expediente</t>
         </is>
       </c>
       <c r="B29" s="6" t="n">
-        <v>10466575.67</v>
+        <v>2091545.81</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>219276</v>
+        <v>168725.58</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>8104.55</v>
+        <v>8076.8</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>0</v>
+        <v>54815.99</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>219276</v>
+        <v>223541.57</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>0.15</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>10474680.22</v>
+        <v>2099622.61</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>0.54</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Materiais de expediente</t>
+          <t>Correspondências e despesas postais</t>
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>2091545.81</v>
+        <v>10466575.67</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>168725.58</v>
+        <v>219276</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>8076.8</v>
+        <v>8104.55</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>48965.99</v>
+        <v>0</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>217691.57</v>
+        <v>219276</v>
       </c>
       <c r="G30" s="6" t="n">
         <v>0.15</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>2099622.61</v>
+        <v>10474680.22</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>0.11</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="31">
@@ -23601,19 +23601,19 @@
         <v>12476.63</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>89588.72</v>
+        <v>90688.66</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>7490.34</v>
+        <v>8337.379999999999</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>19966.97</v>
+        <v>20814.01</v>
       </c>
       <c r="G38" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>354732.11</v>
+        <v>355832.05</v>
       </c>
       <c r="I38" s="6" t="n">
         <v>0.02</v>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-26 09:17:45.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 09:01:54.</t>
         </is>
       </c>
     </row>
@@ -23825,7 +23825,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
@@ -24348,7 +24348,7 @@
         <v>4.6</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>930727493.99</v>
+        <v>931318345.11</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>192144239.43</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-26 09:17:45.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 09:01:54.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-26 09:17:45.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 09:01:54.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 28/09/2026 09:13
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 15:11:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 15:11:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>828</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-27 15:11:15</t>
+          <t>2026-09-28 09:03:04</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 15:11:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 15:11:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 15:11:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 15:11:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 15:11:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 15:11:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-27 15:11:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 28/09/2026 15:08
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>4808553854.53</v>
+        <v>4808907836.6</v>
       </c>
     </row>
     <row r="57">
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>4754610203.83</v>
+        <v>4754847597.83</v>
       </c>
     </row>
     <row r="58">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>502584184.15</v>
+        <v>505778862.15</v>
       </c>
     </row>
     <row r="59">
@@ -1514,7 +1514,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>454860362.3</v>
+        <v>458055040.3</v>
       </c>
     </row>
     <row r="60">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-28 09:03:04</t>
+          <t>2026-09-28 15:01:22</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>75659161.21000001</v>
+        <v>75659161.20999999</v>
       </c>
       <c r="H47" s="6" t="n">
         <v>0.23</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
         </is>
       </c>
     </row>
@@ -22578,7 +22578,7 @@
         <v>20301520.71</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>5043776.95</v>
+        <v>5069389.45</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>7793773.42</v>
@@ -22590,7 +22590,7 @@
         <v>18.45</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>443996722.16</v>
+        <v>444022334.66</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>22.24</v>
@@ -22702,7 +22702,7 @@
         <v>6876918.63</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>10352176.89</v>
+        <v>10360176.89</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>7629708.82</v>
@@ -22714,7 +22714,7 @@
         <v>9.529999999999999</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>108155653.64</v>
+        <v>108163653.64</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>5.42</v>
@@ -22733,7 +22733,7 @@
         <v>7610790.2</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1276644</v>
+        <v>1293819</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>382542.16</v>
@@ -22745,7 +22745,7 @@
         <v>5.25</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>152062636.23</v>
+        <v>152079811.23</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>7.62</v>
@@ -22764,7 +22764,7 @@
         <v>5043295.5</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>2145619.45</v>
+        <v>2148319.45</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>2025570.6</v>
@@ -22776,7 +22776,7 @@
         <v>4.64</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>131513829.82</v>
+        <v>131516529.82</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>6.59</v>
@@ -22826,7 +22826,7 @@
         <v>2460064.76</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>10611259.25</v>
+        <v>10635259.25</v>
       </c>
       <c r="E13" s="6" t="n">
         <v>3833813.59</v>
@@ -22838,7 +22838,7 @@
         <v>4.13</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>65687233.64</v>
+        <v>65711233.64</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>3.29</v>
@@ -22950,7 +22950,7 @@
         <v>1447189.49</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>326185.19</v>
+        <v>360815.21</v>
       </c>
       <c r="E17" s="6" t="n">
         <v>1211542.82</v>
@@ -22962,7 +22962,7 @@
         <v>1.75</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>19607067.63</v>
+        <v>19641697.65</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>0.98</v>
@@ -23167,7 +23167,7 @@
         <v>386653.95</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>933500</v>
+        <v>933850</v>
       </c>
       <c r="E24" s="6" t="n">
         <v>60000</v>
@@ -23179,7 +23179,7 @@
         <v>0.29</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>10612368.8</v>
+        <v>10612718.8</v>
       </c>
       <c r="I24" s="6" t="n">
         <v>0.53</v>
@@ -23229,7 +23229,7 @@
         <v>268457.36</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>19500</v>
+        <v>22074.32</v>
       </c>
       <c r="E26" s="6" t="n">
         <v>69512.94</v>
@@ -23241,7 +23241,7 @@
         <v>0.22</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>4571371.15</v>
+        <v>4573945.470000001</v>
       </c>
       <c r="I26" s="6" t="n">
         <v>0.23</v>
@@ -23415,7 +23415,7 @@
         <v>77483.94</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>3658.83</v>
+        <v>5031.08</v>
       </c>
       <c r="E32" s="6" t="n">
         <v>0</v>
@@ -23427,7 +23427,7 @@
         <v>0.05</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>661413.4399999999</v>
+        <v>662785.6899999999</v>
       </c>
       <c r="I32" s="6" t="n">
         <v>0.03</v>
@@ -23601,7 +23601,7 @@
         <v>12943.55</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>90708.66</v>
+        <v>90882.64</v>
       </c>
       <c r="E38" s="6" t="n">
         <v>8340.879999999999</v>
@@ -23613,7 +23613,7 @@
         <v>0.01</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>362979.89</v>
+        <v>363153.87</v>
       </c>
       <c r="I38" s="6" t="n">
         <v>0.02</v>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 28/09/2026 21:10
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -640,7 +640,7 @@
         <v>2.06</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>337146041.14</v>
+        <v>337221041.14</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>1.04</v>
@@ -671,7 +671,7 @@
         <v>53.81</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>12355307266.73</v>
+        <v>12355427266.73</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>38.14</v>
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32396628420.89</v>
+        <v>32396823420.89</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>77272</v>
+        <v>77274</v>
       </c>
     </row>
     <row r="31">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>32396628420.89</v>
+        <v>32396823420.89</v>
       </c>
     </row>
     <row r="34">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-28 15:01:22</t>
+          <t>2026-09-28 21:01:50</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.9499999</v>
+        <v>575680870.95</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.78</v>
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>75659161.20999999</v>
+        <v>75659161.21000001</v>
       </c>
       <c r="H47" s="6" t="n">
         <v>0.23</v>
@@ -4822,7 +4822,7 @@
         </is>
       </c>
       <c r="G48" s="6" t="n">
-        <v>75658784.06999999</v>
+        <v>75658784.07000001</v>
       </c>
       <c r="H48" s="6" t="n">
         <v>0.23</v>
@@ -5603,7 +5603,7 @@
         </is>
       </c>
       <c r="G59" s="6" t="n">
-        <v>62944315.4</v>
+        <v>62944315.40000001</v>
       </c>
       <c r="H59" s="6" t="n">
         <v>0.19</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
         </is>
       </c>
     </row>
@@ -24072,7 +24072,7 @@
         <v>5.4</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>2533019885.72</v>
+        <v>2533139885.72</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>567960113.11</v>
@@ -24348,7 +24348,7 @@
         <v>4.6</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>931318345.11</v>
+        <v>931393345.11</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>195840397.38</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 15:01:22.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 29/09/2026 03:12
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 03:01:53.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 03:01:53.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-28 21:01:50</t>
+          <t>2026-09-29 03:01:53</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 03:01:53.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 03:01:53.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 03:01:53.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 03:01:53.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 03:01:53.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 03:01:53.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-28 21:01:50.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 03:01:53.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 29/09/2026 21:11
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -665,13 +665,13 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>11293</v>
+        <v>11294</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>53.81</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>12355427266.73</v>
+        <v>12355909075.85</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>38.14</v>
@@ -882,13 +882,13 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>20987</v>
+        <v>20988</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32396823420.89</v>
+        <v>32397305230.01</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 15:04:24.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 15:04:24.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>20987</v>
+        <v>20988</v>
       </c>
     </row>
     <row r="14">
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>20987</v>
+        <v>20988</v>
       </c>
     </row>
     <row r="15">
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>20987</v>
+        <v>20988</v>
       </c>
     </row>
     <row r="16">
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>20984</v>
+        <v>20985</v>
       </c>
     </row>
     <row r="19">
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>77274</v>
+        <v>77280</v>
       </c>
     </row>
     <row r="31">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>32396823420.89</v>
+        <v>32397305230.01</v>
       </c>
     </row>
     <row r="34">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-29 15:04:24</t>
+          <t>2026-09-29 21:01:44</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>75659161.20999999</v>
+        <v>75659161.21000001</v>
       </c>
       <c r="H47" s="6" t="n">
         <v>0.23</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 15:04:24.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 15:04:24.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 15:04:24.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
         </is>
       </c>
     </row>
@@ -21338,10 +21338,10 @@
         </is>
       </c>
       <c r="D180" s="6" t="n">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="E180" s="12" t="n">
-        <v>4.31</v>
+        <v>4.32</v>
       </c>
     </row>
     <row r="181">
@@ -21594,7 +21594,7 @@
         <v>425</v>
       </c>
       <c r="E191" s="12" t="n">
-        <v>2.03</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="192">
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 15:04:24.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 15:04:24.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
         </is>
       </c>
     </row>
@@ -24204,13 +24204,13 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1419</v>
+        <v>1420</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>6.76</v>
+        <v>6.77</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>3339120580.55</v>
+        <v>3339602389.67</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>489418353.19</v>
@@ -24299,7 +24299,7 @@
         <v>1126</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>5.37</v>
+        <v>5.36</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>1457794419.27</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 15:04:24.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 15:04:24.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
         </is>
       </c>
     </row>
@@ -28228,7 +28228,7 @@
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>Nota 2: outras 4501 candidaturas NAO declararam receita alguma, das quais 924 sao vice ou suplente, que nao prestam conta propria. Ausencia de declaracao nao e' autofinanciamento, e por isso elas ficam fora desta tabela.</t>
+          <t>Nota 2: outras 4502 candidaturas NAO declararam receita alguma, das quais 924 sao vice ou suplente, que nao prestam conta propria. Ausencia de declaracao nao e' autofinanciamento, e por isso elas ficam fora desta tabela.</t>
         </is>
       </c>
     </row>
@@ -28844,7 +28844,7 @@
         <v>67.79000000000001</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="G16" s="5" t="n">
         <v>66</v>
@@ -28853,7 +28853,7 @@
         <v>76986</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>17.81</v>
+        <v>17.83</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>211367594.27</v>
@@ -29593,7 +29593,7 @@
         <v>73.69</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>20987</v>
+        <v>20988</v>
       </c>
       <c r="G33" s="8" t="n">
         <v>1790</v>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 30/09/2026 03:08
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-29 21:01:44</t>
+          <t>2026-09-30 03:01:16</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-29 21:01:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 30/09/2026 09:24
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 09:03:54.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 09:03:54.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-30 03:01:16</t>
+          <t>2026-09-30 09:03:54</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>75659161.21000001</v>
+        <v>75659161.20999999</v>
       </c>
       <c r="H47" s="6" t="n">
         <v>0.23</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 09:03:54.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 09:03:54.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 09:03:54.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 09:03:54.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 09:03:54.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 09:03:54.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 03:01:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 09:03:54.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 01/10/2026 10:52
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -671,7 +671,7 @@
         <v>53.81</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>12355909075.85</v>
+        <v>12356029456.34</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>38.14</v>
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32397305230.01</v>
+        <v>32397425610.5</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 15:13:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 15:13:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>77280</v>
+        <v>77287</v>
       </c>
     </row>
     <row r="31">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>32397305230.01</v>
+        <v>32397425610.5</v>
       </c>
     </row>
     <row r="34">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>678</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>4828055659.18</v>
+        <v>4834201798.98</v>
       </c>
     </row>
     <row r="57">
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>4771135909.28</v>
+        <v>4778281329.28</v>
       </c>
     </row>
     <row r="58">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>513845434.28</v>
+        <v>528045214.04</v>
       </c>
     </row>
     <row r="59">
@@ -1514,7 +1514,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>465919753.7</v>
+        <v>476858476.1</v>
       </c>
     </row>
     <row r="60">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-09-30 15:13:21</t>
+          <t>2026-10-01 10:33:02</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.9499999</v>
+        <v>575680870.95</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.78</v>
@@ -4751,7 +4751,7 @@
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>75659161.20999999</v>
+        <v>75659161.21000001</v>
       </c>
       <c r="H47" s="6" t="n">
         <v>0.23</v>
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="G63" s="6" t="n">
-        <v>58445503.79</v>
+        <v>58445503.79000001</v>
       </c>
       <c r="H63" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 15:13:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 15:13:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 15:13:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 15:13:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
         </is>
       </c>
     </row>
@@ -22581,19 +22581,19 @@
         <v>5990625.45</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>7793773.42</v>
+        <v>8052840.52</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>29944904</v>
+        <v>30203971.1</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>18.71</v>
+        <v>18.49</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>458330010.06</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>22.04</v>
+        <v>22.06</v>
       </c>
     </row>
     <row r="6">
@@ -22609,22 +22609,22 @@
         <v>22526202.73</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>15675831.37</v>
+        <v>15829031.37</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>5120836.14</v>
+        <v>5254836.14</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>27647038.87</v>
+        <v>27781038.87</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>17.27</v>
+        <v>17.01</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>339365331.9</v>
+        <v>339518531.9</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>16.32</v>
+        <v>16.34</v>
       </c>
     </row>
     <row r="7">
@@ -22640,7 +22640,7 @@
         <v>18071583.12</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>328350</v>
+        <v>328650</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>162830.33</v>
@@ -22649,13 +22649,13 @@
         <v>18234413.45</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>11.39</v>
+        <v>11.16</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>206512488.29</v>
+        <v>206512788.29</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>9.93</v>
+        <v>9.94</v>
       </c>
     </row>
     <row r="8">
@@ -22674,13 +22674,13 @@
         <v>6113730.34</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>13495322.55</v>
+        <v>14830072.55</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>16538970.14</v>
+        <v>17873720.14</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>10.33</v>
+        <v>10.94</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>136721289.8</v>
@@ -22702,22 +22702,22 @@
         <v>7060017.63</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>10360176.89</v>
+        <v>9164676.890000001</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>7769708.82</v>
+        <v>8666108.82</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>14829726.45</v>
+        <v>15726126.45</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>9.26</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>110842203.64</v>
+        <v>109646703.64</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.33</v>
+        <v>5.28</v>
       </c>
     </row>
     <row r="10">
@@ -22736,13 +22736,13 @@
         <v>1367612</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>382542.16</v>
+        <v>472076.16</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>8713971.99</v>
+        <v>8803505.99</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>5.44</v>
+        <v>5.39</v>
       </c>
       <c r="H10" s="6" t="n">
         <v>162688883.5</v>
@@ -22767,19 +22767,19 @@
         <v>542259.41</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>202368</v>
+        <v>270650.66</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>7681448.78</v>
+        <v>7749731.44</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>4.8</v>
+        <v>4.74</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>154319282.15</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7.42</v>
+        <v>7.43</v>
       </c>
     </row>
     <row r="12">
@@ -22798,13 +22798,13 @@
         <v>2148319.45</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>2025570.6</v>
+        <v>2054580.6</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>7196159.960000001</v>
+        <v>7225169.960000001</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>4.5</v>
+        <v>4.42</v>
       </c>
       <c r="H12" s="6" t="n">
         <v>136550181.98</v>
@@ -22826,19 +22826,19 @@
         <v>2576933.74</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>10668209.27</v>
+        <v>10710109.27</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>3860313.59</v>
+        <v>4232613.59</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>6437247.33</v>
+        <v>6809547.33</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>4.02</v>
+        <v>4.17</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>67165758.36</v>
+        <v>67207658.36</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>3.23</v>
@@ -22860,13 +22860,13 @@
         <v>50040</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>962161.61</v>
+        <v>987161.61</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>3529932.02</v>
+        <v>3554932.02</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>2.21</v>
+        <v>2.18</v>
       </c>
       <c r="H14" s="6" t="n">
         <v>67219062.33</v>
@@ -22897,7 +22897,7 @@
         <v>3401023.78</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>2.12</v>
+        <v>2.08</v>
       </c>
       <c r="H15" s="6" t="n">
         <v>48722266.66</v>
@@ -22928,7 +22928,7 @@
         <v>3112459.75</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>1.94</v>
+        <v>1.91</v>
       </c>
       <c r="H16" s="6" t="n">
         <v>21078988.82</v>
@@ -22953,13 +22953,13 @@
         <v>212885.86</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>649607.63</v>
+        <v>657107.63</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>3014398.19</v>
+        <v>3021898.19</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>1.88</v>
+        <v>1.85</v>
       </c>
       <c r="H17" s="6" t="n">
         <v>34621441.92</v>
@@ -22984,13 +22984,13 @@
         <v>891275</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1585921</v>
+        <v>1630921</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>1812021</v>
+        <v>1857021</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="H18" s="6" t="n">
         <v>11837387.65</v>
@@ -23021,7 +23021,7 @@
         <v>1293333.76</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="H19" s="6" t="n">
         <v>10440788.11</v>
@@ -23052,7 +23052,7 @@
         <v>1217919.04</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H20" s="6" t="n">
         <v>17118044.58</v>
@@ -23083,7 +23083,7 @@
         <v>1162181.93</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
       <c r="H21" s="6" t="n">
         <v>20859987.55</v>
@@ -23114,7 +23114,7 @@
         <v>966073.29</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
       <c r="H22" s="6" t="n">
         <v>9879105.67</v>
@@ -23145,7 +23145,7 @@
         <v>708832.35</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="H23" s="6" t="n">
         <v>12327241.96</v>
@@ -23176,7 +23176,7 @@
         <v>399253.95</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>11576593.4</v>
@@ -23269,7 +23269,7 @@
         <v>318080.58</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="H27" s="6" t="n">
         <v>4891188.27</v>
@@ -23300,7 +23300,7 @@
         <v>299961.15</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="H28" s="6" t="n">
         <v>12151906.48</v>
@@ -23331,7 +23331,7 @@
         <v>269240.64</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="H29" s="6" t="n">
         <v>3081820.14</v>
@@ -23517,7 +23517,7 @@
         <v>40173.94</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="H35" s="6" t="n">
         <v>927554.89</v>
@@ -23601,19 +23601,19 @@
         <v>13299.67</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>92174.00999999999</v>
+        <v>92993.81</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>8413.48</v>
+        <v>8627.08</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>21713.15</v>
+        <v>21926.75</v>
       </c>
       <c r="G38" s="6" t="n">
         <v>0.01</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>400487.27</v>
+        <v>401307.07</v>
       </c>
       <c r="I38" s="6" t="n">
         <v>0.02</v>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 15:13:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
         </is>
       </c>
     </row>
@@ -24394,7 +24394,7 @@
         <v>5.21</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>2591573797.35</v>
+        <v>2591694177.84</v>
       </c>
       <c r="E15" s="6" t="n">
         <v>190867359.45</v>
@@ -24973,7 +24973,7 @@
         <v>4041559.33</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>6970270.9</v>
+        <v>6970270.899999999</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>26.21</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 15:13:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-09-30 15:13:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 01/10/2026 15:34
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 15:18:36.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 15:18:36.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-01 10:33:02</t>
+          <t>2026-10-01 15:18:36</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.95</v>
+        <v>575680870.9499999</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.78</v>
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="G63" s="6" t="n">
-        <v>58445503.79000001</v>
+        <v>58445503.79</v>
       </c>
       <c r="H63" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 15:18:36.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 15:18:36.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 15:18:36.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 15:18:36.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 15:18:36.</t>
         </is>
       </c>
     </row>
@@ -24973,7 +24973,7 @@
         <v>4041559.33</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>6970270.899999999</v>
+        <v>6970270.9</v>
       </c>
       <c r="N27" s="6" t="n">
         <v>26.21</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 15:18:36.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 10:33:02.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-01 15:18:36.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 03/10/2026 16:50
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -665,16 +665,16 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>11294</v>
+        <v>11295</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>53.81</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>12006494956.34</v>
+        <v>12006774956.34</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>37.46</v>
+        <v>37.47</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>1718637324.19</v>
@@ -882,13 +882,13 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>20988</v>
+        <v>20989</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32047377110.5</v>
+        <v>32047657110.5</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 15:14:13.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 15:14:13.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>20988</v>
+        <v>20989</v>
       </c>
     </row>
     <row r="14">
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>20988</v>
+        <v>20989</v>
       </c>
     </row>
     <row r="15">
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>20988</v>
+        <v>20989</v>
       </c>
     </row>
     <row r="16">
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>20985</v>
+        <v>20986</v>
       </c>
     </row>
     <row r="19">
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>77288</v>
+        <v>77289</v>
       </c>
     </row>
     <row r="31">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>32047377110.5</v>
+        <v>32047657110.5</v>
       </c>
     </row>
     <row r="34">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1377</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-03 15:14:13</t>
+          <t>2026-10-03 16:42:27</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.9499999</v>
+        <v>575680870.95</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.8</v>
@@ -5532,7 +5532,7 @@
         </is>
       </c>
       <c r="G58" s="6" t="n">
-        <v>62944315.4</v>
+        <v>62944315.40000001</v>
       </c>
       <c r="H58" s="6" t="n">
         <v>0.2</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 15:14:13.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 15:14:13.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 15:14:13.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
         </is>
       </c>
     </row>
@@ -21384,7 +21384,7 @@
         </is>
       </c>
       <c r="D182" s="6" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="E182" s="12" t="n">
         <v>3.4</v>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 15:14:13.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 15:14:13.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
         </is>
       </c>
     </row>
@@ -24894,13 +24894,13 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>2.76</v>
+        <v>2.77</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>242782021.57</v>
+        <v>243062021.57</v>
       </c>
       <c r="E26" s="6" t="n">
         <v>9423852.75</v>
@@ -25035,7 +25035,7 @@
         <v>467</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>2.23</v>
+        <v>2.22</v>
       </c>
       <c r="D29" s="6" t="n">
         <v>463597846.48</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 15:14:13.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 15:14:13.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
         </is>
       </c>
     </row>
@@ -28228,7 +28228,7 @@
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>Nota 2: outras 4292 candidaturas NAO declararam receita alguma, das quais 924 sao vice ou suplente, que nao prestam conta propria. Ausencia de declaracao nao e' autofinanciamento, e por isso elas ficam fora desta tabela.</t>
+          <t>Nota 2: outras 4293 candidaturas NAO declararam receita alguma, das quais 924 sao vice ou suplente, que nao prestam conta propria. Ausencia de declaracao nao e' autofinanciamento, e por isso elas ficam fora desta tabela.</t>
         </is>
       </c>
     </row>
@@ -28672,7 +28672,7 @@
         <v>75.26000000000001</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>76</v>
@@ -28681,7 +28681,7 @@
         <v>92118</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>10.18</v>
+        <v>10.2</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>242341798.97</v>
@@ -29593,7 +29593,7 @@
         <v>73.69</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>20988</v>
+        <v>20989</v>
       </c>
       <c r="G33" s="8" t="n">
         <v>1790</v>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 03/10/2026 21:11
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -640,10 +640,10 @@
         <v>2.06</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>337221041.14</v>
+        <v>338296381.14</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>45409970.61</v>
@@ -674,7 +674,7 @@
         <v>12006774956.34</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>37.47</v>
+        <v>37.46</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>1718637324.19</v>
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32047657110.5</v>
+        <v>32048732450.5</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 21:02:10.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 21:02:10.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>77289</v>
+        <v>77294</v>
       </c>
     </row>
     <row r="31">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>32047657110.5</v>
+        <v>32048732450.5</v>
       </c>
     </row>
     <row r="34">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-03 16:42:27</t>
+          <t>2026-10-03 21:02:10</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.95</v>
+        <v>575680870.9499999</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.8</v>
@@ -3121,7 +3121,7 @@
         <v>184278955.2</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="I24" s="5" t="n">
         <v>53</v>
@@ -4680,7 +4680,7 @@
         </is>
       </c>
       <c r="G46" s="6" t="n">
-        <v>75659161.20999999</v>
+        <v>75659161.21000001</v>
       </c>
       <c r="H46" s="6" t="n">
         <v>0.24</v>
@@ -5532,7 +5532,7 @@
         </is>
       </c>
       <c r="G58" s="6" t="n">
-        <v>62944315.40000001</v>
+        <v>62944315.4</v>
       </c>
       <c r="H58" s="6" t="n">
         <v>0.2</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 21:02:10.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 21:02:10.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 21:02:10.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 21:02:10.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 21:02:10.</t>
         </is>
       </c>
     </row>
@@ -23934,7 +23934,7 @@
         <v>7.85</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>4898750244.67</v>
+        <v>4898820044.67</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>1120393927.99</v>
@@ -24072,7 +24072,7 @@
         <v>5.4</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>2533139885.72</v>
+        <v>2534145425.72</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>609952077.85</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 21:02:10.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 16:42:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-03 21:02:10.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 05/10/2026 08:34
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -9373,7 +9373,7 @@
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>PL; UNIÃO; REPUBLICANOS; PT</t>
+          <t>PL; UNIÃO; REPUBLICANOS; MDB</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
@@ -9568,7 +9568,7 @@
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>UNIÃO; PSDB; PP; PL</t>
+          <t>UNIÃO; PSDB; REPUBLICANOS; PP</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
@@ -9638,7 +9638,7 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>ANDRÉ DO PRADO (PL); ELEUSES PAIVA (PSD)</t>
+          <t>ELEUSES PAIVA (PSD); ANDRÉ DO PRADO (PL)</t>
         </is>
       </c>
     </row>
@@ -10088,7 +10088,7 @@
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>PDT; PCDOB; PSD; UNIÃO</t>
+          <t>PDT; PSD; PCDOB; UNIÃO</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
@@ -10158,7 +10158,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>LULA (PT); PATRUS ANANIAS (PT)</t>
+          <t>LULA (PT); MENDONÇA FILHO (PL)</t>
         </is>
       </c>
     </row>
@@ -10543,7 +10543,7 @@
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>PL; PSD; UNIÃO; PT</t>
+          <t>PSD; PL; UNIÃO; PT</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
@@ -10613,7 +10613,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>FLAVIO BOLSONARO (PL); ARLINDO CHINAGLIA (PT)</t>
+          <t>FLAVIO BOLSONARO (PL); CARLOS ZARATTINI (PT)</t>
         </is>
       </c>
     </row>
@@ -12038,7 +12038,7 @@
       </c>
       <c r="N51" s="4" t="inlineStr">
         <is>
-          <t>PSD; MDB; UNIÃO; REPUBLICANOS</t>
+          <t>PSD; MDB; REPUBLICANOS; UNIÃO</t>
         </is>
       </c>
       <c r="O51" s="4" t="inlineStr">
@@ -13143,7 +13143,7 @@
       </c>
       <c r="N68" s="4" t="inlineStr">
         <is>
-          <t>PP; PL; NOVO; PSD</t>
+          <t>PP; NOVO; PL; PSD</t>
         </is>
       </c>
       <c r="O68" s="4" t="inlineStr">
@@ -13208,12 +13208,12 @@
       </c>
       <c r="N69" s="4" t="inlineStr">
         <is>
-          <t>PSD; REPUBLICANOS; MDB; PL</t>
+          <t>PSD; MDB; REPUBLICANOS; PL</t>
         </is>
       </c>
       <c r="O69" s="4" t="inlineStr">
         <is>
-          <t>TARCÍSIO (REPUBLICANOS); DUARTE NOGUEIRA (PSD)</t>
+          <t>TARCÍSIO (REPUBLICANOS); BALEIA ROSSI (MDB)</t>
         </is>
       </c>
     </row>
@@ -13533,12 +13533,12 @@
       </c>
       <c r="N74" s="4" t="inlineStr">
         <is>
-          <t>REDE; PSOL; PT; PSD</t>
+          <t>REDE; PSD; PSOL; PT</t>
         </is>
       </c>
       <c r="O74" s="4" t="inlineStr">
         <is>
-          <t>MARINA SILVA (REDE); SÔNIA GUAJAJARA (PSOL)</t>
+          <t>MARINA SILVA (REDE); RACHEL SHEHERAZADE (PSD)</t>
         </is>
       </c>
     </row>
@@ -14058,7 +14058,7 @@
       </c>
       <c r="O82" s="4" t="inlineStr">
         <is>
-          <t>DOUTOR JHONY (PSD); SILVIA DA PESCA (PODE)</t>
+          <t>DOUTOR JHONY (PSD); MERSINHO LUCENA (PSD)</t>
         </is>
       </c>
     </row>
@@ -14313,7 +14313,7 @@
       </c>
       <c r="N86" s="4" t="inlineStr">
         <is>
-          <t>PL; PSD; PP; REPUBLICANOS</t>
+          <t>PL; PSD; PT; PP</t>
         </is>
       </c>
       <c r="O86" s="4" t="inlineStr">
@@ -14833,7 +14833,7 @@
       </c>
       <c r="N94" s="4" t="inlineStr">
         <is>
-          <t>PT; UNIÃO; REPUBLICANOS; MDB</t>
+          <t>UNIÃO; PT; REPUBLICANOS; MDB</t>
         </is>
       </c>
       <c r="O94" s="4" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="N98" s="4" t="inlineStr">
         <is>
-          <t>PL; PV; PT; PDT</t>
+          <t>PL; PT; PV; PDT</t>
         </is>
       </c>
       <c r="O98" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 05/10/2026 15:21
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -671,10 +671,10 @@
         <v>53.81</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>12006774956.34</v>
+        <v>12007234956.34</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>37.46</v>
+        <v>37.47</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>1740653890.53</v>
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32048732450.5</v>
+        <v>32049192450.5</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 10:04:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 15:05:45.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 10:04:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 15:05:45.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>77294</v>
+        <v>77297</v>
       </c>
     </row>
     <row r="31">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>32048732450.5</v>
+        <v>32049192450.5</v>
       </c>
     </row>
     <row r="34">
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0</v>
+        <v>6661888</v>
       </c>
     </row>
     <row r="61">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-05 10:04:29</t>
+          <t>2026-10-05 15:05:45</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>["VOTOS_VALIDOS_1T", "RESULTADO"]</t>
         </is>
       </c>
     </row>
@@ -4680,7 +4680,7 @@
         </is>
       </c>
       <c r="G46" s="6" t="n">
-        <v>75659161.20999999</v>
+        <v>75659161.21000001</v>
       </c>
       <c r="H46" s="6" t="n">
         <v>0.24</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 10:04:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 15:05:45.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 10:04:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 15:05:45.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 10:04:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 15:05:45.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 10:04:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 15:05:45.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 10:04:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 15:05:45.</t>
         </is>
       </c>
     </row>
@@ -24900,7 +24900,7 @@
         <v>2.77</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>243062021.57</v>
+        <v>243522021.57</v>
       </c>
       <c r="E26" s="6" t="n">
         <v>9643703.76</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 10:04:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 15:05:45.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 10:04:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-05 15:05:45.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 06/10/2026 15:45
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 09:12:51.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 15:16:20.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 09:12:51.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 15:16:20.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>758</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-06 09:12:51</t>
+          <t>2026-10-06 15:16:20</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 09:12:51.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 15:16:20.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 09:12:51.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 15:16:20.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 09:12:51.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 15:16:20.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 09:12:51.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 15:16:20.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 09:12:51.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 15:16:20.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 09:12:51.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 15:16:20.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 09:12:51.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-06 15:16:20.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 08/10/2026 09:35
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,14 +909,14 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 06:53:14.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-07.</t>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-08.</t>
         </is>
       </c>
     </row>
@@ -1025,14 +1025,14 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 06:53:14.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-07.</t>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-08.</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>171354</v>
+        <v>172432</v>
       </c>
     </row>
     <row r="24">
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>6485748140.81</v>
+        <v>6499395514.29</v>
       </c>
     </row>
     <row r="26">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>{"REC_FEFC": 4818741267.43, "REC_FINANCIAMENTO_COLETIVO": 17574106.81, "REC_FUNDO_PARTIDARIO": 538846836.48, "REC_ORIGEM_NAO_IDENTIFICADA": 1119823.18, "REC_OUTROS_CANDIDATOS": 118629219.19, "REC_PARTIDO_OUTROS_RECURSOS": 197024752.4, "REC_PESSOAS_FISICAS": 638514963.77, "REC_PROPRIOS": 155297171.55, "REC_SEM_ORIGEM": 0.0}</t>
+          <t>{"REC_FEFC": 4820517991.59, "REC_FINANCIAMENTO_COLETIVO": 17893226.27, "REC_FUNDO_PARTIDARIO": 539998866.01, "REC_ORIGEM_NAO_IDENTIFICADA": 1111351.96, "REC_OUTROS_CANDIDATOS": 119614174.89, "REC_PARTIDO_OUTROS_RECURSOS": 197783790.57, "REC_PESSOAS_FISICAS": 644833517.92, "REC_PROPRIOS": 157642595.08, "REC_SEM_ORIGEM": 0.0}</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>76673</v>
+        <v>77181</v>
       </c>
     </row>
     <row r="30">
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>972276</v>
+        <v>978191</v>
       </c>
     </row>
     <row r="36">
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>773200</v>
+        <v>777849</v>
       </c>
     </row>
     <row r="37">
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>4446361078.23</v>
+        <v>4462223543.88</v>
       </c>
     </row>
     <row r="38">
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>668061</v>
+        <v>683428</v>
       </c>
     </row>
     <row r="39">
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3051673419.1</v>
+        <v>3088142099.12</v>
       </c>
     </row>
     <row r="40">
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>70429</v>
+        <v>71176</v>
       </c>
     </row>
     <row r="43">
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>703318.24</v>
+        <v>711894.52</v>
       </c>
     </row>
     <row r="44">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>536391</v>
+        <v>538865</v>
       </c>
     </row>
     <row r="46">
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>55116</v>
+        <v>55393</v>
       </c>
     </row>
     <row r="48">
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>54975</v>
+        <v>55248</v>
       </c>
     </row>
     <row r="49">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="50">
@@ -1434,7 +1434,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>973</v>
+        <v>957</v>
       </c>
     </row>
     <row r="52">
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2476493769.98</v>
+        <v>2497165173.04</v>
       </c>
     </row>
     <row r="53">
@@ -1454,7 +1454,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>62467265.72</v>
+        <v>63098984.72</v>
       </c>
     </row>
     <row r="54">
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>171112707.12</v>
+        <v>175037098.64</v>
       </c>
     </row>
     <row r="55">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2454620.52</v>
+        <v>2458620.52</v>
       </c>
     </row>
     <row r="56">
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>4866017907.18</v>
+        <v>4867433267.48</v>
       </c>
     </row>
     <row r="57">
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>4792590050.36</v>
+        <v>4794001980.36</v>
       </c>
     </row>
     <row r="58">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>560363771.8200001</v>
+        <v>560638228.26</v>
       </c>
     </row>
     <row r="59">
@@ -1514,7 +1514,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>501831902.14</v>
+        <v>501966882.14</v>
       </c>
     </row>
     <row r="60">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-08 06:53:14</t>
+          <t>2026-10-08 09:03:34</t>
         </is>
       </c>
     </row>
@@ -8842,14 +8842,14 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 06:53:14.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-07.</t>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-08.</t>
         </is>
       </c>
     </row>
@@ -15495,14 +15495,14 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 06:53:14.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-07.</t>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-08.</t>
         </is>
       </c>
     </row>
@@ -17206,14 +17206,14 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 06:53:14.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-07.</t>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-08.</t>
         </is>
       </c>
     </row>
@@ -22451,14 +22451,14 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 06:53:14.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="10" t="inlineStr">
         <is>
-          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-07.</t>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-08.</t>
         </is>
       </c>
     </row>
@@ -23777,14 +23777,14 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 06:53:14.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-07.</t>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-08.</t>
         </is>
       </c>
     </row>
@@ -25304,14 +25304,14 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 06:53:14.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-07.</t>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-08.</t>
         </is>
       </c>
     </row>
@@ -28207,14 +28207,14 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 06:53:14.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-07.</t>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-08.</t>
         </is>
       </c>
     </row>
@@ -29627,7 +29627,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-07.</t>
+          <t>Nota: a prestacao de contas eleitoral e' PARCIAL e e' atualizada diariamente pelo TSE. Ultima data de prestacao presente na base: 2026-10-08.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 08/10/2026 15:11
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -578,10 +578,10 @@
         <v>1.66</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>4461861531.07</v>
+        <v>4464124482.29</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>13.92</v>
+        <v>13.93</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>0</v>
@@ -674,7 +674,7 @@
         <v>12007434756.34</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>37.47</v>
+        <v>37.46</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>1772759804.56</v>
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32049392250.5</v>
+        <v>32051655201.72</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 15:03:33.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 15:03:33.</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>77297</v>
+        <v>77316</v>
       </c>
     </row>
     <row r="31">
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>32049392250.5</v>
+        <v>32051655201.72</v>
       </c>
     </row>
     <row r="34">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-08 09:03:34</t>
+          <t>2026-10-08 15:03:33</t>
         </is>
       </c>
     </row>
@@ -4680,7 +4680,7 @@
         </is>
       </c>
       <c r="G46" s="6" t="n">
-        <v>75659161.21000001</v>
+        <v>75659161.20999999</v>
       </c>
       <c r="H46" s="6" t="n">
         <v>0.24</v>
@@ -8446,7 +8446,7 @@
         <v>40063200</v>
       </c>
       <c r="H99" s="6" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="I99" s="5" t="n">
         <v>22</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 15:03:33.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 15:03:33.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 15:03:33.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 15:03:33.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 15:03:33.</t>
         </is>
       </c>
     </row>
@@ -24072,7 +24072,7 @@
         <v>5.4</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>2534145425.72</v>
+        <v>2536408376.94</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>630875611.73</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 15:03:33.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 09:03:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-08 15:03:33.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 09/10/2026 19:00
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 13:33:26.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 18:50:07.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 13:33:26.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 18:50:07.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3</v>
+        <v>231</v>
       </c>
     </row>
     <row r="47">
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>55396</v>
+        <v>55637</v>
       </c>
     </row>
     <row r="48">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>282</v>
+        <v>58</v>
       </c>
     </row>
     <row r="50">
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>6737183</v>
+        <v>6706621</v>
       </c>
     </row>
     <row r="61">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-09 13:33:26</t>
+          <t>2026-10-09 18:50:07</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.95</v>
+        <v>575680870.9499999</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.79</v>
@@ -5816,7 +5816,7 @@
         </is>
       </c>
       <c r="G62" s="6" t="n">
-        <v>58445503.79000001</v>
+        <v>58445503.79</v>
       </c>
       <c r="H62" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 13:33:26.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 18:50:07.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 13:33:26.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 18:50:07.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 13:33:26.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 18:50:07.</t>
         </is>
       </c>
     </row>
@@ -19245,7 +19245,7 @@
         </is>
       </c>
       <c r="D89" s="6" t="n">
-        <v>803006087.61</v>
+        <v>803275588.21</v>
       </c>
       <c r="E89" s="12" t="n">
         <v>25.84</v>
@@ -19268,7 +19268,7 @@
         </is>
       </c>
       <c r="D90" s="6" t="n">
-        <v>201274903.61</v>
+        <v>201313907.16</v>
       </c>
       <c r="E90" s="12" t="n">
         <v>6.48</v>
@@ -19291,7 +19291,7 @@
         </is>
       </c>
       <c r="D91" s="6" t="n">
-        <v>185694104.16</v>
+        <v>185868293.63</v>
       </c>
       <c r="E91" s="12" t="n">
         <v>5.98</v>
@@ -19314,7 +19314,7 @@
         </is>
       </c>
       <c r="D92" s="6" t="n">
-        <v>156000157.57</v>
+        <v>156006823.63</v>
       </c>
       <c r="E92" s="12" t="n">
         <v>5.02</v>
@@ -19337,7 +19337,7 @@
         </is>
       </c>
       <c r="D93" s="6" t="n">
-        <v>139922914.49</v>
+        <v>139965790.09</v>
       </c>
       <c r="E93" s="12" t="n">
         <v>4.5</v>
@@ -19360,7 +19360,7 @@
         </is>
       </c>
       <c r="D94" s="6" t="n">
-        <v>124693773.27</v>
+        <v>124777509.58</v>
       </c>
       <c r="E94" s="12" t="n">
         <v>4.01</v>
@@ -19383,7 +19383,7 @@
         </is>
       </c>
       <c r="D95" s="6" t="n">
-        <v>122765809.64</v>
+        <v>122776549.64</v>
       </c>
       <c r="E95" s="12" t="n">
         <v>3.95</v>
@@ -19406,7 +19406,7 @@
         </is>
       </c>
       <c r="D96" s="6" t="n">
-        <v>118110886.99</v>
+        <v>118244586.69</v>
       </c>
       <c r="E96" s="12" t="n">
         <v>3.8</v>
@@ -19429,7 +19429,7 @@
         </is>
       </c>
       <c r="D97" s="6" t="n">
-        <v>107392100.21</v>
+        <v>107587049.99</v>
       </c>
       <c r="E97" s="12" t="n">
         <v>3.46</v>
@@ -19452,7 +19452,7 @@
         </is>
       </c>
       <c r="D98" s="6" t="n">
-        <v>106467061.09</v>
+        <v>106774005.47</v>
       </c>
       <c r="E98" s="12" t="n">
         <v>3.43</v>
@@ -19475,7 +19475,7 @@
         </is>
       </c>
       <c r="D99" s="6" t="n">
-        <v>93776156.98999999</v>
+        <v>93790000.17</v>
       </c>
       <c r="E99" s="12" t="n">
         <v>3.02</v>
@@ -19498,7 +19498,7 @@
         </is>
       </c>
       <c r="D100" s="6" t="n">
-        <v>93667391.73</v>
+        <v>93696280.23</v>
       </c>
       <c r="E100" s="12" t="n">
         <v>3.01</v>
@@ -19521,7 +19521,7 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>85800132.06</v>
+        <v>85821334.78</v>
       </c>
       <c r="E101" s="12" t="n">
         <v>2.76</v>
@@ -19544,7 +19544,7 @@
         </is>
       </c>
       <c r="D102" s="6" t="n">
-        <v>84864555.48999999</v>
+        <v>84954922.27</v>
       </c>
       <c r="E102" s="12" t="n">
         <v>2.73</v>
@@ -19567,7 +19567,7 @@
         </is>
       </c>
       <c r="D103" s="6" t="n">
-        <v>74041631.22</v>
+        <v>74061922.67</v>
       </c>
       <c r="E103" s="12" t="n">
         <v>2.38</v>
@@ -19590,7 +19590,7 @@
         </is>
       </c>
       <c r="D104" s="6" t="n">
-        <v>73221516.77</v>
+        <v>73223846.77</v>
       </c>
       <c r="E104" s="12" t="n">
         <v>2.36</v>
@@ -19636,7 +19636,7 @@
         </is>
       </c>
       <c r="D106" s="6" t="n">
-        <v>59710995.88</v>
+        <v>59767995.88</v>
       </c>
       <c r="E106" s="12" t="n">
         <v>1.92</v>
@@ -19659,7 +19659,7 @@
         </is>
       </c>
       <c r="D107" s="6" t="n">
-        <v>56858624.46</v>
+        <v>56904220.24</v>
       </c>
       <c r="E107" s="12" t="n">
         <v>1.83</v>
@@ -19682,7 +19682,7 @@
         </is>
       </c>
       <c r="D108" s="6" t="n">
-        <v>53771897.11</v>
+        <v>53815730.83</v>
       </c>
       <c r="E108" s="12" t="n">
         <v>1.73</v>
@@ -19705,7 +19705,7 @@
         </is>
       </c>
       <c r="D109" s="6" t="n">
-        <v>51930816.04</v>
+        <v>52017316.04</v>
       </c>
       <c r="E109" s="12" t="n">
         <v>1.67</v>
@@ -19731,7 +19731,7 @@
         <v>51437272.95</v>
       </c>
       <c r="E110" s="12" t="n">
-        <v>1.66</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="111">
@@ -19751,7 +19751,7 @@
         </is>
       </c>
       <c r="D111" s="6" t="n">
-        <v>48042549.9</v>
+        <v>48046110.9</v>
       </c>
       <c r="E111" s="12" t="n">
         <v>1.55</v>
@@ -19820,7 +19820,7 @@
         </is>
       </c>
       <c r="D114" s="6" t="n">
-        <v>30805520.48</v>
+        <v>30823545.36</v>
       </c>
       <c r="E114" s="12" t="n">
         <v>0.99</v>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 13:33:26.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 18:50:07.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 13:33:26.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 18:50:07.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 13:33:26.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 18:50:07.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 13:33:26.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-09 18:50:07.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 10/10/2026 09:10
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 06:49:42.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 06:49:42.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>253</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-10 06:49:42</t>
+          <t>2026-10-10 09:03:04</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 06:49:42.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 06:49:42.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 06:49:42.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 06:49:42.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 06:49:42.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 06:49:42.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 06:49:42.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 10/10/2026 15:10
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -581,7 +581,7 @@
         <v>4495080252.41</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>13.67</v>
+        <v>13.66</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>0</v>
@@ -655,7 +655,7 @@
         <v>31995985.59</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="8">
@@ -668,25 +668,25 @@
         <v>11295</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>53.66</v>
+        <v>53.63</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>12007434756.34</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>36.51</v>
+        <v>36.5</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>1783225197.04</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>24.61</v>
+        <v>24.54</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>1174536671.28</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>23.39</v>
+        <v>23.25</v>
       </c>
     </row>
     <row r="9">
@@ -699,25 +699,25 @@
         <v>7803</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>37.07</v>
+        <v>37.05</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>8707767692.280001</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>26.48</v>
+        <v>26.47</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>3396921482.72</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>46.88</v>
+        <v>46.74</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>2271018014.26</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>45.22</v>
+        <v>44.96</v>
       </c>
     </row>
     <row r="10">
@@ -727,28 +727,28 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>1.07</v>
+        <v>1.1</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1753027042.26</v>
+        <v>1755573651.78</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.33</v>
+        <v>5.34</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>729348136.9300001</v>
+        <v>749780272.78</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>10.06</v>
+        <v>10.32</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>580042105.5700001</v>
+        <v>608553187</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>11.55</v>
+        <v>12.05</v>
       </c>
     </row>
     <row r="11">
@@ -761,7 +761,7 @@
         <v>20</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>1223996865.97</v>
@@ -773,13 +773,13 @@
         <v>771349229.63</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>10.64</v>
+        <v>10.61</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>577600810.63</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>11.5</v>
+        <v>11.44</v>
       </c>
     </row>
     <row r="12">
@@ -792,7 +792,7 @@
         <v>319</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>1.52</v>
+        <v>1.51</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>2079741446.05</v>
@@ -804,13 +804,13 @@
         <v>518076265.71</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>7.15</v>
+        <v>7.13</v>
       </c>
       <c r="H12" s="6" t="n">
         <v>387212575.68</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>7.71</v>
+        <v>7.67</v>
       </c>
     </row>
     <row r="13">
@@ -820,16 +820,16 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>785862735.59</v>
+        <v>791514463.25</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>2.39</v>
+        <v>2.41</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>0</v>
@@ -854,7 +854,7 @@
         <v>20</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>575737935.76</v>
@@ -882,25 +882,25 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>21049</v>
+        <v>21061</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32890384607.86</v>
+        <v>32898582945.04</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>7246570798.099999</v>
+        <v>7267002933.95</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>100</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>5022406163.01</v>
+        <v>5050917244.440001</v>
       </c>
       <c r="I15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>21009</v>
+        <v>21013</v>
       </c>
     </row>
     <row r="14">
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21009</v>
+        <v>21013</v>
       </c>
     </row>
     <row r="16">
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>21046</v>
+        <v>21058</v>
       </c>
     </row>
     <row r="19">
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>171</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22">
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>279</v>
+        <v>295</v>
       </c>
     </row>
     <row r="23">
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>6706621</v>
+        <v>6737183</v>
       </c>
     </row>
     <row r="61">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-10 09:03:04</t>
+          <t>2026-10-10 15:03:15</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>-691554841.14</v>
+        <v>-711986976.99</v>
       </c>
     </row>
     <row r="65">
@@ -2340,7 +2340,7 @@
         <v>495030000</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>1.51</v>
+        <v>1.5</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>5</v>
@@ -3209,7 +3209,7 @@
         <v>5446578.61</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="N25" s="6" t="n">
         <v>0</v>
@@ -3221,7 +3221,7 @@
         <v>4300000</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="R25" s="6" t="n">
         <v>500000</v>
@@ -5765,7 +5765,7 @@
         <v>3264000</v>
       </c>
       <c r="M61" s="6" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="N61" s="6" t="n">
         <v>220000</v>
@@ -8552,7 +8552,7 @@
         <v>270000</v>
       </c>
       <c r="S100" s="6" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
         </is>
       </c>
     </row>
@@ -9038,7 +9038,7 @@
         <v>274430273.36</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>5.46</v>
+        <v>5.43</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>266900377</v>
@@ -9103,7 +9103,7 @@
         <v>96854689.95</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>1.93</v>
+        <v>1.92</v>
       </c>
       <c r="L6" s="6" t="n">
         <v>95147634.26000001</v>
@@ -9168,7 +9168,7 @@
         <v>31000000</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>15000000</v>
@@ -9493,7 +9493,7 @@
         <v>9817290</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="L12" s="6" t="n">
         <v>5620170</v>
@@ -9948,7 +9948,7 @@
         <v>6279227</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>4672182.32</v>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
         </is>
       </c>
     </row>
@@ -17316,7 +17316,7 @@
         <v>939338671.25</v>
       </c>
       <c r="E5" s="12" t="n">
-        <v>12.96</v>
+        <v>12.93</v>
       </c>
     </row>
     <row r="6">
@@ -17339,7 +17339,7 @@
         <v>771349229.63</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>10.64</v>
+        <v>10.61</v>
       </c>
     </row>
     <row r="7">
@@ -17362,7 +17362,7 @@
         <v>538365356.08</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>7.43</v>
+        <v>7.41</v>
       </c>
     </row>
     <row r="8">
@@ -17385,7 +17385,7 @@
         <v>500975044.6</v>
       </c>
       <c r="E8" s="12" t="n">
-        <v>6.91</v>
+        <v>6.89</v>
       </c>
     </row>
     <row r="9">
@@ -17408,7 +17408,7 @@
         <v>347379154.28</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>4.79</v>
+        <v>4.78</v>
       </c>
     </row>
     <row r="10">
@@ -17431,7 +17431,7 @@
         <v>346218803.68</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>4.78</v>
+        <v>4.76</v>
       </c>
     </row>
     <row r="11">
@@ -17454,7 +17454,7 @@
         <v>319429268.6</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>4.41</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="12">
@@ -17477,7 +17477,7 @@
         <v>260376041.15</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>3.59</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="13">
@@ -17500,7 +17500,7 @@
         <v>248129335.7</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>3.42</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="14">
@@ -17523,7 +17523,7 @@
         <v>231968669.42</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>3.2</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="15">
@@ -17546,7 +17546,7 @@
         <v>223427397.48</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>3.08</v>
+        <v>3.07</v>
       </c>
     </row>
     <row r="16">
@@ -17569,7 +17569,7 @@
         <v>215953205.16</v>
       </c>
       <c r="E16" s="12" t="n">
-        <v>2.98</v>
+        <v>2.97</v>
       </c>
     </row>
     <row r="17">
@@ -17592,7 +17592,7 @@
         <v>206561665.78</v>
       </c>
       <c r="E17" s="12" t="n">
-        <v>2.85</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="18">
@@ -17615,7 +17615,7 @@
         <v>191413183.8</v>
       </c>
       <c r="E18" s="12" t="n">
-        <v>2.64</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="19">
@@ -17638,7 +17638,7 @@
         <v>189081171.59</v>
       </c>
       <c r="E19" s="12" t="n">
-        <v>2.61</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="20">
@@ -17661,7 +17661,7 @@
         <v>176143006.2</v>
       </c>
       <c r="E20" s="12" t="n">
-        <v>2.43</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="21">
@@ -17684,7 +17684,7 @@
         <v>162298081</v>
       </c>
       <c r="E21" s="12" t="n">
-        <v>2.24</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="22">
@@ -17730,7 +17730,7 @@
         <v>146357084.1</v>
       </c>
       <c r="E23" s="12" t="n">
-        <v>2.02</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="24">
@@ -17776,7 +17776,7 @@
         <v>134640502.61</v>
       </c>
       <c r="E25" s="12" t="n">
-        <v>1.86</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="26">
@@ -17787,19 +17787,19 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Sergipe</t>
+          <t>Rio Grande do Norte</t>
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>122885231.77</v>
+        <v>125207710.92</v>
       </c>
       <c r="E26" s="12" t="n">
-        <v>1.7</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="27">
@@ -17810,19 +17810,19 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Tocantins</t>
+          <t>Sergipe</t>
         </is>
       </c>
       <c r="D27" s="6" t="n">
-        <v>118738334.43</v>
+        <v>122885231.77</v>
       </c>
       <c r="E27" s="12" t="n">
-        <v>1.64</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="28">
@@ -17833,16 +17833,16 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso do Sul</t>
+          <t>Tocantins</t>
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>118100015.06</v>
+        <v>118738334.43</v>
       </c>
       <c r="E28" s="12" t="n">
         <v>1.63</v>
@@ -17856,19 +17856,19 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Alagoas</t>
+          <t>Mato Grosso do Sul</t>
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>116112117.63</v>
+        <v>118100015.06</v>
       </c>
       <c r="E29" s="12" t="n">
-        <v>1.6</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="30">
@@ -17879,16 +17879,16 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Amapá</t>
+          <t>Alagoas</t>
         </is>
       </c>
       <c r="D30" s="6" t="n">
-        <v>116027014.96</v>
+        <v>116112117.63</v>
       </c>
       <c r="E30" s="12" t="n">
         <v>1.6</v>
@@ -17902,19 +17902,19 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Roraima</t>
+          <t>Amapá</t>
         </is>
       </c>
       <c r="D31" s="6" t="n">
-        <v>105896079.13</v>
+        <v>116027014.96</v>
       </c>
       <c r="E31" s="12" t="n">
-        <v>1.46</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="32">
@@ -17925,19 +17925,19 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Norte</t>
+          <t>Roraima</t>
         </is>
       </c>
       <c r="D32" s="6" t="n">
-        <v>104775575.07</v>
+        <v>105896079.13</v>
       </c>
       <c r="E32" s="12" t="n">
-        <v>1.45</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="33">
@@ -17960,7 +17960,7 @@
         <v>148115915.91</v>
       </c>
       <c r="E33" s="12" t="n">
-        <v>23.94</v>
+        <v>23.89</v>
       </c>
     </row>
     <row r="34">
@@ -17983,7 +17983,7 @@
         <v>63540943.62</v>
       </c>
       <c r="E34" s="12" t="n">
-        <v>10.27</v>
+        <v>10.25</v>
       </c>
     </row>
     <row r="35">
@@ -18006,7 +18006,7 @@
         <v>35734691.7</v>
       </c>
       <c r="E35" s="12" t="n">
-        <v>5.78</v>
+        <v>5.76</v>
       </c>
     </row>
     <row r="36">
@@ -18029,7 +18029,7 @@
         <v>31641290.85</v>
       </c>
       <c r="E36" s="12" t="n">
-        <v>5.11</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="37">
@@ -18052,7 +18052,7 @@
         <v>30492838.61</v>
       </c>
       <c r="E37" s="12" t="n">
-        <v>4.93</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="38">
@@ -18075,7 +18075,7 @@
         <v>27973665.98</v>
       </c>
       <c r="E38" s="12" t="n">
-        <v>4.52</v>
+        <v>4.51</v>
       </c>
     </row>
     <row r="39">
@@ -18121,7 +18121,7 @@
         <v>21166735.92</v>
       </c>
       <c r="E40" s="12" t="n">
-        <v>3.42</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="41">
@@ -18144,7 +18144,7 @@
         <v>18058068.75</v>
       </c>
       <c r="E41" s="12" t="n">
-        <v>2.92</v>
+        <v>2.91</v>
       </c>
     </row>
     <row r="42">
@@ -18190,7 +18190,7 @@
         <v>17621238</v>
       </c>
       <c r="E43" s="12" t="n">
-        <v>2.85</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="44">
@@ -18236,7 +18236,7 @@
         <v>16319200.1</v>
       </c>
       <c r="E45" s="12" t="n">
-        <v>2.64</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="46">
@@ -18282,7 +18282,7 @@
         <v>15345139.27</v>
       </c>
       <c r="E47" s="12" t="n">
-        <v>2.48</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="48">
@@ -18420,7 +18420,7 @@
         <v>10240268.05</v>
       </c>
       <c r="E53" s="12" t="n">
-        <v>1.66</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="54">
@@ -18546,19 +18546,19 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Roraima</t>
+          <t>Rio Grande do Norte</t>
         </is>
       </c>
       <c r="D59" s="6" t="n">
-        <v>6569838.31</v>
+        <v>6693216.87</v>
       </c>
       <c r="E59" s="12" t="n">
-        <v>1.06</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="60">
@@ -18569,19 +18569,19 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Norte</t>
+          <t>Roraima</t>
         </is>
       </c>
       <c r="D60" s="6" t="n">
-        <v>5311997.37</v>
+        <v>6569838.31</v>
       </c>
       <c r="E60" s="12" t="n">
-        <v>0.86</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="61">
@@ -18604,7 +18604,7 @@
         <v>621682134.8</v>
       </c>
       <c r="E61" s="12" t="n">
-        <v>11.52</v>
+        <v>11.48</v>
       </c>
     </row>
     <row r="62">
@@ -18627,7 +18627,7 @@
         <v>613298902.3</v>
       </c>
       <c r="E62" s="12" t="n">
-        <v>11.36</v>
+        <v>11.33</v>
       </c>
     </row>
     <row r="63">
@@ -18650,7 +18650,7 @@
         <v>412090448.93</v>
       </c>
       <c r="E63" s="12" t="n">
-        <v>7.63</v>
+        <v>7.61</v>
       </c>
     </row>
     <row r="64">
@@ -18673,7 +18673,7 @@
         <v>375418971.54</v>
       </c>
       <c r="E64" s="12" t="n">
-        <v>6.95</v>
+        <v>6.93</v>
       </c>
     </row>
     <row r="65">
@@ -18696,7 +18696,7 @@
         <v>282735417.37</v>
       </c>
       <c r="E65" s="12" t="n">
-        <v>5.24</v>
+        <v>5.22</v>
       </c>
     </row>
     <row r="66">
@@ -18719,7 +18719,7 @@
         <v>248689457.06</v>
       </c>
       <c r="E66" s="12" t="n">
-        <v>4.61</v>
+        <v>4.59</v>
       </c>
     </row>
     <row r="67">
@@ -18742,7 +18742,7 @@
         <v>237550200.29</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>4.4</v>
+        <v>4.39</v>
       </c>
     </row>
     <row r="68">
@@ -18765,7 +18765,7 @@
         <v>199480839.32</v>
       </c>
       <c r="E68" s="12" t="n">
-        <v>3.7</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="69">
@@ -18788,7 +18788,7 @@
         <v>183040826.39</v>
       </c>
       <c r="E69" s="12" t="n">
-        <v>3.39</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="70">
@@ -18811,7 +18811,7 @@
         <v>172963239.83</v>
       </c>
       <c r="E70" s="12" t="n">
-        <v>3.2</v>
+        <v>3.19</v>
       </c>
     </row>
     <row r="71">
@@ -18834,7 +18834,7 @@
         <v>164184836.19</v>
       </c>
       <c r="E71" s="12" t="n">
-        <v>3.04</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="72">
@@ -18857,7 +18857,7 @@
         <v>154899399.83</v>
       </c>
       <c r="E72" s="12" t="n">
-        <v>2.87</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="73">
@@ -18880,7 +18880,7 @@
         <v>151165278.8</v>
       </c>
       <c r="E73" s="12" t="n">
-        <v>2.8</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="74">
@@ -18903,7 +18903,7 @@
         <v>145779081.5</v>
       </c>
       <c r="E74" s="12" t="n">
-        <v>2.7</v>
+        <v>2.69</v>
       </c>
     </row>
     <row r="75">
@@ -19018,7 +19018,7 @@
         <v>105817480.74</v>
       </c>
       <c r="E79" s="12" t="n">
-        <v>1.96</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="80">
@@ -19029,16 +19029,16 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Piauí</t>
+          <t>Rio Grande do Norte</t>
         </is>
       </c>
       <c r="D80" s="6" t="n">
-        <v>104059277.83</v>
+        <v>104528005.98</v>
       </c>
       <c r="E80" s="12" t="n">
         <v>1.93</v>
@@ -19052,19 +19052,19 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Sergipe</t>
+          <t>Piauí</t>
         </is>
       </c>
       <c r="D81" s="6" t="n">
-        <v>97316118.98</v>
+        <v>104059277.83</v>
       </c>
       <c r="E81" s="12" t="n">
-        <v>1.8</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="82">
@@ -19075,19 +19075,19 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Amapá</t>
+          <t>Sergipe</t>
         </is>
       </c>
       <c r="D82" s="6" t="n">
-        <v>96676722.64</v>
+        <v>97316118.98</v>
       </c>
       <c r="E82" s="12" t="n">
-        <v>1.79</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="83">
@@ -19098,19 +19098,19 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Alagoas</t>
+          <t>Amapá</t>
         </is>
       </c>
       <c r="D83" s="6" t="n">
-        <v>96310229.08</v>
+        <v>96676722.64</v>
       </c>
       <c r="E83" s="12" t="n">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="84">
@@ -19121,19 +19121,19 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Roraima</t>
+          <t>Alagoas</t>
         </is>
       </c>
       <c r="D84" s="6" t="n">
-        <v>92214955.93000001</v>
+        <v>96310229.08</v>
       </c>
       <c r="E84" s="12" t="n">
-        <v>1.71</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="85">
@@ -19144,19 +19144,19 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Norte</t>
+          <t>Roraima</t>
         </is>
       </c>
       <c r="D85" s="6" t="n">
-        <v>89116564.23</v>
+        <v>92214955.93000001</v>
       </c>
       <c r="E85" s="12" t="n">
-        <v>1.65</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="86">
@@ -19179,7 +19179,7 @@
         <v>88384512.84999999</v>
       </c>
       <c r="E86" s="12" t="n">
-        <v>1.64</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="87">
@@ -20536,7 +20536,7 @@
         <v>96577263.26000001</v>
       </c>
       <c r="E145" s="12" t="n">
-        <v>13.84</v>
+        <v>13.82</v>
       </c>
     </row>
     <row r="146">
@@ -20559,7 +20559,7 @@
         <v>79531300.44</v>
       </c>
       <c r="E146" s="12" t="n">
-        <v>11.39</v>
+        <v>11.38</v>
       </c>
     </row>
     <row r="147">
@@ -20582,7 +20582,7 @@
         <v>48942505.72</v>
       </c>
       <c r="E147" s="12" t="n">
-        <v>7.01</v>
+        <v>7</v>
       </c>
     </row>
     <row r="148">
@@ -20628,7 +20628,7 @@
         <v>38085709.47</v>
       </c>
       <c r="E149" s="12" t="n">
-        <v>5.46</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="150">
@@ -20674,7 +20674,7 @@
         <v>34900719.44</v>
       </c>
       <c r="E151" s="12" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="152">
@@ -20697,7 +20697,7 @@
         <v>34253029.36</v>
       </c>
       <c r="E152" s="12" t="n">
-        <v>4.91</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="153">
@@ -20720,7 +20720,7 @@
         <v>26980128.92</v>
       </c>
       <c r="E153" s="12" t="n">
-        <v>3.87</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="154">
@@ -20858,7 +20858,7 @@
         <v>20297773.72</v>
       </c>
       <c r="E159" s="12" t="n">
-        <v>2.91</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="160">
@@ -20927,7 +20927,7 @@
         <v>15534495.24</v>
       </c>
       <c r="E162" s="12" t="n">
-        <v>2.23</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="163">
@@ -21085,10 +21085,10 @@
         </is>
       </c>
       <c r="D169" s="6" t="n">
-        <v>5630860.16</v>
+        <v>6396511.16</v>
       </c>
       <c r="E169" s="12" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="170">
@@ -21249,7 +21249,7 @@
         <v>1224</v>
       </c>
       <c r="E176" s="12" t="n">
-        <v>5.82</v>
+        <v>5.81</v>
       </c>
     </row>
     <row r="177">
@@ -21295,7 +21295,7 @@
         <v>1054</v>
       </c>
       <c r="E178" s="12" t="n">
-        <v>5.01</v>
+        <v>5</v>
       </c>
     </row>
     <row r="179">
@@ -21318,7 +21318,7 @@
         <v>961</v>
       </c>
       <c r="E179" s="12" t="n">
-        <v>4.57</v>
+        <v>4.56</v>
       </c>
     </row>
     <row r="180">
@@ -21410,7 +21410,7 @@
         <v>700</v>
       </c>
       <c r="E183" s="12" t="n">
-        <v>3.33</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="184">
@@ -21729,10 +21729,10 @@
         </is>
       </c>
       <c r="D197" s="6" t="n">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="E197" s="12" t="n">
-        <v>1.57</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="198">
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
         </is>
       </c>
     </row>
@@ -23931,7 +23931,7 @@
         <v>1662</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>7.9</v>
+        <v>7.89</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>5281805806.47</v>
@@ -23940,19 +23940,19 @@
         <v>1405735148.87</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>19.4</v>
+        <v>19.34</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>1023721550.1</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>18.96</v>
+        <v>18.91</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>150890397.42</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>24.39</v>
+        <v>24.33</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>21851884.12</v>
@@ -23974,135 +23974,135 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>5.27</v>
+        <v>5.28</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>788242541.16</v>
+        <v>788542541.16</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>1048828854.66</v>
+        <v>1054100225.91</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>14.47</v>
+        <v>14.51</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>915483382.37</v>
+        <v>918728039.12</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>16.96</v>
+        <v>16.97</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>6064915.15</v>
+        <v>6246134.65</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>0.98</v>
+        <v>1.01</v>
       </c>
       <c r="K6" s="6" t="n">
         <v>12220887.03</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>83634087.52</v>
+        <v>84399738.52</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>692449994.6800001</v>
+        <v>701055413.41</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>87.86</v>
+        <v>87.75</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>PSD</t>
+          <t>UNIÃO</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>1140</v>
+        <v>849</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>5.42</v>
+        <v>4.03</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>2577905190.84</v>
+        <v>1819943318.34</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>654049334.59</v>
+        <v>658108511.73</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>9.029999999999999</v>
+        <v>9.06</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>448626803.71</v>
+        <v>536542994.33</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>8.31</v>
+        <v>9.91</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>34632737.02</v>
+        <v>65276808.97</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>5.6</v>
+        <v>10.53</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>18839446.7</v>
+        <v>8056189.56</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>83964607.95999999</v>
+        <v>29340316.97</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>511180752.93</v>
+        <v>472711959.95</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>73.89</v>
+        <v>91.45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>UNIÃO</t>
+          <t>PSD</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>846</v>
+        <v>1140</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>4.02</v>
+        <v>5.41</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1817696708.82</v>
+        <v>2577905190.84</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>642947747.13</v>
+        <v>654049334.59</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>8.869999999999999</v>
+        <v>9</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>524376209.33</v>
+        <v>448626803.71</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>9.710000000000001</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>64076808.97</v>
+        <v>34632737.02</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>10.36</v>
+        <v>5.59</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>7912189.56</v>
+        <v>18839446.7</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>29340316.97</v>
+        <v>83964607.95999999</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>452806297.25</v>
+        <v>511180752.93</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>91.52</v>
+        <v>73.89</v>
       </c>
     </row>
     <row r="9">
@@ -24115,7 +24115,7 @@
         <v>1321</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>6.28</v>
+        <v>6.27</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>2779509683.8</v>
@@ -24124,19 +24124,19 @@
         <v>604229188.12</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>8.34</v>
+        <v>8.31</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>370429872.29</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>6.86</v>
+        <v>6.84</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>126534864</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>20.45</v>
+        <v>20.41</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>11619412.8</v>
@@ -24170,19 +24170,19 @@
         <v>576017200.2</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>7.95</v>
+        <v>7.93</v>
       </c>
       <c r="G10" s="6" t="n">
         <v>446416289.17</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>8.27</v>
+        <v>8.25</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>74186678.76000001</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>11.99</v>
+        <v>11.96</v>
       </c>
       <c r="K10" s="6" t="n">
         <v>7762845.27</v>
@@ -24204,31 +24204,31 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1426</v>
+        <v>1429</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>6.77</v>
+        <v>6.79</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>3426703758.32</v>
+        <v>3431895006.71</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>536133443.18</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>7.4</v>
+        <v>7.38</v>
       </c>
       <c r="G11" s="6" t="n">
         <v>407807248.96</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>7.55</v>
+        <v>7.53</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>17628836.54</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>2.85</v>
+        <v>2.84</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>14746735.62</v>
@@ -24253,7 +24253,7 @@
         <v>1237</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>5.88</v>
+        <v>5.87</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>1812875005.9</v>
@@ -24262,13 +24262,13 @@
         <v>295199071.52</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>4.07</v>
+        <v>4.06</v>
       </c>
       <c r="G12" s="6" t="n">
         <v>237965482.3</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>4.41</v>
+        <v>4.4</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>5640256.810000001</v>
@@ -24308,19 +24308,19 @@
         <v>229740786.52</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>3.17</v>
+        <v>3.16</v>
       </c>
       <c r="G13" s="6" t="n">
         <v>166995631.66</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>3.09</v>
+        <v>3.08</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>46290560.08</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>7.48</v>
+        <v>7.47</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>2903506.06</v>
@@ -24342,25 +24342,25 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>968</v>
+        <v>971</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>4.6</v>
+        <v>4.61</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>941267717.34</v>
+        <v>941728196.61</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>222285982.7</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>3.07</v>
+        <v>3.06</v>
       </c>
       <c r="G14" s="6" t="n">
         <v>148455951.38</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>2.75</v>
+        <v>2.74</v>
       </c>
       <c r="I14" s="6" t="n">
         <v>6709805.88</v>
@@ -24391,7 +24391,7 @@
         <v>1094</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>5.2</v>
+        <v>5.19</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>2591694177.84</v>
@@ -24400,7 +24400,7 @@
         <v>209562747.69</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>2.89</v>
+        <v>2.88</v>
       </c>
       <c r="G15" s="6" t="n">
         <v>150291927.09</v>
@@ -24446,7 +24446,7 @@
         <v>144146207.42</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>1.99</v>
+        <v>1.98</v>
       </c>
       <c r="G16" s="6" t="n">
         <v>34396229.06</v>
@@ -24458,7 +24458,7 @@
         <v>44449677.11</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>7.18</v>
+        <v>7.17</v>
       </c>
       <c r="K16" s="6" t="n">
         <v>7309289.36</v>
@@ -24467,7 +24467,7 @@
         <v>27042953.19</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>88921572.93000001</v>
+        <v>88921572.92999999</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>54.7</v>
@@ -24483,7 +24483,7 @@
         <v>799</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>3.8</v>
+        <v>3.79</v>
       </c>
       <c r="D17" s="6" t="n">
         <v>139488473.87</v>
@@ -24492,13 +24492,13 @@
         <v>135333277.13</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>1.87</v>
+        <v>1.86</v>
       </c>
       <c r="G17" s="6" t="n">
         <v>123925665.62</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>2.3</v>
+        <v>2.29</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>1959373.78</v>
@@ -24529,7 +24529,7 @@
         <v>980</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>4.66</v>
+        <v>4.65</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>1072776812.99</v>
@@ -24596,7 +24596,7 @@
         <v>14150615.09</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>2.29</v>
+        <v>2.28</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>3349975.82</v>
@@ -24713,7 +24713,7 @@
         <v>239</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="D22" s="6" t="n">
         <v>330099422.77</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 09:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
         </is>
       </c>
     </row>
@@ -28228,7 +28228,7 @@
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>Nota 2: outras 4171 candidaturas NAO declararam receita alguma, das quais 954 sao vice ou suplente, que nao prestam conta propria. Ausencia de declaracao nao e' autofinanciamento, e por isso elas ficam fora desta tabela.</t>
+          <t>Nota 2: outras 4177 candidaturas NAO declararam receita alguma, das quais 960 sao vice ou suplente, que nao prestam conta propria. Ausencia de declaracao nao e' autofinanciamento, e por isso elas ficam fora desta tabela.</t>
         </is>
       </c>
     </row>
@@ -29059,7 +29059,7 @@
         <v>76.81999999999999</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="G21" s="5" t="n">
         <v>40</v>
@@ -29068,19 +29068,19 @@
         <v>66524</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>12.4</v>
+        <v>12.85</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>104775575.07</v>
+        <v>125207710.92</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>30.25</v>
+        <v>36.15</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>39.38</v>
+        <v>47.05</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>35.49</v>
+        <v>41.8</v>
       </c>
     </row>
     <row r="22">
@@ -29593,7 +29593,7 @@
         <v>73.69</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>21049</v>
+        <v>21061</v>
       </c>
       <c r="G33" s="8" t="n">
         <v>1790</v>
@@ -29605,16 +29605,16 @@
         <v>13.34</v>
       </c>
       <c r="J33" s="9" t="n">
-        <v>7246570798.1</v>
+        <v>7267002933.950001</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>33.83</v>
+        <v>33.92</v>
       </c>
       <c r="L33" s="9" t="n">
-        <v>45.91</v>
+        <v>46.04</v>
       </c>
       <c r="M33" s="9" t="n">
-        <v>38.12</v>
+        <v>38.23</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 10/10/2026 15:40
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-10 15:03:15</t>
+          <t>2026-10-10 15:32:40</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:03:15.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 10/10/2026 21:11
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>6737183</v>
+        <v>6736268</v>
       </c>
     </row>
     <row r="61">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-10 15:32:40</t>
+          <t>2026-10-10 21:03:37</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
         </is>
       </c>
     </row>
@@ -24467,7 +24467,7 @@
         <v>27042953.19</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>88921572.92999999</v>
+        <v>88921572.93000001</v>
       </c>
       <c r="N16" s="6" t="n">
         <v>54.7</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 15:32:40.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 11/10/2026 03:10
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 03:02:32.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 03:02:32.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-10 21:03:37</t>
+          <t>2026-10-11 03:02:32</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 03:02:32.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 03:02:32.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 03:02:32.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 03:02:32.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 03:02:32.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 03:02:32.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-10 21:03:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 03:02:32.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 11/10/2026 15:10
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 09:04:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 09:04:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>172</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-11 09:04:27</t>
+          <t>2026-10-11 15:03:10</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.9499999</v>
+        <v>575680870.95</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.75</v>
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="G65" s="6" t="n">
-        <v>58445503.79</v>
+        <v>58445503.79000001</v>
       </c>
       <c r="H65" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 09:04:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 09:04:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 09:04:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 09:04:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 09:04:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
         </is>
       </c>
     </row>
@@ -24271,7 +24271,7 @@
         <v>4.39</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5664780.810000001</v>
+        <v>5664780.81</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>0.91</v>
@@ -24927,7 +24927,7 @@
         <v>5498396.57</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>8287319.060000001</v>
+        <v>8287319.06</v>
       </c>
       <c r="N26" s="6" t="n">
         <v>23.06</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 09:04:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 09:04:27.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 11/10/2026 21:12
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-11 15:03:10</t>
+          <t>2026-10-11 21:04:53</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.95</v>
+        <v>575680870.9499999</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.75</v>
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="G65" s="6" t="n">
-        <v>58445503.79000001</v>
+        <v>58445503.79</v>
       </c>
       <c r="H65" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
         </is>
       </c>
     </row>
@@ -24271,7 +24271,7 @@
         <v>4.39</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5664780.81</v>
+        <v>5664780.810000001</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>0.91</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 15:03:10.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 12/10/2026 03:11
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-11 21:04:53</t>
+          <t>2026-10-12 03:02:46</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-11 21:04:53.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 12/10/2026 09:11
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-12 03:02:46</t>
+          <t>2026-10-12 09:03:29</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 03:02:46.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 12/10/2026 15:11
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-12 09:03:29</t>
+          <t>2026-10-12 15:03:07</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 09:03:29.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 12/10/2026 21:10
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-12 15:03:07</t>
+          <t>2026-10-12 21:03:04</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 15:03:07.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 13/10/2026 03:11
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-12 21:03:04</t>
+          <t>2026-10-13 03:02:52</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-12 21:03:04.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 13/10/2026 09:37
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 09:13:47.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 09:13:47.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-13 03:02:52</t>
+          <t>2026-10-13 09:13:47</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 09:13:47.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 09:13:47.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 09:13:47.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 09:13:47.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 09:13:47.</t>
         </is>
       </c>
     </row>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 09:13:47.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 03:02:52.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-13 09:13:47.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 14/10/2026 22:19
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 09:12:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 16:19:51.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 09:12:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 16:19:51.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>526</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-14 09:12:37</t>
+          <t>2026-10-14 16:19:51</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 09:12:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 16:19:51.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 09:12:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 16:19:51.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 09:12:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 16:19:51.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 09:12:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 16:19:51.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 09:12:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 16:19:51.</t>
         </is>
       </c>
     </row>
@@ -24271,7 +24271,7 @@
         <v>4.4</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5680836.81</v>
+        <v>5680836.810000001</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>0.9</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 09:12:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 16:19:51.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 09:12:37.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-14 16:19:51.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 15/10/2026 15:14
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -581,7 +581,7 @@
         <v>4495080252.41</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>13.66</v>
+        <v>13.64</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>0</v>
@@ -612,7 +612,7 @@
         <v>923439500.0599999</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>2.81</v>
+        <v>2.8</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>0</v>
@@ -637,7 +637,7 @@
         <v>433</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>2.06</v>
+        <v>2.05</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>338296381.14</v>
@@ -649,13 +649,13 @@
         <v>47902742.53</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>33142536.24</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="8">
@@ -668,25 +668,25 @@
         <v>11295</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>53.63</v>
+        <v>53.6</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>12007434756.34</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>36.5</v>
+        <v>36.43</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>1795036958.61</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>24.56</v>
+        <v>24.41</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>1185992166.35</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>23.17</v>
+        <v>23.03</v>
       </c>
     </row>
     <row r="9">
@@ -699,25 +699,25 @@
         <v>7803</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>37.05</v>
+        <v>37.03</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>8707767692.280001</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>26.47</v>
+        <v>26.42</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>3405144473.64</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>46.59</v>
+        <v>46.31</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>2300421308.43</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>44.94</v>
+        <v>44.67</v>
       </c>
     </row>
     <row r="10">
@@ -727,28 +727,28 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>1.1</v>
+        <v>1.12</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1755573651.78</v>
+        <v>1774582066.62</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.34</v>
+        <v>5.38</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>764441395.64</v>
+        <v>807767933.9299999</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>10.46</v>
+        <v>10.99</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>622010881.96</v>
+        <v>653491781.3200001</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>12.15</v>
+        <v>12.69</v>
       </c>
     </row>
     <row r="11">
@@ -767,19 +767,19 @@
         <v>1223996865.97</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>3.72</v>
+        <v>3.71</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>777520950.2900001</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>10.64</v>
+        <v>10.57</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>587347887.3099999</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>11.47</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="12">
@@ -798,19 +798,19 @@
         <v>2079741446.05</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>6.32</v>
+        <v>6.31</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>519238923.51</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>7.1</v>
+        <v>7.06</v>
       </c>
       <c r="H12" s="6" t="n">
         <v>389674253.59</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>7.61</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="13">
@@ -820,16 +820,16 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>1.14</v>
+        <v>1.17</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>791514463.25</v>
+        <v>834903841.25</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>2.41</v>
+        <v>2.53</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>0</v>
@@ -882,25 +882,25 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>21061</v>
+        <v>21073</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32898582945.04</v>
+        <v>32960980737.88</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>7309285444.219999</v>
+        <v>7352611982.51</v>
       </c>
       <c r="G15" s="9" t="n">
         <v>100</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>5118589033.88</v>
+        <v>5150069933.24</v>
       </c>
       <c r="I15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 09:44:30.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 15:05:24.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 09:44:30.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 15:05:24.</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>21013</v>
+        <v>21017</v>
       </c>
     </row>
     <row r="14">
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21013</v>
+        <v>21017</v>
       </c>
     </row>
     <row r="16">
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>21058</v>
+        <v>21070</v>
       </c>
     </row>
     <row r="19">
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>183</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22">
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>295</v>
+        <v>311</v>
       </c>
     </row>
     <row r="23">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>56603</v>
+        <v>56604</v>
       </c>
     </row>
     <row r="48">
@@ -1414,7 +1414,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="50">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-15 09:44:30</t>
+          <t>2026-10-15 15:05:24</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>-724835644.71</v>
+        <v>-768162183</v>
       </c>
     </row>
     <row r="65">
@@ -1772,7 +1772,7 @@
         <v>1226983360</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>3.73</v>
+        <v>3.72</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>4</v>
@@ -1914,7 +1914,7 @@
         <v>650405604.49</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>1.98</v>
+        <v>1.97</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>15</v>
@@ -2073,7 +2073,7 @@
         <v>7713744.35</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>678014</v>
@@ -2085,7 +2085,7 @@
         <v>1000000</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>3000000</v>
@@ -2127,7 +2127,7 @@
         <v>548600000</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>1.67</v>
+        <v>1.66</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>3</v>
@@ -2269,7 +2269,7 @@
         <v>495224296</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>1.51</v>
+        <v>1.5</v>
       </c>
       <c r="I12" s="5" t="n">
         <v>7</v>
@@ -2482,7 +2482,7 @@
         <v>478688485.93</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>1.46</v>
+        <v>1.45</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>58</v>
@@ -2553,7 +2553,7 @@
         <v>400000000</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>1.22</v>
+        <v>1.21</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>3</v>
@@ -3008,7 +3008,7 @@
         <v>1744850.78</v>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="R22" s="6" t="n">
         <v>1230953.08</v>
@@ -3221,7 +3221,7 @@
         <v>4300000</v>
       </c>
       <c r="Q25" s="6" t="n">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="R25" s="6" t="n">
         <v>500000</v>
@@ -4044,7 +4044,7 @@
         <v>107108276.43</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="I37" s="5" t="n">
         <v>22</v>
@@ -4186,7 +4186,7 @@
         <v>103733556.02</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="I39" s="5" t="n">
         <v>146</v>
@@ -4647,7 +4647,7 @@
         <v>16008194.03</v>
       </c>
       <c r="S45" s="6" t="n">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="46">
@@ -5251,7 +5251,7 @@
         <v>67500000</v>
       </c>
       <c r="H54" s="6" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="I54" s="5" t="n">
         <v>5</v>
@@ -5606,7 +5606,7 @@
         <v>64220956.82</v>
       </c>
       <c r="H59" s="6" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="I59" s="5" t="n">
         <v>35</v>
@@ -6274,7 +6274,7 @@
         <v>611286.47</v>
       </c>
       <c r="Q68" s="6" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="R68" s="6" t="n">
         <v>800000</v>
@@ -6558,7 +6558,7 @@
         <v>1499763</v>
       </c>
       <c r="Q72" s="6" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="R72" s="6" t="n">
         <v>0</v>
@@ -6600,7 +6600,7 @@
         <v>51000000</v>
       </c>
       <c r="H73" s="6" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="I73" s="5" t="n">
         <v>8</v>
@@ -7339,7 +7339,7 @@
         <v>2396323.01</v>
       </c>
       <c r="Q83" s="6" t="n">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="R83" s="6" t="n">
         <v>0</v>
@@ -8049,7 +8049,7 @@
         <v>95000</v>
       </c>
       <c r="Q93" s="6" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="R93" s="6" t="n">
         <v>2507629.39</v>
@@ -8659,7 +8659,7 @@
         <v>44497052.1</v>
       </c>
       <c r="H102" s="6" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="I102" s="5" t="n">
         <v>45</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 09:44:30.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 15:05:24.</t>
         </is>
       </c>
     </row>
@@ -9038,7 +9038,7 @@
         <v>281516195.39</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>5.5</v>
+        <v>5.47</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>274070810.41</v>
@@ -9103,7 +9103,7 @@
         <v>99805530.3</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>1.95</v>
+        <v>1.94</v>
       </c>
       <c r="L6" s="6" t="n">
         <v>98296574.61</v>
@@ -9168,7 +9168,7 @@
         <v>31000000</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>0.61</v>
+        <v>0.6</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>15000000</v>
@@ -10273,7 +10273,7 @@
         <v>5400000</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="L24" s="6" t="n">
         <v>3600000</v>
@@ -10468,7 +10468,7 @@
         <v>4866473.9</v>
       </c>
       <c r="K27" s="6" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="L27" s="6" t="n">
         <v>3925144.9</v>
@@ -12483,7 +12483,7 @@
         <v>3345250.5</v>
       </c>
       <c r="K58" s="6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="L58" s="6" t="n">
         <v>2472030</v>
@@ -12548,7 +12548,7 @@
         <v>3343294.16</v>
       </c>
       <c r="K59" s="6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="L59" s="6" t="n">
         <v>2233258.46</v>
@@ -12613,7 +12613,7 @@
         <v>3334759.25</v>
       </c>
       <c r="K60" s="6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="L60" s="6" t="n">
         <v>2131410</v>
@@ -15408,7 +15408,7 @@
         <v>2304363.37</v>
       </c>
       <c r="K103" s="6" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="L103" s="6" t="n">
         <v>1820773.33</v>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 09:44:30.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 15:05:24.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 09:44:30.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 15:05:24.</t>
         </is>
       </c>
     </row>
@@ -17316,7 +17316,7 @@
         <v>941863602.37</v>
       </c>
       <c r="E5" s="12" t="n">
-        <v>12.89</v>
+        <v>12.81</v>
       </c>
     </row>
     <row r="6">
@@ -17339,7 +17339,7 @@
         <v>777520950.29</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>10.64</v>
+        <v>10.57</v>
       </c>
     </row>
     <row r="7">
@@ -17362,7 +17362,7 @@
         <v>540734381.52</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>7.4</v>
+        <v>7.35</v>
       </c>
     </row>
     <row r="8">
@@ -17385,7 +17385,7 @@
         <v>501949079.58</v>
       </c>
       <c r="E8" s="12" t="n">
-        <v>6.87</v>
+        <v>6.83</v>
       </c>
     </row>
     <row r="9">
@@ -17408,7 +17408,7 @@
         <v>348809893.96</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>4.77</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="10">
@@ -17431,7 +17431,7 @@
         <v>348269323.09</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>4.76</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="11">
@@ -17454,7 +17454,7 @@
         <v>320180921.52</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>4.38</v>
+        <v>4.35</v>
       </c>
     </row>
     <row r="12">
@@ -17477,7 +17477,7 @@
         <v>260758408.08</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>3.57</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="13">
@@ -17500,7 +17500,7 @@
         <v>248829183.34</v>
       </c>
       <c r="E13" s="12" t="n">
-        <v>3.4</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="14">
@@ -17523,7 +17523,7 @@
         <v>233931458.5</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>3.2</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="15">
@@ -17546,7 +17546,7 @@
         <v>224083484.48</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>3.07</v>
+        <v>3.05</v>
       </c>
     </row>
     <row r="16">
@@ -17569,7 +17569,7 @@
         <v>217166956.08</v>
       </c>
       <c r="E16" s="12" t="n">
-        <v>2.97</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="17">
@@ -17592,7 +17592,7 @@
         <v>206920736.24</v>
       </c>
       <c r="E17" s="12" t="n">
-        <v>2.83</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="18">
@@ -17615,7 +17615,7 @@
         <v>192361636.49</v>
       </c>
       <c r="E18" s="12" t="n">
-        <v>2.63</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="19">
@@ -17638,7 +17638,7 @@
         <v>189655533.43</v>
       </c>
       <c r="E19" s="12" t="n">
-        <v>2.59</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="20">
@@ -17661,7 +17661,7 @@
         <v>176872010.23</v>
       </c>
       <c r="E20" s="12" t="n">
-        <v>2.42</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="21">
@@ -17672,19 +17672,19 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso</t>
+          <t>Tocantins</t>
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>163121695.8</v>
+        <v>164723028.18</v>
       </c>
       <c r="E21" s="12" t="n">
-        <v>2.23</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="22">
@@ -17695,19 +17695,19 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Paraíba</t>
+          <t>Mato Grosso</t>
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>149765818.85</v>
+        <v>163121695.8</v>
       </c>
       <c r="E22" s="12" t="n">
-        <v>2.05</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="23">
@@ -17718,19 +17718,19 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Rondônia</t>
+          <t>Paraíba</t>
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>147279582.87</v>
+        <v>149765818.85</v>
       </c>
       <c r="E23" s="12" t="n">
-        <v>2.01</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="24">
@@ -17741,19 +17741,19 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Piauí</t>
+          <t>Rondônia</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>145500892.28</v>
+        <v>147279582.87</v>
       </c>
       <c r="E24" s="12" t="n">
-        <v>1.99</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -17764,19 +17764,19 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Norte</t>
+          <t>Piauí</t>
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>136913290.09</v>
+        <v>145500892.28</v>
       </c>
       <c r="E25" s="12" t="n">
-        <v>1.87</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="26">
@@ -17787,19 +17787,19 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Acre</t>
+          <t>Rio Grande do Norte</t>
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>134882233.11</v>
+        <v>136913290.09</v>
       </c>
       <c r="E26" s="12" t="n">
-        <v>1.85</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="27">
@@ -17810,19 +17810,19 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Sergipe</t>
+          <t>Acre</t>
         </is>
       </c>
       <c r="D27" s="6" t="n">
-        <v>123217657.01</v>
+        <v>134882233.11</v>
       </c>
       <c r="E27" s="12" t="n">
-        <v>1.69</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="28">
@@ -17833,19 +17833,19 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Tocantins</t>
+          <t>Sergipe</t>
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>121396489.89</v>
+        <v>123217657.01</v>
       </c>
       <c r="E28" s="12" t="n">
-        <v>1.66</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="29">
@@ -17868,7 +17868,7 @@
         <v>118199043.81</v>
       </c>
       <c r="E29" s="12" t="n">
-        <v>1.62</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="30">
@@ -17891,7 +17891,7 @@
         <v>116947052.84</v>
       </c>
       <c r="E30" s="12" t="n">
-        <v>1.6</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="31">
@@ -17914,7 +17914,7 @@
         <v>116160099.96</v>
       </c>
       <c r="E31" s="12" t="n">
-        <v>1.59</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="32">
@@ -17937,7 +17937,7 @@
         <v>105994028.51</v>
       </c>
       <c r="E32" s="12" t="n">
-        <v>1.45</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="33">
@@ -17960,7 +17960,7 @@
         <v>148152716.75</v>
       </c>
       <c r="E33" s="12" t="n">
-        <v>23.44</v>
+        <v>22.93</v>
       </c>
     </row>
     <row r="34">
@@ -17983,7 +17983,7 @@
         <v>63540943.62</v>
       </c>
       <c r="E34" s="12" t="n">
-        <v>10.05</v>
+        <v>9.83</v>
       </c>
     </row>
     <row r="35">
@@ -18006,7 +18006,7 @@
         <v>35779143.44</v>
       </c>
       <c r="E35" s="12" t="n">
-        <v>5.66</v>
+        <v>5.54</v>
       </c>
     </row>
     <row r="36">
@@ -18029,7 +18029,7 @@
         <v>32389921.59</v>
       </c>
       <c r="E36" s="12" t="n">
-        <v>5.12</v>
+        <v>5.01</v>
       </c>
     </row>
     <row r="37">
@@ -18052,7 +18052,7 @@
         <v>30508223.61</v>
       </c>
       <c r="E37" s="12" t="n">
-        <v>4.83</v>
+        <v>4.72</v>
       </c>
     </row>
     <row r="38">
@@ -18063,19 +18063,19 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Rio de Janeiro</t>
+          <t>Tocantins</t>
         </is>
       </c>
       <c r="D38" s="6" t="n">
-        <v>27996415.41</v>
+        <v>28980195.23</v>
       </c>
       <c r="E38" s="12" t="n">
-        <v>4.43</v>
+        <v>4.49</v>
       </c>
     </row>
     <row r="39">
@@ -18086,19 +18086,19 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Rio de Janeiro</t>
         </is>
       </c>
       <c r="D39" s="6" t="n">
-        <v>22120475.07</v>
+        <v>27996415.41</v>
       </c>
       <c r="E39" s="12" t="n">
-        <v>3.5</v>
+        <v>4.33</v>
       </c>
     </row>
     <row r="40">
@@ -18109,19 +18109,19 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Pernambuco</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="D40" s="6" t="n">
-        <v>21168199.92</v>
+        <v>22120475.07</v>
       </c>
       <c r="E40" s="12" t="n">
-        <v>3.35</v>
+        <v>3.42</v>
       </c>
     </row>
     <row r="41">
@@ -18132,19 +18132,19 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Sul</t>
+          <t>Pernambuco</t>
         </is>
       </c>
       <c r="D41" s="6" t="n">
-        <v>18088163.75</v>
+        <v>21168199.92</v>
       </c>
       <c r="E41" s="12" t="n">
-        <v>2.86</v>
+        <v>3.28</v>
       </c>
     </row>
     <row r="42">
@@ -18155,19 +18155,19 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Santa Catarina</t>
+          <t>Rio Grande do Sul</t>
         </is>
       </c>
       <c r="D42" s="6" t="n">
-        <v>17842960.01</v>
+        <v>18088163.75</v>
       </c>
       <c r="E42" s="12" t="n">
-        <v>2.82</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="43">
@@ -18178,19 +18178,19 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Espírito Santo</t>
+          <t>Santa Catarina</t>
         </is>
       </c>
       <c r="D43" s="6" t="n">
-        <v>17644336</v>
+        <v>17842960.01</v>
       </c>
       <c r="E43" s="12" t="n">
-        <v>2.79</v>
+        <v>2.76</v>
       </c>
     </row>
     <row r="44">
@@ -18201,19 +18201,19 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Ceará</t>
+          <t>Espírito Santo</t>
         </is>
       </c>
       <c r="D44" s="6" t="n">
-        <v>17151108.64</v>
+        <v>17644336</v>
       </c>
       <c r="E44" s="12" t="n">
-        <v>2.71</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="45">
@@ -18224,19 +18224,19 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Maranhão</t>
+          <t>Ceará</t>
         </is>
       </c>
       <c r="D45" s="6" t="n">
-        <v>16469200.1</v>
+        <v>17151108.64</v>
       </c>
       <c r="E45" s="12" t="n">
-        <v>2.61</v>
+        <v>2.65</v>
       </c>
     </row>
     <row r="46">
@@ -18247,19 +18247,19 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Acre</t>
+          <t>Maranhão</t>
         </is>
       </c>
       <c r="D46" s="6" t="n">
-        <v>15904796.74</v>
+        <v>16469200.1</v>
       </c>
       <c r="E46" s="12" t="n">
-        <v>2.52</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="47">
@@ -18270,19 +18270,19 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Piauí</t>
+          <t>Acre</t>
         </is>
       </c>
       <c r="D47" s="6" t="n">
-        <v>15345139.27</v>
+        <v>15904796.74</v>
       </c>
       <c r="E47" s="12" t="n">
-        <v>2.43</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="48">
@@ -18293,19 +18293,19 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Tocantins</t>
+          <t>Piauí</t>
         </is>
       </c>
       <c r="D48" s="6" t="n">
-        <v>14904755.93</v>
+        <v>15345139.27</v>
       </c>
       <c r="E48" s="12" t="n">
-        <v>2.36</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="49">
@@ -18328,7 +18328,7 @@
         <v>14693216.87</v>
       </c>
       <c r="E49" s="12" t="n">
-        <v>2.32</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="50">
@@ -18351,7 +18351,7 @@
         <v>12945672.35</v>
       </c>
       <c r="E50" s="12" t="n">
-        <v>2.05</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
@@ -18374,7 +18374,7 @@
         <v>12136324.21</v>
       </c>
       <c r="E51" s="12" t="n">
-        <v>1.92</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="52">
@@ -18397,7 +18397,7 @@
         <v>11715177.76</v>
       </c>
       <c r="E52" s="12" t="n">
-        <v>1.85</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="53">
@@ -18420,7 +18420,7 @@
         <v>10741115.61</v>
       </c>
       <c r="E53" s="12" t="n">
-        <v>1.7</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="54">
@@ -18443,7 +18443,7 @@
         <v>10241492.54</v>
       </c>
       <c r="E54" s="12" t="n">
-        <v>1.62</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="55">
@@ -18466,7 +18466,7 @@
         <v>8226531.29</v>
       </c>
       <c r="E55" s="12" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="56">
@@ -18489,7 +18489,7 @@
         <v>7868672.31</v>
       </c>
       <c r="E56" s="12" t="n">
-        <v>1.24</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="57">
@@ -18512,7 +18512,7 @@
         <v>7668205.73</v>
       </c>
       <c r="E57" s="12" t="n">
-        <v>1.21</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="58">
@@ -18535,7 +18535,7 @@
         <v>7286528.8</v>
       </c>
       <c r="E58" s="12" t="n">
-        <v>1.15</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="59">
@@ -18558,7 +18558,7 @@
         <v>6936280.45</v>
       </c>
       <c r="E59" s="12" t="n">
-        <v>1.1</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="60">
@@ -18581,7 +18581,7 @@
         <v>6559838.31</v>
       </c>
       <c r="E60" s="12" t="n">
-        <v>1.04</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="61">
@@ -18604,7 +18604,7 @@
         <v>622281029.6</v>
       </c>
       <c r="E61" s="12" t="n">
-        <v>11.48</v>
+        <v>11.43</v>
       </c>
     </row>
     <row r="62">
@@ -18627,7 +18627,7 @@
         <v>613298902.3</v>
       </c>
       <c r="E62" s="12" t="n">
-        <v>11.31</v>
+        <v>11.26</v>
       </c>
     </row>
     <row r="63">
@@ -18650,7 +18650,7 @@
         <v>412265001.24</v>
       </c>
       <c r="E63" s="12" t="n">
-        <v>7.61</v>
+        <v>7.57</v>
       </c>
     </row>
     <row r="64">
@@ -18673,7 +18673,7 @@
         <v>375702323.79</v>
       </c>
       <c r="E64" s="12" t="n">
-        <v>6.93</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="65">
@@ -18696,7 +18696,7 @@
         <v>282920761.37</v>
       </c>
       <c r="E65" s="12" t="n">
-        <v>5.22</v>
+        <v>5.19</v>
       </c>
     </row>
     <row r="66">
@@ -18719,7 +18719,7 @@
         <v>248720457.06</v>
       </c>
       <c r="E66" s="12" t="n">
-        <v>4.59</v>
+        <v>4.57</v>
       </c>
     </row>
     <row r="67">
@@ -18742,7 +18742,7 @@
         <v>238190400.29</v>
       </c>
       <c r="E67" s="12" t="n">
-        <v>4.39</v>
+        <v>4.37</v>
       </c>
     </row>
     <row r="68">
@@ -18765,7 +18765,7 @@
         <v>199545419.32</v>
       </c>
       <c r="E68" s="12" t="n">
-        <v>3.68</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="69">
@@ -18788,7 +18788,7 @@
         <v>183040826.39</v>
       </c>
       <c r="E69" s="12" t="n">
-        <v>3.38</v>
+        <v>3.36</v>
       </c>
     </row>
     <row r="70">
@@ -18811,7 +18811,7 @@
         <v>173113239.83</v>
       </c>
       <c r="E70" s="12" t="n">
-        <v>3.19</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="71">
@@ -18834,7 +18834,7 @@
         <v>164218808.19</v>
       </c>
       <c r="E71" s="12" t="n">
-        <v>3.03</v>
+        <v>3.02</v>
       </c>
     </row>
     <row r="72">
@@ -18857,7 +18857,7 @@
         <v>154899399.83</v>
       </c>
       <c r="E72" s="12" t="n">
-        <v>2.86</v>
+        <v>2.84</v>
       </c>
     </row>
     <row r="73">
@@ -18880,7 +18880,7 @@
         <v>151175278.8</v>
       </c>
       <c r="E73" s="12" t="n">
-        <v>2.79</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="74">
@@ -18903,7 +18903,7 @@
         <v>145738001.5</v>
       </c>
       <c r="E74" s="12" t="n">
-        <v>2.69</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="75">
@@ -18926,7 +18926,7 @@
         <v>134563486.7</v>
       </c>
       <c r="E75" s="12" t="n">
-        <v>2.48</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="76">
@@ -18949,7 +18949,7 @@
         <v>127872892.47</v>
       </c>
       <c r="E76" s="12" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="77">
@@ -18972,7 +18972,7 @@
         <v>122216962.45</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>2.25</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="78">
@@ -18983,19 +18983,19 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>TO</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Acre</t>
+          <t>Tocantins</t>
         </is>
       </c>
       <c r="D78" s="6" t="n">
-        <v>108586825.06</v>
+        <v>110836787.34</v>
       </c>
       <c r="E78" s="12" t="n">
-        <v>2</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="79">
@@ -19006,16 +19006,16 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Rio Grande do Norte</t>
+          <t>Acre</t>
         </is>
       </c>
       <c r="D79" s="6" t="n">
-        <v>107735283.55</v>
+        <v>108586825.06</v>
       </c>
       <c r="E79" s="12" t="n">
         <v>1.99</v>
@@ -19029,19 +19029,19 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Rondônia</t>
+          <t>Rio Grande do Norte</t>
         </is>
       </c>
       <c r="D80" s="6" t="n">
-        <v>106467480.73</v>
+        <v>107735283.55</v>
       </c>
       <c r="E80" s="12" t="n">
-        <v>1.96</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="81">
@@ -19052,19 +19052,19 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Piauí</t>
+          <t>Rondônia</t>
         </is>
       </c>
       <c r="D81" s="6" t="n">
-        <v>104059277.83</v>
+        <v>106467480.73</v>
       </c>
       <c r="E81" s="12" t="n">
-        <v>1.92</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="82">
@@ -19075,19 +19075,19 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Sergipe</t>
+          <t>Piauí</t>
         </is>
       </c>
       <c r="D82" s="6" t="n">
-        <v>97316118.98</v>
+        <v>104059277.83</v>
       </c>
       <c r="E82" s="12" t="n">
-        <v>1.8</v>
+        <v>1.91</v>
       </c>
     </row>
     <row r="83">
@@ -19098,19 +19098,19 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Amapá</t>
+          <t>Sergipe</t>
         </is>
       </c>
       <c r="D83" s="6" t="n">
-        <v>96676722.64</v>
+        <v>97316118.98</v>
       </c>
       <c r="E83" s="12" t="n">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="84">
@@ -19121,16 +19121,16 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Alagoas</t>
+          <t>Amapá</t>
         </is>
       </c>
       <c r="D84" s="6" t="n">
-        <v>96310229.08</v>
+        <v>96676722.64</v>
       </c>
       <c r="E84" s="12" t="n">
         <v>1.78</v>
@@ -19144,19 +19144,19 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Roraima</t>
+          <t>Alagoas</t>
         </is>
       </c>
       <c r="D85" s="6" t="n">
-        <v>92302455.93000001</v>
+        <v>96310229.08</v>
       </c>
       <c r="E85" s="12" t="n">
-        <v>1.7</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="86">
@@ -19167,19 +19167,19 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso</t>
+          <t>Roraima</t>
         </is>
       </c>
       <c r="D86" s="6" t="n">
-        <v>88414512.84999999</v>
+        <v>92302455.93000001</v>
       </c>
       <c r="E86" s="12" t="n">
-        <v>1.63</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="87">
@@ -19190,16 +19190,16 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Mato Grosso do Sul</t>
+          <t>Mato Grosso</t>
         </is>
       </c>
       <c r="D87" s="6" t="n">
-        <v>88057920.31999999</v>
+        <v>88414512.84999999</v>
       </c>
       <c r="E87" s="12" t="n">
         <v>1.62</v>
@@ -19213,19 +19213,19 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Tocantins</t>
+          <t>Mato Grosso do Sul</t>
         </is>
       </c>
       <c r="D88" s="6" t="n">
-        <v>84766787.34</v>
+        <v>88057920.31999999</v>
       </c>
       <c r="E88" s="12" t="n">
-        <v>1.56</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="89">
@@ -19521,7 +19521,7 @@
         </is>
       </c>
       <c r="D101" s="6" t="n">
-        <v>87718083.37</v>
+        <v>87723073.27</v>
       </c>
       <c r="E101" s="12" t="n">
         <v>2.76</v>
@@ -20536,7 +20536,7 @@
         <v>97718685.43000001</v>
       </c>
       <c r="E145" s="12" t="n">
-        <v>13.69</v>
+        <v>13.67</v>
       </c>
     </row>
     <row r="146">
@@ -20559,7 +20559,7 @@
         <v>80313354.70999999</v>
       </c>
       <c r="E146" s="12" t="n">
-        <v>11.25</v>
+        <v>11.24</v>
       </c>
     </row>
     <row r="147">
@@ -20582,7 +20582,7 @@
         <v>53079939.7</v>
       </c>
       <c r="E147" s="12" t="n">
-        <v>7.44</v>
+        <v>7.43</v>
       </c>
     </row>
     <row r="148">
@@ -20651,7 +20651,7 @@
         <v>37050385.8</v>
       </c>
       <c r="E150" s="12" t="n">
-        <v>5.19</v>
+        <v>5.18</v>
       </c>
     </row>
     <row r="151">
@@ -20697,7 +20697,7 @@
         <v>35024163.86</v>
       </c>
       <c r="E152" s="12" t="n">
-        <v>4.91</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="153">
@@ -20835,7 +20835,7 @@
         <v>21242788.55</v>
       </c>
       <c r="E158" s="12" t="n">
-        <v>2.98</v>
+        <v>2.97</v>
       </c>
     </row>
     <row r="159">
@@ -20858,7 +20858,7 @@
         <v>20466197.66</v>
       </c>
       <c r="E159" s="12" t="n">
-        <v>2.87</v>
+        <v>2.86</v>
       </c>
     </row>
     <row r="160">
@@ -20970,10 +20970,10 @@
         </is>
       </c>
       <c r="D164" s="6" t="n">
-        <v>9976101.710000001</v>
+        <v>10803801.71</v>
       </c>
       <c r="E164" s="12" t="n">
-        <v>1.4</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="165">
@@ -21019,7 +21019,7 @@
         <v>9749891.75</v>
       </c>
       <c r="E166" s="12" t="n">
-        <v>1.37</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="167">
@@ -21042,7 +21042,7 @@
         <v>8182957.14</v>
       </c>
       <c r="E167" s="12" t="n">
-        <v>1.15</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="168">
@@ -21088,7 +21088,7 @@
         <v>6891650.26</v>
       </c>
       <c r="E169" s="12" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="170">
@@ -21180,7 +21180,7 @@
         <v>2630</v>
       </c>
       <c r="E173" s="12" t="n">
-        <v>12.49</v>
+        <v>12.48</v>
       </c>
     </row>
     <row r="174">
@@ -21203,7 +21203,7 @@
         <v>2055</v>
       </c>
       <c r="E174" s="12" t="n">
-        <v>9.76</v>
+        <v>9.75</v>
       </c>
     </row>
     <row r="175">
@@ -21226,7 +21226,7 @@
         <v>1832</v>
       </c>
       <c r="E175" s="12" t="n">
-        <v>8.699999999999999</v>
+        <v>8.69</v>
       </c>
     </row>
     <row r="176">
@@ -21272,7 +21272,7 @@
         <v>1090</v>
       </c>
       <c r="E177" s="12" t="n">
-        <v>5.18</v>
+        <v>5.17</v>
       </c>
     </row>
     <row r="178">
@@ -21706,10 +21706,10 @@
         </is>
       </c>
       <c r="D196" s="6" t="n">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="E196" s="12" t="n">
-        <v>1.75</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="197">
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 09:44:30.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 15:05:24.</t>
         </is>
       </c>
     </row>
@@ -23777,7 +23777,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 09:44:30.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 15:05:24.</t>
         </is>
       </c>
     </row>
@@ -23940,19 +23940,19 @@
         <v>1413776054.28</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>19.34</v>
+        <v>19.23</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>1024813021.59</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>18.91</v>
+        <v>18.82</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>151203289.93</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>23.92</v>
+        <v>23.4</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>22416742.52</v>
@@ -23986,19 +23986,19 @@
         <v>1060582328.58</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>14.51</v>
+        <v>14.42</v>
       </c>
       <c r="G6" s="6" t="n">
         <v>922036459.12</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>17.01</v>
+        <v>16.93</v>
       </c>
       <c r="I6" s="6" t="n">
         <v>6176134.65</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>0.98</v>
+        <v>0.96</v>
       </c>
       <c r="K6" s="6" t="n">
         <v>12304578.6</v>
@@ -24020,43 +24020,43 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>849</v>
+        <v>852</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>4.03</v>
+        <v>4.04</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>1819943318.34</v>
+        <v>1827001539.18</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>669850325.22</v>
+        <v>696999939.51</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>9.16</v>
+        <v>9.48</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>536659271.9</v>
+        <v>550159271.9</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>9.9</v>
+        <v>10.1</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>75858680.52</v>
+        <v>88792469.81999999</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>12</v>
+        <v>13.74</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>8281262.19</v>
+        <v>8381262.18</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>29808686.9</v>
+        <v>30288686.9</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>475884693.06</v>
+        <v>495138295.62</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>91.44</v>
+        <v>91.67</v>
       </c>
     </row>
     <row r="8">
@@ -24078,19 +24078,19 @@
         <v>656146458.72</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>8.98</v>
+        <v>8.92</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>448681803.71</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>8.279999999999999</v>
+        <v>8.24</v>
       </c>
       <c r="I8" s="6" t="n">
         <v>34632737.02</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>5.48</v>
+        <v>5.36</v>
       </c>
       <c r="K8" s="6" t="n">
         <v>19103480.73</v>
@@ -24112,10 +24112,10 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1321</v>
+        <v>1324</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>6.27</v>
+        <v>6.28</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>2779509683.8</v>
@@ -24124,19 +24124,19 @@
         <v>606632208.83</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>8.300000000000001</v>
+        <v>8.25</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>371047010.25</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>6.85</v>
+        <v>6.81</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>126722570.76</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>20.05</v>
+        <v>19.61</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>11984849.21</v>
@@ -24170,19 +24170,19 @@
         <v>576844006.83</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>7.89</v>
+        <v>7.85</v>
       </c>
       <c r="G10" s="6" t="n">
         <v>446516289.17</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>8.24</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>74245455</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>11.75</v>
+        <v>11.49</v>
       </c>
       <c r="K10" s="6" t="n">
         <v>8163972.08</v>
@@ -24204,31 +24204,31 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1429</v>
+        <v>1432</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>6.79</v>
+        <v>6.8</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>3431895006.71</v>
+        <v>3475284384.71</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>538110397.7</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>7.36</v>
+        <v>7.32</v>
       </c>
       <c r="G11" s="6" t="n">
         <v>407807248.96</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>7.52</v>
+        <v>7.49</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>17656542.34</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>2.79</v>
+        <v>2.73</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>15114290.24</v>
@@ -24262,19 +24262,19 @@
         <v>296602895.22</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>4.06</v>
+        <v>4.03</v>
       </c>
       <c r="G12" s="6" t="n">
         <v>238186413.63</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>4.39</v>
+        <v>4.37</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>5685501.33</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="K12" s="6" t="n">
         <v>10352171.45</v>
@@ -24299,7 +24299,7 @@
         <v>1126</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>5.35</v>
+        <v>5.34</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>1457794419.27</v>
@@ -24308,19 +24308,19 @@
         <v>230984307.78</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>3.16</v>
+        <v>3.14</v>
       </c>
       <c r="G13" s="6" t="n">
         <v>167145631.66</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>3.08</v>
+        <v>3.07</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>46909124.75</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>7.42</v>
+        <v>7.26</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>2971655.13</v>
@@ -24338,93 +24338,93 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>PSB</t>
+          <t>PSDB</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>971</v>
+        <v>1097</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>4.61</v>
+        <v>5.21</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>941728196.61</v>
+        <v>2603644371.84</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>222860869.79</v>
+        <v>227388323.13</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>3.05</v>
+        <v>3.09</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>148532548.4</v>
+        <v>162942927.09</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>2.74</v>
+        <v>2.99</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>6709805.88</v>
+        <v>5601357.34</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>1.06</v>
+        <v>0.87</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>11064396.82</v>
+        <v>13720983.93</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>36522867.5</v>
+        <v>32726838.19</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>173478904.89</v>
+        <v>157552582.81</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>69.66</v>
+        <v>74.12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>PSDB</t>
+          <t>PSB</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1094</v>
+        <v>971</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>5.19</v>
+        <v>4.61</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>2591694177.84</v>
+        <v>941728196.61</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>211211399.13</v>
+        <v>222860869.79</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>2.89</v>
+        <v>3.03</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>150372927.09</v>
+        <v>148532548.4</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>2.77</v>
+        <v>2.73</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>4459707.34</v>
+        <v>6709805.88</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0.71</v>
+        <v>1.04</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>11793159.93</v>
+        <v>11064396.82</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>32379138.19</v>
+        <v>36522867.5</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>145325286.01</v>
+        <v>173478904.89</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>73.31</v>
+        <v>69.66</v>
       </c>
     </row>
     <row r="16">
@@ -24437,7 +24437,7 @@
         <v>1309</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>6.22</v>
+        <v>6.21</v>
       </c>
       <c r="D16" s="6" t="n">
         <v>1884208841.62</v>
@@ -24446,7 +24446,7 @@
         <v>144440245.46</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>1.98</v>
+        <v>1.96</v>
       </c>
       <c r="G16" s="6" t="n">
         <v>34400765.53</v>
@@ -24458,7 +24458,7 @@
         <v>44459677.11</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>7.03</v>
+        <v>6.88</v>
       </c>
       <c r="K16" s="6" t="n">
         <v>7331199.03</v>
@@ -24492,19 +24492,19 @@
         <v>135624564.31</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>1.86</v>
+        <v>1.84</v>
       </c>
       <c r="G17" s="6" t="n">
         <v>124041740.42</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>2.29</v>
+        <v>2.28</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>1959373.78</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="K17" s="6" t="n">
         <v>836322.0800000001</v>
@@ -24544,13 +24544,13 @@
         <v>65447540.29</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>1.21</v>
+        <v>1.2</v>
       </c>
       <c r="I18" s="6" t="n">
         <v>13887392.18</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>2.2</v>
+        <v>2.15</v>
       </c>
       <c r="K18" s="6" t="n">
         <v>4906960.64</v>
@@ -24584,19 +24584,19 @@
         <v>97835344.19</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>1.34</v>
+        <v>1.33</v>
       </c>
       <c r="G19" s="6" t="n">
         <v>67589577.34999999</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>1.25</v>
+        <v>1.24</v>
       </c>
       <c r="I19" s="6" t="n">
         <v>14150621.49</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>2.24</v>
+        <v>2.19</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>3535138.7</v>
@@ -24630,19 +24630,19 @@
         <v>92105331.40000001</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>1.26</v>
+        <v>1.25</v>
       </c>
       <c r="G20" s="6" t="n">
         <v>83794222.27</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>1.55</v>
+        <v>1.54</v>
       </c>
       <c r="I20" s="6" t="n">
         <v>1699330</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="K20" s="6" t="n">
         <v>1869153.42</v>
@@ -24676,7 +24676,7 @@
         <v>73534843.78</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="G21" s="6" t="n">
         <v>60379791.05</v>
@@ -24688,7 +24688,7 @@
         <v>4467405.01</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>0.71</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>1319520.67</v>
@@ -24728,7 +24728,7 @@
         <v>43108728</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>193073.13</v>
@@ -24805,7 +24805,7 @@
         <v>355</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>1.69</v>
+        <v>1.68</v>
       </c>
       <c r="D24" s="6" t="n">
         <v>587079065.02</v>
@@ -24820,13 +24820,13 @@
         <v>29563402.63</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
       <c r="I24" s="6" t="n">
         <v>412960.64</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="K24" s="6" t="n">
         <v>540283.86</v>
@@ -24851,7 +24851,7 @@
         <v>475</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>2.26</v>
+        <v>2.25</v>
       </c>
       <c r="D25" s="6" t="n">
         <v>286783798.5</v>
@@ -24860,7 +24860,7 @@
         <v>12107937.16</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>2234662.44</v>
@@ -25304,7 +25304,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 09:44:30.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 15:05:24.</t>
         </is>
       </c>
     </row>
@@ -28207,7 +28207,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 09:44:30.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-15 15:05:24.</t>
         </is>
       </c>
     </row>
@@ -28228,7 +28228,7 @@
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>Nota 2: outras 4107 candidaturas NAO declararam receita alguma, das quais 960 sao vice ou suplente, que nao prestam conta propria. Ausencia de declaracao nao e' autofinanciamento, e por isso elas ficam fora desta tabela.</t>
+          <t>Nota 2: outras 4113 candidaturas NAO declararam receita alguma, das quais 966 sao vice ou suplente, que nao prestam conta propria. Ausencia de declaracao nao e' autofinanciamento, e por isso elas ficam fora desta tabela.</t>
         </is>
       </c>
     </row>
@@ -29360,7 +29360,7 @@
         <v>74.11</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="G28" s="5" t="n">
         <v>40</v>
@@ -29369,19 +29369,19 @@
         <v>29569</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>31.11</v>
+        <v>32.13</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>121396489.89</v>
+        <v>164723028.18</v>
       </c>
       <c r="K28" s="6" t="n">
-        <v>76.06</v>
+        <v>103.21</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>102.64</v>
+        <v>139.27</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>84.27</v>
+        <v>118.21</v>
       </c>
     </row>
     <row r="29">
@@ -29593,7 +29593,7 @@
         <v>73.69</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>21061</v>
+        <v>21073</v>
       </c>
       <c r="G33" s="8" t="n">
         <v>1790</v>
@@ -29602,19 +29602,19 @@
         <v>88182</v>
       </c>
       <c r="I33" s="9" t="n">
-        <v>13.34</v>
+        <v>13.35</v>
       </c>
       <c r="J33" s="9" t="n">
-        <v>7309285444.22</v>
+        <v>7352611982.509999</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>34.12</v>
+        <v>34.32</v>
       </c>
       <c r="L33" s="9" t="n">
-        <v>46.31</v>
+        <v>46.58</v>
       </c>
       <c r="M33" s="9" t="n">
-        <v>38.34</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 18/10/2026 15:45
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 13:45:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 13:45:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-18 13:45:20</t>
+          <t>2026-10-18 15:36:55</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 13:45:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 13:45:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 13:45:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 13:45:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 13:45:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 13:45:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 13:45:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 19/10/2026 09:27
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-18 15:36:55</t>
+          <t>2026-10-19 09:08:31</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-18 15:36:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 19/10/2026 15:13
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-19 09:08:31</t>
+          <t>2026-10-19 15:04:16</t>
         </is>
       </c>
     </row>
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="G65" s="6" t="n">
-        <v>58445503.79</v>
+        <v>58445503.79000001</v>
       </c>
       <c r="H65" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 09:08:31.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 20/10/2026 08:30
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 22:12:16.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 22:12:16.</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>6735370</v>
+        <v>6730564</v>
       </c>
     </row>
     <row r="61">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-19 15:04:16</t>
+          <t>2026-10-19 22:12:16</t>
         </is>
       </c>
     </row>
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="G65" s="6" t="n">
-        <v>58445503.79000001</v>
+        <v>58445503.79</v>
       </c>
       <c r="H65" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 22:12:16.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 22:12:16.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 22:12:16.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 22:12:16.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 22:12:16.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 22:12:16.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 15:04:16.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-19 22:12:16.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 20/10/2026 09:14
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 08:37:00.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 09:06:41.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 08:37:00.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 09:06:41.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>310</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-20 08:37:00</t>
+          <t>2026-10-20 09:06:41</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 08:37:00.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 09:06:41.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 08:37:00.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 09:06:41.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 08:37:00.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 09:06:41.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 08:37:00.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 09:06:41.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 08:37:00.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 09:06:41.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 08:37:00.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 09:06:41.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 08:37:00.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-20 09:06:41.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 21/10/2026 15:14
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 09:08:28.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 09:08:28.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>366</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-21 09:08:28</t>
+          <t>2026-10-21 15:04:33</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 09:08:28.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 09:08:28.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 09:08:28.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 09:08:28.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 09:08:28.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
         </is>
       </c>
     </row>
@@ -23854,7 +23854,7 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 09:08:28.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 09:08:28.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 21/10/2026 21:16
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32960938517.57999</v>
+        <v>32960938517.58</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 21:05:51.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 21:05:51.</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>6735370</v>
+        <v>6731920</v>
       </c>
     </row>
     <row r="61">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-21 15:04:33</t>
+          <t>2026-10-21 21:05:51</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.9499999</v>
+        <v>575680870.95</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.75</v>
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="G65" s="6" t="n">
-        <v>58445503.79</v>
+        <v>58445503.79000001</v>
       </c>
       <c r="H65" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 21:05:51.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 21:05:51.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 21:05:51.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 21:05:51.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 21:05:51.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 21:05:51.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 15:04:33.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-21 21:05:51.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 23/10/2026 10:57
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 08:25:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 08:25:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>783</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-23 08:25:44</t>
+          <t>2026-10-23 10:45:18</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 08:25:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 08:25:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 08:25:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 08:25:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 08:25:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 08:25:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 08:25:44.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 23/10/2026 15:26
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-23 10:45:18</t>
+          <t>2026-10-23 13:22:47</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 10:45:18.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 23/10/2026 16:16
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-23 13:22:47</t>
+          <t>2026-10-23 16:06:34</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 13:22:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 23/10/2026 18:26
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32960938517.57999</v>
+        <v>32960938517.58</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-23 16:06:34</t>
+          <t>2026-10-23 18:16:56</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.9499999</v>
+        <v>575680870.95</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.75</v>
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="G65" s="6" t="n">
-        <v>58445503.79</v>
+        <v>58445503.79000001</v>
       </c>
       <c r="H65" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 16:06:34.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 24/10/2026 03:25
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 03:10:26.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 03:10:26.</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>6735370</v>
+        <v>6714482</v>
       </c>
     </row>
     <row r="61">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-23 18:16:56</t>
+          <t>2026-10-24 03:10:26</t>
         </is>
       </c>
     </row>
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="G65" s="6" t="n">
-        <v>58445503.79000001</v>
+        <v>58445503.79</v>
       </c>
       <c r="H65" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 03:10:26.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 03:10:26.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 03:10:26.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 03:10:26.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 03:10:26.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 03:10:26.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-23 18:16:56.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 03:10:26.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 24/10/2026 16:10
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 09:07:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 09:07:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>370</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-24 09:07:41</t>
+          <t>2026-10-24 15:31:47</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 09:07:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 09:07:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 09:07:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 09:07:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 09:07:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 09:07:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 09:07:41.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 24/10/2026 17:15
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 17:05:26.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 17:05:26.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-24 15:31:47</t>
+          <t>2026-10-24 17:05:26</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 17:05:26.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 17:05:26.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 17:05:26.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 17:05:26.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 17:05:26.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 17:05:26.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 15:31:47.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-24 17:05:26.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 26/10/2026 09:32
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 08:12:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 08:12:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>111</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-26 08:12:20</t>
+          <t>2026-10-26 09:15:55</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 08:12:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 08:12:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 08:12:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 08:12:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 08:12:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 08:12:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 08:12:20.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 26/10/2026 21:30
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 21:07:07.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 21:07:07.</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-26 09:15:55</t>
+          <t>2026-10-26 21:07:07</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 21:07:07.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 21:07:07.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 21:07:07.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 21:07:07.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 21:07:07.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 21:07:07.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 09:15:55.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-26 21:07:07.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Painel do dinheiro das Eleicoes 2026, 28/10/2026 15:19
</commit_message>
<xml_diff>
--- a/dados/TABELAS-IBGE-ABNT-2026.xlsx
+++ b/dados/TABELAS-IBGE-ABNT-2026.xlsx
@@ -888,7 +888,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>32960938517.58</v>
+        <v>32960938517.57999</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>100</v>
@@ -909,7 +909,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 12:20:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 15:06:08.</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 12:20:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 15:06:08.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>870</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-10-28 12:20:21</t>
+          <t>2026-10-28 15:06:08</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>575680870.95</v>
+        <v>575680870.9499999</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.75</v>
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="G65" s="6" t="n">
-        <v>58445503.79000001</v>
+        <v>58445503.79</v>
       </c>
       <c r="H65" s="6" t="n">
         <v>0.18</v>
@@ -8842,7 +8842,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 12:20:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 15:06:08.</t>
         </is>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 12:20:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 15:06:08.</t>
         </is>
       </c>
     </row>
@@ -17206,7 +17206,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 12:20:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 15:06:08.</t>
         </is>
       </c>
     </row>
@@ -22451,7 +22451,7 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 12:20:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 15:06:08.</t>
         </is>
       </c>
     </row>
@@ -23808,7 +23808,7 @@
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 12:20:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 15:06:08.</t>
         </is>
       </c>
     </row>
@@ -25335,7 +25335,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 12:20:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 15:06:08.</t>
         </is>
       </c>
     </row>
@@ -28238,7 +28238,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 12:20:21.</t>
+          <t>Fonte: Brasil. Tribunal Superior Eleitoral. Dados abertos eleitorais, Eleicoes Gerais de 2026. Disponivel em: https://dadosabertos.tse.jus.br. Extracao de 2026-10-28 15:06:08.</t>
         </is>
       </c>
     </row>

</xml_diff>